<commit_message>
Site guncellemesi - 16.09.2026 12:16
</commit_message>
<xml_diff>
--- a/app/fonlar/getiri/menkul-kiymet-yatirim-fonlari/data/menkul-kiymet-yatirim-fonlari-getiri.xlsx
+++ b/app/fonlar/getiri/menkul-kiymet-yatirim-fonlari/data/menkul-kiymet-yatirim-fonlari-getiri.xlsx
@@ -19,7 +19,7 @@
     <t>Dışa Aktarım Tarihi:</t>
   </si>
   <si>
-    <t>16.09.2026 09:34:01</t>
+    <t>16.09.2026 12:14:07</t>
   </si>
   <si>
     <t>Toplam Kayıt Sayısı:</t>
@@ -7442,25 +7442,25 @@
         <v>7</v>
       </c>
       <c r="E19" s="7">
-        <v>0</v>
+        <v>0.213033</v>
       </c>
       <c r="F19" s="7">
-        <v>0</v>
+        <v>0.30478500000000003</v>
       </c>
       <c r="G19" s="7">
-        <v>0</v>
+        <v>0.395934</v>
       </c>
       <c r="H19" s="7">
-        <v>0</v>
+        <v>1.187495</v>
       </c>
       <c r="I19" s="7">
-        <v>0</v>
+        <v>1.118031</v>
       </c>
       <c r="J19" s="7">
-        <v>0</v>
+        <v>1.690632</v>
       </c>
       <c r="K19" s="7">
-        <v>0</v>
+        <v>11.243251</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -7788,25 +7788,25 @@
         <v>1</v>
       </c>
       <c r="E29" s="7">
-        <v>0.026598</v>
+        <v>0.026591999999999998</v>
       </c>
       <c r="F29" s="7">
-        <v>0.09475099999999999</v>
+        <v>0.09474500000000001</v>
       </c>
       <c r="G29" s="7">
-        <v>0.19558599999999998</v>
+        <v>0.195579</v>
       </c>
       <c r="H29" s="7">
-        <v>0.287306</v>
+        <v>0.287298</v>
       </c>
       <c r="I29" s="7">
-        <v>0.429165</v>
+        <v>0.429157</v>
       </c>
       <c r="J29" s="7">
-        <v>2.50284</v>
+        <v>2.502819</v>
       </c>
       <c r="K29" s="7">
-        <v>4.785182</v>
+        <v>4.7851479999999995</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -7823,25 +7823,25 @@
         <v>4</v>
       </c>
       <c r="E30" s="7">
-        <v>0.028448</v>
+        <v>0.022729</v>
       </c>
       <c r="F30" s="7">
-        <v>0.070357</v>
+        <v>0.064405</v>
       </c>
       <c r="G30" s="7">
-        <v>0.17639</v>
+        <v>0.169847</v>
       </c>
       <c r="H30" s="7">
-        <v>0.313507</v>
+        <v>0.30620200000000003</v>
       </c>
       <c r="I30" s="7">
-        <v>0.456809</v>
+        <v>0.44870699999999997</v>
       </c>
       <c r="J30" s="7">
-        <v>1.8332579999999998</v>
+        <v>1.8175020000000002</v>
       </c>
       <c r="K30" s="7">
-        <v>8.32671</v>
+        <v>8.274842</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -8328,25 +8328,25 @@
         <v>6</v>
       </c>
       <c r="E45" s="7">
-        <v>0</v>
+        <v>0.002114</v>
       </c>
       <c r="F45" s="7">
-        <v>0</v>
+        <v>-0.021472</v>
       </c>
       <c r="G45" s="7">
-        <v>0</v>
+        <v>0.037408000000000004</v>
       </c>
       <c r="H45" s="7">
-        <v>0</v>
+        <v>0.158389</v>
       </c>
       <c r="I45" s="7">
-        <v>0</v>
+        <v>0.207043</v>
       </c>
       <c r="J45" s="7">
-        <v>0</v>
+        <v>0.9411320000000001</v>
       </c>
       <c r="K45" s="7">
-        <v>0</v>
+        <v>2.859427</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
@@ -8431,25 +8431,25 @@
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="7">
-        <v>0</v>
+        <v>0.0034260000000000002</v>
       </c>
       <c r="F48" s="7">
-        <v>0</v>
+        <v>0.042815000000000006</v>
       </c>
       <c r="G48" s="7">
-        <v>0</v>
+        <v>0.110324</v>
       </c>
       <c r="H48" s="7">
-        <v>0</v>
+        <v>0.20930700000000002</v>
       </c>
       <c r="I48" s="7">
-        <v>0</v>
+        <v>0.32853299999999996</v>
       </c>
       <c r="J48" s="7">
-        <v>0</v>
+        <v>1.9911459999999999</v>
       </c>
       <c r="K48" s="7">
-        <v>0</v>
+        <v>5.374736</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -8464,25 +8464,25 @@
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="7">
-        <v>0</v>
+        <v>-0.012024</v>
       </c>
       <c r="F49" s="7">
-        <v>0</v>
+        <v>0.009709</v>
       </c>
       <c r="G49" s="7">
-        <v>0</v>
+        <v>0.059770000000000004</v>
       </c>
       <c r="H49" s="7">
-        <v>0</v>
+        <v>0.16700299999999998</v>
       </c>
       <c r="I49" s="7">
-        <v>0</v>
+        <v>0.277483</v>
       </c>
       <c r="J49" s="7">
-        <v>0</v>
+        <v>1.7625739999999999</v>
       </c>
       <c r="K49" s="7">
-        <v>0</v>
+        <v>5.843411</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -9752,19 +9752,19 @@
         <v>7</v>
       </c>
       <c r="E91" s="7">
-        <v>0.009425</v>
+        <v>0.009426</v>
       </c>
       <c r="F91" s="7">
-        <v>-0.106375</v>
+        <v>-0.106373</v>
       </c>
       <c r="G91" s="7">
-        <v>-0.018346</v>
+        <v>-0.018344</v>
       </c>
       <c r="H91" s="7">
-        <v>-0.026184</v>
+        <v>-0.026181999999999997</v>
       </c>
       <c r="I91" s="7">
-        <v>-0.0031490000000000003</v>
+        <v>-0.003148</v>
       </c>
       <c r="J91" s="7"/>
       <c r="K91" s="7"/>
@@ -9934,19 +9934,19 @@
         <v>5</v>
       </c>
       <c r="E97" s="7">
-        <v>0.014809000000000001</v>
+        <v>0.00404</v>
       </c>
       <c r="F97" s="7">
-        <v>-0.000145</v>
+        <v>-0.010755999999999998</v>
       </c>
       <c r="G97" s="7">
-        <v>0.20877600000000002</v>
+        <v>0.19594899999999998</v>
       </c>
       <c r="H97" s="7">
-        <v>0.316933</v>
+        <v>0.302958</v>
       </c>
       <c r="I97" s="7">
-        <v>0.42749899999999996</v>
+        <v>0.412351</v>
       </c>
       <c r="J97" s="7"/>
       <c r="K97" s="7"/>
@@ -10300,10 +10300,10 @@
         <v>3</v>
       </c>
       <c r="E109" s="7">
-        <v>0.043487</v>
+        <v>0.031548</v>
       </c>
       <c r="F109" s="7">
-        <v>0.207828</v>
+        <v>0.19401</v>
       </c>
       <c r="G109" s="7"/>
       <c r="H109" s="7"/>
@@ -10662,19 +10662,19 @@
         <v>6</v>
       </c>
       <c r="E121" s="7">
-        <v>0.0008550000000000001</v>
+        <v>-0.011202</v>
       </c>
       <c r="F121" s="7">
-        <v>-0.026861000000000003</v>
+        <v>-0.038584</v>
       </c>
       <c r="G121" s="7">
-        <v>0.19795300000000002</v>
+        <v>0.183521</v>
       </c>
       <c r="H121" s="7">
-        <v>0.27494399999999997</v>
+        <v>0.259585</v>
       </c>
       <c r="I121" s="7">
-        <v>0.317506</v>
+        <v>0.301634</v>
       </c>
       <c r="J121" s="7"/>
       <c r="K121" s="7"/>
@@ -11593,22 +11593,22 @@
         <v>6</v>
       </c>
       <c r="E150" s="7">
-        <v>0.005104</v>
+        <v>-0.005289</v>
       </c>
       <c r="F150" s="7">
-        <v>0.008907</v>
+        <v>-0.0015249999999999999</v>
       </c>
       <c r="G150" s="7">
-        <v>0.122199</v>
+        <v>0.110595</v>
       </c>
       <c r="H150" s="7">
-        <v>0.22477</v>
+        <v>0.212105</v>
       </c>
       <c r="I150" s="7">
-        <v>0.269086</v>
+        <v>0.25596399999999997</v>
       </c>
       <c r="J150" s="7">
-        <v>1.327704</v>
+        <v>1.3036349999999999</v>
       </c>
       <c r="K150" s="7"/>
     </row>
@@ -11684,19 +11684,19 @@
         <v>5</v>
       </c>
       <c r="E153" s="7">
-        <v>-0.014117</v>
+        <v>-0.014173999999999999</v>
       </c>
       <c r="F153" s="7">
-        <v>0.03682</v>
+        <v>0.03676</v>
       </c>
       <c r="G153" s="7">
-        <v>0.131273</v>
+        <v>0.131207</v>
       </c>
       <c r="H153" s="7">
-        <v>0.196553</v>
+        <v>0.196484</v>
       </c>
       <c r="I153" s="7">
-        <v>0.298524</v>
+        <v>0.29844899999999996</v>
       </c>
       <c r="J153" s="7"/>
       <c r="K153" s="7"/>
@@ -11998,22 +11998,22 @@
         <v>7</v>
       </c>
       <c r="E163" s="7">
-        <v>-0.008178</v>
+        <v>-0.007838000000000001</v>
       </c>
       <c r="F163" s="7">
-        <v>-0.056191000000000005</v>
+        <v>-0.055868</v>
       </c>
       <c r="G163" s="7">
-        <v>-0.152345</v>
+        <v>-0.152054</v>
       </c>
       <c r="H163" s="7">
-        <v>-0.021336</v>
+        <v>-0.021001</v>
       </c>
       <c r="I163" s="7">
-        <v>0.6954089999999999</v>
+        <v>0.69599</v>
       </c>
       <c r="J163" s="7">
-        <v>3.4721789999999997</v>
+        <v>3.473712</v>
       </c>
       <c r="K163" s="7"/>
     </row>
@@ -12031,16 +12031,16 @@
         <v>4</v>
       </c>
       <c r="E164" s="7">
-        <v>0.077768</v>
+        <v>0.07871</v>
       </c>
       <c r="F164" s="7">
-        <v>0.122279</v>
+        <v>0.12326000000000001</v>
       </c>
       <c r="G164" s="7">
-        <v>0.233217</v>
+        <v>0.234295</v>
       </c>
       <c r="H164" s="7">
-        <v>0.332519</v>
+        <v>0.33368299999999995</v>
       </c>
       <c r="I164" s="7"/>
       <c r="J164" s="7"/>
@@ -12118,19 +12118,19 @@
       </c>
       <c r="D167" s="6"/>
       <c r="E167" s="7">
-        <v>0.006338</v>
+        <v>0.005817</v>
       </c>
       <c r="F167" s="7">
-        <v>0.074522</v>
+        <v>0.073965</v>
       </c>
       <c r="G167" s="7">
-        <v>0.090527</v>
+        <v>0.089962</v>
       </c>
       <c r="H167" s="7">
-        <v>0.127191</v>
+        <v>0.126607</v>
       </c>
       <c r="I167" s="7">
-        <v>0.236709</v>
+        <v>0.236069</v>
       </c>
       <c r="J167" s="7"/>
       <c r="K167" s="7"/>
@@ -12506,25 +12506,25 @@
         <v>3</v>
       </c>
       <c r="E179" s="7">
-        <v>-0.0026889999999999996</v>
+        <v>0.008681</v>
       </c>
       <c r="F179" s="7">
-        <v>0.046801</v>
+        <v>0.058735</v>
       </c>
       <c r="G179" s="7">
-        <v>0.127971</v>
+        <v>0.14083</v>
       </c>
       <c r="H179" s="7">
-        <v>0.20308199999999998</v>
+        <v>0.216798</v>
       </c>
       <c r="I179" s="7">
-        <v>0.34244300000000005</v>
+        <v>0.357748</v>
       </c>
       <c r="J179" s="7">
-        <v>1.6884919999999999</v>
+        <v>1.719142</v>
       </c>
       <c r="K179" s="7">
-        <v>6.522854</v>
+        <v>6.608619999999999</v>
       </c>
     </row>
     <row r="180" spans="1:11" x14ac:dyDescent="0.25">
@@ -13562,16 +13562,16 @@
         <v>6</v>
       </c>
       <c r="E213" s="7">
-        <v>-0.009692</v>
+        <v>-0.010125</v>
       </c>
       <c r="F213" s="7">
-        <v>-0.01996</v>
+        <v>-0.020388000000000003</v>
       </c>
       <c r="G213" s="7">
-        <v>-0.12256</v>
+        <v>-0.122943</v>
       </c>
       <c r="H213" s="7">
-        <v>0.031105</v>
+        <v>0.030654</v>
       </c>
       <c r="I213" s="7"/>
       <c r="J213" s="7"/>
@@ -13823,13 +13823,13 @@
         <v>6</v>
       </c>
       <c r="E222" s="7">
-        <v>0.018569</v>
+        <v>0.018308</v>
       </c>
       <c r="F222" s="7">
-        <v>0.056662</v>
+        <v>0.056391</v>
       </c>
       <c r="G222" s="7">
-        <v>0.124163</v>
+        <v>0.123875</v>
       </c>
       <c r="H222" s="7"/>
       <c r="I222" s="7"/>
@@ -13850,19 +13850,19 @@
         <v>3</v>
       </c>
       <c r="E223" s="7">
-        <v>0.004341</v>
+        <v>-0.000149</v>
       </c>
       <c r="F223" s="7">
-        <v>0.039371</v>
+        <v>0.034725</v>
       </c>
       <c r="G223" s="7">
-        <v>0.132204</v>
+        <v>0.127142</v>
       </c>
       <c r="H223" s="7">
-        <v>0.263387</v>
+        <v>0.257739</v>
       </c>
       <c r="I223" s="7">
-        <v>0.458287</v>
+        <v>0.451767</v>
       </c>
       <c r="J223" s="7"/>
       <c r="K223" s="7"/>
@@ -13941,22 +13941,22 @@
         <v>6</v>
       </c>
       <c r="E226" s="7">
-        <v>-0.072687</v>
+        <v>-0.072689</v>
       </c>
       <c r="F226" s="7">
-        <v>-0.20045300000000002</v>
+        <v>-0.20045400000000002</v>
       </c>
       <c r="G226" s="7">
-        <v>-0.081732</v>
+        <v>-0.08173400000000001</v>
       </c>
       <c r="H226" s="7">
-        <v>-0.025695000000000003</v>
+        <v>-0.025696</v>
       </c>
       <c r="I226" s="7">
-        <v>0.052537</v>
+        <v>0.052535</v>
       </c>
       <c r="J226" s="7">
-        <v>0.577465</v>
+        <v>0.577462</v>
       </c>
       <c r="K226" s="7"/>
     </row>
@@ -14040,25 +14040,25 @@
         <v>6</v>
       </c>
       <c r="E229" s="7">
-        <v>-0.016533</v>
+        <v>-0.016523</v>
       </c>
       <c r="F229" s="7">
-        <v>0.032916</v>
+        <v>0.032926000000000004</v>
       </c>
       <c r="G229" s="7">
-        <v>0.303997</v>
+        <v>0.30401</v>
       </c>
       <c r="H229" s="7">
-        <v>0.284628</v>
+        <v>0.284641</v>
       </c>
       <c r="I229" s="7">
-        <v>0.41518</v>
+        <v>0.415195</v>
       </c>
       <c r="J229" s="7">
-        <v>1.824123</v>
+        <v>1.824152</v>
       </c>
       <c r="K229" s="7">
-        <v>3.1853339999999997</v>
+        <v>3.185378</v>
       </c>
     </row>
     <row r="230" spans="1:11" x14ac:dyDescent="0.25">
@@ -14236,25 +14236,25 @@
         <v>4</v>
       </c>
       <c r="E235" s="7">
-        <v>0.022677</v>
+        <v>0.015650999999999998</v>
       </c>
       <c r="F235" s="7">
-        <v>0.052241</v>
+        <v>0.045011999999999996</v>
       </c>
       <c r="G235" s="7">
-        <v>0.085727</v>
+        <v>0.078267</v>
       </c>
       <c r="H235" s="7">
-        <v>0.17183900000000002</v>
+        <v>0.163788</v>
       </c>
       <c r="I235" s="7">
-        <v>0.371833</v>
+        <v>0.362408</v>
       </c>
       <c r="J235" s="7">
-        <v>1.946386</v>
+        <v>1.926143</v>
       </c>
       <c r="K235" s="7">
-        <v>5.7617259999999995</v>
+        <v>5.715271</v>
       </c>
     </row>
     <row r="236" spans="1:11" x14ac:dyDescent="0.25">
@@ -14667,25 +14667,25 @@
         <v>4</v>
       </c>
       <c r="E248" s="7">
-        <v>0.015004</v>
+        <v>0.014448</v>
       </c>
       <c r="F248" s="7">
-        <v>0.062034000000000006</v>
+        <v>0.061453</v>
       </c>
       <c r="G248" s="7">
-        <v>0.09034800000000001</v>
+        <v>0.089751</v>
       </c>
       <c r="H248" s="7">
-        <v>0.16825299999999999</v>
+        <v>0.16761299999999998</v>
       </c>
       <c r="I248" s="7">
-        <v>0.33882100000000004</v>
+        <v>0.338087</v>
       </c>
       <c r="J248" s="7">
-        <v>1.8785020000000001</v>
+        <v>1.876925</v>
       </c>
       <c r="K248" s="7">
-        <v>6.218661</v>
+        <v>6.214708000000001</v>
       </c>
     </row>
     <row r="249" spans="1:11" x14ac:dyDescent="0.25">
@@ -15099,7 +15099,7 @@
         <v>0.033554</v>
       </c>
       <c r="F261" s="7">
-        <v>0.197547</v>
+        <v>0.197548</v>
       </c>
       <c r="G261" s="7">
         <v>0.21931599999999998</v>
@@ -15108,7 +15108,7 @@
         <v>0.38569400000000004</v>
       </c>
       <c r="I261" s="7">
-        <v>0.6530819999999999</v>
+        <v>0.6530830000000001</v>
       </c>
       <c r="J261" s="7"/>
       <c r="K261" s="7"/>
@@ -15195,22 +15195,22 @@
         <v>6</v>
       </c>
       <c r="E264" s="7">
-        <v>-0.016934</v>
+        <v>-0.015752</v>
       </c>
       <c r="F264" s="7">
-        <v>-0.0032379999999999996</v>
+        <v>-0.002039</v>
       </c>
       <c r="G264" s="7">
-        <v>0.34915399999999996</v>
+        <v>0.350777</v>
       </c>
       <c r="H264" s="7">
-        <v>0.34390099999999996</v>
+        <v>0.34551699999999996</v>
       </c>
       <c r="I264" s="7">
-        <v>0.45637</v>
+        <v>0.458121</v>
       </c>
       <c r="J264" s="7">
-        <v>2.4078880000000003</v>
+        <v>2.411986</v>
       </c>
       <c r="K264" s="7"/>
     </row>
@@ -15321,16 +15321,16 @@
         <v>6</v>
       </c>
       <c r="E268" s="7">
-        <v>0</v>
+        <v>0.12498</v>
       </c>
       <c r="F268" s="7">
-        <v>0</v>
+        <v>0.11080999999999999</v>
       </c>
       <c r="G268" s="7">
-        <v>0</v>
+        <v>0.197407</v>
       </c>
       <c r="H268" s="7">
-        <v>0</v>
+        <v>0.37709699999999996</v>
       </c>
       <c r="I268" s="7"/>
       <c r="J268" s="7"/>
@@ -15554,22 +15554,22 @@
         <v>4</v>
       </c>
       <c r="E275" s="7">
-        <v>0.026400999999999997</v>
+        <v>0.018024</v>
       </c>
       <c r="F275" s="7">
-        <v>0.062221</v>
+        <v>0.053551</v>
       </c>
       <c r="G275" s="7">
-        <v>0.156815</v>
+        <v>0.147373</v>
       </c>
       <c r="H275" s="7">
-        <v>0.22673500000000002</v>
+        <v>0.216722</v>
       </c>
       <c r="I275" s="7">
-        <v>0.34974400000000005</v>
+        <v>0.338727</v>
       </c>
       <c r="J275" s="7">
-        <v>1.8557599999999999</v>
+        <v>1.832451</v>
       </c>
       <c r="K275" s="7"/>
     </row>
@@ -16067,22 +16067,22 @@
         <v>6</v>
       </c>
       <c r="E290" s="7">
-        <v>0.031225999999999997</v>
+        <v>0.031716</v>
       </c>
       <c r="F290" s="7">
-        <v>0.042986</v>
+        <v>0.043482</v>
       </c>
       <c r="G290" s="7">
-        <v>0.09542099999999999</v>
+        <v>0.09594200000000001</v>
       </c>
       <c r="H290" s="7">
-        <v>0.296545</v>
+        <v>0.297161</v>
       </c>
       <c r="I290" s="7">
-        <v>0.45169899999999996</v>
+        <v>0.452389</v>
       </c>
       <c r="J290" s="7">
-        <v>1.4775260000000001</v>
+        <v>1.4787039999999998</v>
       </c>
       <c r="K290" s="7"/>
     </row>
@@ -16170,19 +16170,19 @@
         <v>5</v>
       </c>
       <c r="E293" s="7">
-        <v>0</v>
+        <v>-0.035105</v>
       </c>
       <c r="F293" s="7">
-        <v>0</v>
+        <v>-0.050492999999999996</v>
       </c>
       <c r="G293" s="7">
-        <v>0</v>
+        <v>0.029939</v>
       </c>
       <c r="H293" s="7">
-        <v>0</v>
+        <v>0.104536</v>
       </c>
       <c r="I293" s="7">
-        <v>0</v>
+        <v>0.142773</v>
       </c>
       <c r="J293" s="7"/>
       <c r="K293" s="7"/>
@@ -16267,25 +16267,25 @@
         <v>5</v>
       </c>
       <c r="E296" s="7">
-        <v>-0.011644000000000002</v>
+        <v>-0.02205</v>
       </c>
       <c r="F296" s="7">
-        <v>-0.038748</v>
+        <v>-0.04887</v>
       </c>
       <c r="G296" s="7">
-        <v>0.099497</v>
+        <v>0.08792</v>
       </c>
       <c r="H296" s="7">
-        <v>0.208675</v>
+        <v>0.19594899999999998</v>
       </c>
       <c r="I296" s="7">
-        <v>0.45181</v>
+        <v>0.436523</v>
       </c>
       <c r="J296" s="7">
-        <v>1.6512440000000002</v>
+        <v>1.6233279999999999</v>
       </c>
       <c r="K296" s="7">
-        <v>9.198966</v>
+        <v>9.091578</v>
       </c>
     </row>
     <row r="297" spans="1:11" x14ac:dyDescent="0.25">
@@ -16469,22 +16469,22 @@
         <v>5</v>
       </c>
       <c r="E302" s="7">
-        <v>0.017659</v>
+        <v>0.007043000000000001</v>
       </c>
       <c r="F302" s="7">
-        <v>0.032019</v>
+        <v>0.021253</v>
       </c>
       <c r="G302" s="7">
-        <v>0.073484</v>
+        <v>0.06228500000000001</v>
       </c>
       <c r="H302" s="7">
-        <v>0.089648</v>
+        <v>0.078281</v>
       </c>
       <c r="I302" s="7">
-        <v>0.1881</v>
+        <v>0.175706</v>
       </c>
       <c r="J302" s="7">
-        <v>1.471387</v>
+        <v>1.4456049999999998</v>
       </c>
       <c r="K302" s="7"/>
     </row>
@@ -16626,22 +16626,22 @@
         <v>7</v>
       </c>
       <c r="E307" s="7">
-        <v>0</v>
+        <v>-0.016966000000000002</v>
       </c>
       <c r="F307" s="7">
-        <v>0</v>
+        <v>-0.07989099999999999</v>
       </c>
       <c r="G307" s="7">
-        <v>0</v>
+        <v>-0.188522</v>
       </c>
       <c r="H307" s="7">
-        <v>0</v>
+        <v>-0.067103</v>
       </c>
       <c r="I307" s="7">
-        <v>0</v>
+        <v>0.652366</v>
       </c>
       <c r="J307" s="7">
-        <v>0</v>
+        <v>3.343413</v>
       </c>
       <c r="K307" s="7"/>
     </row>
@@ -16847,22 +16847,22 @@
         <v>3</v>
       </c>
       <c r="E314" s="7">
-        <v>0.023663</v>
+        <v>0.023944</v>
       </c>
       <c r="F314" s="7">
-        <v>0.073813</v>
+        <v>0.07410800000000001</v>
       </c>
       <c r="G314" s="7">
-        <v>0.17027699999999998</v>
+        <v>0.170599</v>
       </c>
       <c r="H314" s="7">
-        <v>0.314204</v>
+        <v>0.314565</v>
       </c>
       <c r="I314" s="7">
-        <v>0.48578499999999997</v>
+        <v>0.48619300000000004</v>
       </c>
       <c r="J314" s="7">
-        <v>2.7341269999999995</v>
+        <v>2.735154</v>
       </c>
       <c r="K314" s="7"/>
     </row>
@@ -16880,22 +16880,22 @@
         <v>5</v>
       </c>
       <c r="E315" s="7">
-        <v>-0.009673000000000001</v>
+        <v>-0.01113</v>
       </c>
       <c r="F315" s="7">
-        <v>0.001997</v>
+        <v>0.000523</v>
       </c>
       <c r="G315" s="7">
-        <v>0.065884</v>
+        <v>0.064315</v>
       </c>
       <c r="H315" s="7">
-        <v>0.207152</v>
+        <v>0.205375</v>
       </c>
       <c r="I315" s="7">
-        <v>0.33193399999999995</v>
+        <v>0.329973</v>
       </c>
       <c r="J315" s="7">
-        <v>1.8811660000000001</v>
+        <v>1.876925</v>
       </c>
       <c r="K315" s="7"/>
     </row>
@@ -16913,22 +16913,22 @@
         <v>5</v>
       </c>
       <c r="E316" s="7">
-        <v>-0.0014269999999999999</v>
+        <v>-0.0025919999999999997</v>
       </c>
       <c r="F316" s="7">
-        <v>0.011818</v>
+        <v>0.010637</v>
       </c>
       <c r="G316" s="7">
-        <v>0.07209</v>
+        <v>0.070839</v>
       </c>
       <c r="H316" s="7">
-        <v>0.199785</v>
+        <v>0.198384</v>
       </c>
       <c r="I316" s="7">
-        <v>0.340466</v>
+        <v>0.338902</v>
       </c>
       <c r="J316" s="7">
-        <v>1.9140000000000001</v>
+        <v>1.9106</v>
       </c>
       <c r="K316" s="7"/>
     </row>
@@ -17493,19 +17493,19 @@
         <v>5</v>
       </c>
       <c r="E334" s="7">
-        <v>-0.001697</v>
+        <v>0.002293</v>
       </c>
       <c r="F334" s="7">
-        <v>0.049672</v>
+        <v>0.053867000000000005</v>
       </c>
       <c r="G334" s="7">
-        <v>0.047588</v>
+        <v>0.051775</v>
       </c>
       <c r="H334" s="7">
-        <v>0.204455</v>
+        <v>0.209269</v>
       </c>
       <c r="I334" s="7">
-        <v>0.337209</v>
+        <v>0.342554</v>
       </c>
       <c r="J334" s="7"/>
       <c r="K334" s="7"/>
@@ -17790,25 +17790,25 @@
         <v>7</v>
       </c>
       <c r="E343" s="7">
-        <v>0</v>
+        <v>-0.011794</v>
       </c>
       <c r="F343" s="7">
-        <v>0</v>
+        <v>-0.068829</v>
       </c>
       <c r="G343" s="7">
-        <v>0</v>
+        <v>-0.17325800000000002</v>
       </c>
       <c r="H343" s="7">
-        <v>0</v>
+        <v>-0.051531</v>
       </c>
       <c r="I343" s="7">
-        <v>0</v>
+        <v>0.645713</v>
       </c>
       <c r="J343" s="7">
-        <v>0</v>
+        <v>3.4221269999999997</v>
       </c>
       <c r="K343" s="7">
-        <v>0</v>
+        <v>10.675065</v>
       </c>
     </row>
     <row r="344" spans="1:11" x14ac:dyDescent="0.25">
@@ -17916,16 +17916,16 @@
         <v>7</v>
       </c>
       <c r="E347" s="7">
-        <v>0</v>
+        <v>-0.013756999999999998</v>
       </c>
       <c r="F347" s="7">
-        <v>0</v>
+        <v>-0.07489</v>
       </c>
       <c r="G347" s="7">
-        <v>0</v>
+        <v>-0.178706</v>
       </c>
       <c r="H347" s="7">
-        <v>0</v>
+        <v>-0.077709</v>
       </c>
       <c r="I347" s="7"/>
       <c r="J347" s="7"/>
@@ -17945,25 +17945,25 @@
         <v>7</v>
       </c>
       <c r="E348" s="7">
-        <v>0</v>
+        <v>-0.008282000000000001</v>
       </c>
       <c r="F348" s="7">
-        <v>0</v>
+        <v>-0.055434000000000004</v>
       </c>
       <c r="G348" s="7">
-        <v>0</v>
+        <v>-0.16659400000000002</v>
       </c>
       <c r="H348" s="7">
-        <v>0</v>
+        <v>-0.035125</v>
       </c>
       <c r="I348" s="7">
-        <v>0</v>
+        <v>0.67193</v>
       </c>
       <c r="J348" s="7">
-        <v>0</v>
+        <v>3.341087</v>
       </c>
       <c r="K348" s="7">
-        <v>0</v>
+        <v>11.168299999999999</v>
       </c>
     </row>
     <row r="349" spans="1:11" x14ac:dyDescent="0.25">
@@ -18112,25 +18112,25 @@
         <v>6</v>
       </c>
       <c r="E353" s="7">
-        <v>0</v>
+        <v>0.06579600000000001</v>
       </c>
       <c r="F353" s="7">
-        <v>0</v>
+        <v>0.147417</v>
       </c>
       <c r="G353" s="7">
-        <v>0</v>
+        <v>0.117602</v>
       </c>
       <c r="H353" s="7">
-        <v>0</v>
+        <v>0.302272</v>
       </c>
       <c r="I353" s="7">
-        <v>0</v>
+        <v>0.550935</v>
       </c>
       <c r="J353" s="7">
-        <v>0</v>
+        <v>1.5685120000000001</v>
       </c>
       <c r="K353" s="7">
-        <v>0</v>
+        <v>6.690396</v>
       </c>
     </row>
     <row r="354" spans="1:11" x14ac:dyDescent="0.25">
@@ -18355,25 +18355,25 @@
         <v>3</v>
       </c>
       <c r="E360" s="7">
-        <v>0</v>
+        <v>0.015486999999999999</v>
       </c>
       <c r="F360" s="7">
-        <v>0</v>
+        <v>0.062278</v>
       </c>
       <c r="G360" s="7">
-        <v>0</v>
+        <v>0.14616300000000002</v>
       </c>
       <c r="H360" s="7">
-        <v>0</v>
+        <v>0.238516</v>
       </c>
       <c r="I360" s="7">
-        <v>0</v>
+        <v>0.371501</v>
       </c>
       <c r="J360" s="7">
-        <v>0</v>
+        <v>2.176992</v>
       </c>
       <c r="K360" s="7">
-        <v>0</v>
+        <v>6.055241</v>
       </c>
     </row>
     <row r="361" spans="1:11" x14ac:dyDescent="0.25">
@@ -18425,25 +18425,25 @@
         <v>5</v>
       </c>
       <c r="E362" s="7">
-        <v>0</v>
+        <v>-0.018778</v>
       </c>
       <c r="F362" s="7">
-        <v>0</v>
+        <v>0.017962</v>
       </c>
       <c r="G362" s="7">
-        <v>0</v>
+        <v>0.179679</v>
       </c>
       <c r="H362" s="7">
-        <v>0</v>
+        <v>0.228532</v>
       </c>
       <c r="I362" s="7">
-        <v>0</v>
+        <v>0.324635</v>
       </c>
       <c r="J362" s="7">
-        <v>0</v>
+        <v>1.403544</v>
       </c>
       <c r="K362" s="7">
-        <v>0</v>
+        <v>6.107834</v>
       </c>
     </row>
     <row r="363" spans="1:11" x14ac:dyDescent="0.25">
@@ -18673,22 +18673,22 @@
       </c>
       <c r="D370" s="6"/>
       <c r="E370" s="7">
-        <v>0</v>
+        <v>0.006422</v>
       </c>
       <c r="F370" s="7">
-        <v>0</v>
+        <v>0.036472000000000004</v>
       </c>
       <c r="G370" s="7">
-        <v>0</v>
+        <v>0.124006</v>
       </c>
       <c r="H370" s="7">
-        <v>0</v>
+        <v>0.21948499999999999</v>
       </c>
       <c r="I370" s="7">
-        <v>0</v>
+        <v>0.294164</v>
       </c>
       <c r="J370" s="7">
-        <v>0</v>
+        <v>1.536507</v>
       </c>
       <c r="K370" s="7"/>
     </row>
@@ -19564,25 +19564,25 @@
       </c>
       <c r="D399" s="6"/>
       <c r="E399" s="7">
-        <v>-0.007984</v>
+        <v>-0.008025</v>
       </c>
       <c r="F399" s="7">
-        <v>0.025169</v>
+        <v>0.025127</v>
       </c>
       <c r="G399" s="7">
-        <v>0.19067399999999998</v>
+        <v>0.190626</v>
       </c>
       <c r="H399" s="7">
-        <v>0.226879</v>
+        <v>0.226829</v>
       </c>
       <c r="I399" s="7">
-        <v>0.30640999999999996</v>
+        <v>0.306356</v>
       </c>
       <c r="J399" s="7">
-        <v>1.531365</v>
+        <v>1.531261</v>
       </c>
       <c r="K399" s="7">
-        <v>6.447319</v>
+        <v>6.447012999999999</v>
       </c>
     </row>
     <row r="400" spans="1:11" x14ac:dyDescent="0.25">
@@ -19919,19 +19919,19 @@
         <v>4</v>
       </c>
       <c r="E410" s="7">
-        <v>-0.010966</v>
+        <v>-0.010749</v>
       </c>
       <c r="F410" s="7">
-        <v>0.060974</v>
+        <v>0.061205999999999997</v>
       </c>
       <c r="G410" s="7">
-        <v>0.346423</v>
+        <v>0.346717</v>
       </c>
       <c r="H410" s="7">
-        <v>0.306427</v>
+        <v>0.306713</v>
       </c>
       <c r="I410" s="7">
-        <v>0.366209</v>
+        <v>0.366509</v>
       </c>
       <c r="J410" s="7"/>
       <c r="K410" s="7"/>
@@ -19950,10 +19950,10 @@
         <v>6</v>
       </c>
       <c r="E411" s="7">
-        <v>-0.101064</v>
+        <v>-0.10278000000000001</v>
       </c>
       <c r="F411" s="7">
-        <v>-0.025234999999999997</v>
+        <v>-0.027094999999999998</v>
       </c>
       <c r="G411" s="7"/>
       <c r="H411" s="7"/>
@@ -21114,16 +21114,16 @@
         <v>6</v>
       </c>
       <c r="E447" s="7">
-        <v>-0.036104</v>
+        <v>-0.036101</v>
       </c>
       <c r="F447" s="7">
-        <v>-0.088453</v>
+        <v>-0.08845</v>
       </c>
       <c r="G447" s="7">
-        <v>0.039839</v>
+        <v>0.039842</v>
       </c>
       <c r="H447" s="7">
-        <v>0.164377</v>
+        <v>0.164381</v>
       </c>
       <c r="I447" s="7"/>
       <c r="J447" s="7"/>
@@ -21273,7 +21273,7 @@
         <v>6</v>
       </c>
       <c r="E452" s="7">
-        <v>0.011166</v>
+        <v>0.011169</v>
       </c>
       <c r="F452" s="7"/>
       <c r="G452" s="7"/>
@@ -21397,19 +21397,19 @@
         <v>6</v>
       </c>
       <c r="E456" s="7">
-        <v>-0.09898199999999999</v>
+        <v>-0.098985</v>
       </c>
       <c r="F456" s="7">
-        <v>-0.07136</v>
+        <v>-0.07136300000000001</v>
       </c>
       <c r="G456" s="7">
-        <v>0.048957</v>
+        <v>0.048954000000000004</v>
       </c>
       <c r="H456" s="7">
-        <v>0.192036</v>
+        <v>0.19203199999999998</v>
       </c>
       <c r="I456" s="7">
-        <v>0.178476</v>
+        <v>0.17847200000000002</v>
       </c>
       <c r="J456" s="7"/>
       <c r="K456" s="7"/>
@@ -21556,25 +21556,25 @@
         <v>7</v>
       </c>
       <c r="E461" s="7">
-        <v>-0.007368</v>
+        <v>-0.007372999999999999</v>
       </c>
       <c r="F461" s="7">
-        <v>-0.022354</v>
+        <v>-0.022359</v>
       </c>
       <c r="G461" s="7">
-        <v>0.068415</v>
+        <v>0.068409</v>
       </c>
       <c r="H461" s="7">
-        <v>0.189805</v>
+        <v>0.189799</v>
       </c>
       <c r="I461" s="7">
-        <v>0.22543600000000003</v>
+        <v>0.22543</v>
       </c>
       <c r="J461" s="7">
-        <v>1.3596180000000002</v>
+        <v>1.359607</v>
       </c>
       <c r="K461" s="7">
-        <v>18.230218</v>
+        <v>18.230125</v>
       </c>
     </row>
     <row r="462" spans="1:11" x14ac:dyDescent="0.25">
@@ -21725,25 +21725,25 @@
         <v>3</v>
       </c>
       <c r="E466" s="7">
-        <v>0</v>
+        <v>0.022458999999999996</v>
       </c>
       <c r="F466" s="7">
-        <v>0</v>
+        <v>0.066066</v>
       </c>
       <c r="G466" s="7">
-        <v>0</v>
+        <v>0.144531</v>
       </c>
       <c r="H466" s="7">
-        <v>0</v>
+        <v>0.22593800000000003</v>
       </c>
       <c r="I466" s="7">
-        <v>0</v>
+        <v>0.34002699999999997</v>
       </c>
       <c r="J466" s="7">
-        <v>0</v>
+        <v>2.01021</v>
       </c>
       <c r="K466" s="7">
-        <v>0</v>
+        <v>6.080286</v>
       </c>
     </row>
     <row r="467" spans="1:11" x14ac:dyDescent="0.25">
@@ -22034,19 +22034,19 @@
         <v>6</v>
       </c>
       <c r="E475" s="7">
-        <v>-0.06698</v>
+        <v>-0.066981</v>
       </c>
       <c r="F475" s="7">
-        <v>-0.035436999999999996</v>
+        <v>-0.035438</v>
       </c>
       <c r="G475" s="7">
-        <v>0.13320600000000002</v>
+        <v>0.133205</v>
       </c>
       <c r="H475" s="7">
-        <v>0.012629999999999999</v>
+        <v>0.012629</v>
       </c>
       <c r="I475" s="7">
-        <v>0.432883</v>
+        <v>0.43288200000000004</v>
       </c>
       <c r="J475" s="7"/>
       <c r="K475" s="7"/>
@@ -22265,25 +22265,25 @@
         <v>6</v>
       </c>
       <c r="E482" s="7">
-        <v>-0.058708</v>
+        <v>-0.058599</v>
       </c>
       <c r="F482" s="7">
-        <v>-0.036355</v>
+        <v>-0.036243</v>
       </c>
       <c r="G482" s="7">
-        <v>0.05168300000000001</v>
+        <v>0.051805000000000004</v>
       </c>
       <c r="H482" s="7">
-        <v>0.250552</v>
+        <v>0.250697</v>
       </c>
       <c r="I482" s="7">
-        <v>0.276596</v>
+        <v>0.276744</v>
       </c>
       <c r="J482" s="7">
-        <v>1.637944</v>
+        <v>1.63825</v>
       </c>
       <c r="K482" s="7">
-        <v>16.065657</v>
+        <v>16.067634</v>
       </c>
     </row>
     <row r="483" spans="1:11" x14ac:dyDescent="0.25">
@@ -22403,16 +22403,16 @@
         <v>3</v>
       </c>
       <c r="E486" s="7">
-        <v>0</v>
+        <v>0.027146</v>
       </c>
       <c r="F486" s="7">
-        <v>0</v>
+        <v>0.09353500000000001</v>
       </c>
       <c r="G486" s="7">
-        <v>0</v>
+        <v>0.22283799999999998</v>
       </c>
       <c r="H486" s="7">
-        <v>0</v>
+        <v>0.329861</v>
       </c>
       <c r="I486" s="7"/>
       <c r="J486" s="7"/>
@@ -22432,22 +22432,22 @@
         <v>3</v>
       </c>
       <c r="E487" s="7">
-        <v>0</v>
+        <v>0.029801</v>
       </c>
       <c r="F487" s="7">
-        <v>0</v>
+        <v>0.12091400000000001</v>
       </c>
       <c r="G487" s="7">
-        <v>0</v>
+        <v>0.269213</v>
       </c>
       <c r="H487" s="7">
-        <v>0</v>
+        <v>0.383615</v>
       </c>
       <c r="I487" s="7">
-        <v>0</v>
+        <v>0.602912</v>
       </c>
       <c r="J487" s="7">
-        <v>0</v>
+        <v>2.1457859999999997</v>
       </c>
       <c r="K487" s="7"/>
     </row>
@@ -22529,22 +22529,22 @@
         <v>3</v>
       </c>
       <c r="E490" s="7">
-        <v>0.034979</v>
+        <v>0.034971999999999996</v>
       </c>
       <c r="F490" s="7">
-        <v>0.113768</v>
+        <v>0.11376099999999999</v>
       </c>
       <c r="G490" s="7">
-        <v>0.189255</v>
+        <v>0.18924700000000003</v>
       </c>
       <c r="H490" s="7">
-        <v>0.271892</v>
+        <v>0.271884</v>
       </c>
       <c r="I490" s="7">
-        <v>0.40143900000000005</v>
+        <v>0.40143</v>
       </c>
       <c r="J490" s="7">
-        <v>2.028046</v>
+        <v>2.028027</v>
       </c>
       <c r="K490" s="7"/>
     </row>
@@ -22723,22 +22723,22 @@
         <v>5</v>
       </c>
       <c r="E496" s="7">
-        <v>-0.028618</v>
+        <v>-0.029449999999999997</v>
       </c>
       <c r="F496" s="7">
-        <v>0.0029709999999999997</v>
+        <v>0.002113</v>
       </c>
       <c r="G496" s="7">
-        <v>0.34476999999999997</v>
+        <v>0.343619</v>
       </c>
       <c r="H496" s="7">
-        <v>0.40598100000000004</v>
+        <v>0.404778</v>
       </c>
       <c r="I496" s="7">
-        <v>0.506758</v>
+        <v>0.505468</v>
       </c>
       <c r="J496" s="7">
-        <v>2.19033</v>
+        <v>2.187599</v>
       </c>
       <c r="K496" s="7"/>
     </row>
@@ -22919,16 +22919,16 @@
         <v>6</v>
       </c>
       <c r="E502" s="7">
-        <v>0.014728000000000002</v>
+        <v>0.014726</v>
       </c>
       <c r="F502" s="7">
-        <v>-0.04827</v>
+        <v>-0.048272</v>
       </c>
       <c r="G502" s="7">
-        <v>0.042821</v>
+        <v>0.042817999999999995</v>
       </c>
       <c r="H502" s="7">
-        <v>0.088047</v>
+        <v>0.08804500000000001</v>
       </c>
       <c r="I502" s="7"/>
       <c r="J502" s="7"/>
@@ -25854,16 +25854,16 @@
         <v>6</v>
       </c>
       <c r="E595" s="7">
-        <v>0.091594</v>
+        <v>0.091677</v>
       </c>
       <c r="F595" s="7">
-        <v>0.14372400000000002</v>
+        <v>0.143811</v>
       </c>
       <c r="G595" s="7">
-        <v>0.052652000000000004</v>
+        <v>0.052732</v>
       </c>
       <c r="H595" s="7">
-        <v>0.221885</v>
+        <v>0.221978</v>
       </c>
       <c r="I595" s="7"/>
       <c r="J595" s="7"/>
@@ -26009,22 +26009,22 @@
         <v>6</v>
       </c>
       <c r="E600" s="7">
-        <v>-0.016354</v>
+        <v>-0.018975</v>
       </c>
       <c r="F600" s="7">
-        <v>-0.033273000000000004</v>
+        <v>-0.035849</v>
       </c>
       <c r="G600" s="7">
-        <v>0.143344</v>
+        <v>0.140297</v>
       </c>
       <c r="H600" s="7">
-        <v>0.284698</v>
+        <v>0.281275</v>
       </c>
       <c r="I600" s="7">
-        <v>0.36607100000000004</v>
+        <v>0.362431</v>
       </c>
       <c r="J600" s="7">
-        <v>1.7285579999999998</v>
+        <v>1.721287</v>
       </c>
       <c r="K600" s="7"/>
     </row>
@@ -26042,25 +26042,25 @@
         <v>7</v>
       </c>
       <c r="E601" s="7">
-        <v>-0.016715999999999998</v>
+        <v>-0.010703</v>
       </c>
       <c r="F601" s="7">
-        <v>-0.06676</v>
+        <v>-0.061054000000000004</v>
       </c>
       <c r="G601" s="7">
-        <v>-0.153683</v>
+        <v>-0.148508</v>
       </c>
       <c r="H601" s="7">
-        <v>-0.054498</v>
+        <v>-0.048716999999999996</v>
       </c>
       <c r="I601" s="7">
-        <v>0.6216170000000001</v>
+        <v>0.631533</v>
       </c>
       <c r="J601" s="7">
-        <v>3.4867250000000003</v>
+        <v>3.5141590000000003</v>
       </c>
       <c r="K601" s="7">
-        <v>11.648239</v>
+        <v>11.725577000000001</v>
       </c>
     </row>
     <row r="602" spans="1:11" x14ac:dyDescent="0.25">
@@ -26077,25 +26077,25 @@
         <v>6</v>
       </c>
       <c r="E602" s="7">
-        <v>0.017377</v>
+        <v>-0.0038900000000000002</v>
       </c>
       <c r="F602" s="7">
-        <v>-0.030368</v>
+        <v>-0.050637999999999996</v>
       </c>
       <c r="G602" s="7">
-        <v>0.012309</v>
+        <v>-0.008852</v>
       </c>
       <c r="H602" s="7">
-        <v>-0.068747</v>
+        <v>-0.088214</v>
       </c>
       <c r="I602" s="7">
-        <v>-0.061448</v>
+        <v>-0.081067</v>
       </c>
       <c r="J602" s="7">
-        <v>0.427919</v>
+        <v>0.398069</v>
       </c>
       <c r="K602" s="7">
-        <v>3.054818</v>
+        <v>2.970055</v>
       </c>
     </row>
     <row r="603" spans="1:11" x14ac:dyDescent="0.25">
@@ -26176,25 +26176,25 @@
         <v>6</v>
       </c>
       <c r="E605" s="7">
-        <v>0.002147</v>
+        <v>-0.000974</v>
       </c>
       <c r="F605" s="7">
-        <v>0.036158</v>
+        <v>0.032931</v>
       </c>
       <c r="G605" s="7">
-        <v>-0.068529</v>
+        <v>-0.071429</v>
       </c>
       <c r="H605" s="7">
-        <v>0.092477</v>
+        <v>0.089075</v>
       </c>
       <c r="I605" s="7">
-        <v>0.35192799999999996</v>
+        <v>0.34771799999999997</v>
       </c>
       <c r="J605" s="7">
-        <v>3.089289</v>
+        <v>3.0765550000000004</v>
       </c>
       <c r="K605" s="7">
-        <v>13.166685</v>
+        <v>13.122572</v>
       </c>
     </row>
     <row r="606" spans="1:11" x14ac:dyDescent="0.25">
@@ -26810,22 +26810,22 @@
         <v>5</v>
       </c>
       <c r="E625" s="7">
-        <v>0.02862</v>
+        <v>0.020583</v>
       </c>
       <c r="F625" s="7">
-        <v>0.032167</v>
+        <v>0.024102000000000002</v>
       </c>
       <c r="G625" s="7">
-        <v>0.113355</v>
+        <v>0.104656</v>
       </c>
       <c r="H625" s="7">
-        <v>0.20061800000000002</v>
+        <v>0.191237</v>
       </c>
       <c r="I625" s="7">
-        <v>0.26508</v>
+        <v>0.255195</v>
       </c>
       <c r="J625" s="7">
-        <v>1.10535</v>
+        <v>1.0889</v>
       </c>
       <c r="K625" s="7"/>
     </row>
@@ -27033,19 +27033,19 @@
         <v>2</v>
       </c>
       <c r="E632" s="7">
-        <v>0.031021</v>
+        <v>0.031638</v>
       </c>
       <c r="F632" s="7">
-        <v>0.103809</v>
+        <v>0.10446899999999999</v>
       </c>
       <c r="G632" s="7">
-        <v>0.22776800000000003</v>
+        <v>0.228502</v>
       </c>
       <c r="H632" s="7">
-        <v>0.33987</v>
+        <v>0.34067100000000006</v>
       </c>
       <c r="I632" s="7">
-        <v>0.5406580000000001</v>
+        <v>0.5415800000000001</v>
       </c>
       <c r="J632" s="7"/>
       <c r="K632" s="7"/>
@@ -27130,19 +27130,19 @@
         <v>5</v>
       </c>
       <c r="E635" s="7">
-        <v>0</v>
+        <v>0.026018</v>
       </c>
       <c r="F635" s="7">
-        <v>0</v>
+        <v>0.08940899999999999</v>
       </c>
       <c r="G635" s="7">
-        <v>0</v>
+        <v>0.180385</v>
       </c>
       <c r="H635" s="7">
-        <v>0</v>
+        <v>0.051071</v>
       </c>
       <c r="I635" s="7">
-        <v>0</v>
+        <v>0.1242</v>
       </c>
       <c r="J635" s="7"/>
       <c r="K635" s="7"/>
@@ -27161,22 +27161,22 @@
         <v>3</v>
       </c>
       <c r="E636" s="7">
-        <v>0</v>
+        <v>0.016382</v>
       </c>
       <c r="F636" s="7">
-        <v>0</v>
+        <v>0.027139000000000003</v>
       </c>
       <c r="G636" s="7">
-        <v>0</v>
+        <v>0.116824</v>
       </c>
       <c r="H636" s="7">
-        <v>0</v>
+        <v>0.171364</v>
       </c>
       <c r="I636" s="7">
-        <v>0</v>
+        <v>0.315262</v>
       </c>
       <c r="J636" s="7">
-        <v>0</v>
+        <v>1.720882</v>
       </c>
       <c r="K636" s="7"/>
     </row>
@@ -27725,22 +27725,22 @@
         <v>1</v>
       </c>
       <c r="E654" s="7">
-        <v>0.031179000000000002</v>
+        <v>0.031169</v>
       </c>
       <c r="F654" s="7">
-        <v>0.10147</v>
+        <v>0.10146000000000001</v>
       </c>
       <c r="G654" s="7">
-        <v>0.217716</v>
+        <v>0.21770399999999998</v>
       </c>
       <c r="H654" s="7">
-        <v>0.310875</v>
+        <v>0.310863</v>
       </c>
       <c r="I654" s="7">
-        <v>0.474775</v>
+        <v>0.47476100000000004</v>
       </c>
       <c r="J654" s="7">
-        <v>2.656021</v>
+        <v>2.655987</v>
       </c>
       <c r="K654" s="7"/>
     </row>
@@ -28099,22 +28099,22 @@
       </c>
       <c r="D666" s="6"/>
       <c r="E666" s="7">
-        <v>0.030892</v>
+        <v>0.030881</v>
       </c>
       <c r="F666" s="7">
-        <v>0.10068099999999999</v>
+        <v>0.10066900000000001</v>
       </c>
       <c r="G666" s="7">
-        <v>0.21534199999999998</v>
+        <v>0.21532800000000002</v>
       </c>
       <c r="H666" s="7">
-        <v>0.307052</v>
+        <v>0.30703800000000003</v>
       </c>
       <c r="I666" s="7">
-        <v>0.47031799999999996</v>
+        <v>0.470302</v>
       </c>
       <c r="J666" s="7">
-        <v>2.6330669999999996</v>
+        <v>2.6330270000000002</v>
       </c>
       <c r="K666" s="7"/>
     </row>
@@ -28357,22 +28357,22 @@
         <v>3</v>
       </c>
       <c r="E674" s="7">
-        <v>0.035787</v>
+        <v>0.035777</v>
       </c>
       <c r="F674" s="7">
-        <v>0.092636</v>
+        <v>0.09262600000000001</v>
       </c>
       <c r="G674" s="7">
-        <v>0.182521</v>
+        <v>0.18251</v>
       </c>
       <c r="H674" s="7">
-        <v>0.193231</v>
+        <v>0.19322</v>
       </c>
       <c r="I674" s="7">
-        <v>0.372896</v>
+        <v>0.372883</v>
       </c>
       <c r="J674" s="7">
-        <v>1.64737</v>
+        <v>1.647346</v>
       </c>
       <c r="K674" s="7"/>
     </row>
@@ -28390,25 +28390,25 @@
         <v>4</v>
       </c>
       <c r="E675" s="7">
-        <v>0.027478</v>
+        <v>0.027468</v>
       </c>
       <c r="F675" s="7">
-        <v>0.075902</v>
+        <v>0.075892</v>
       </c>
       <c r="G675" s="7">
-        <v>0.16217199999999998</v>
+        <v>0.162161</v>
       </c>
       <c r="H675" s="7">
-        <v>0.221696</v>
+        <v>0.221684</v>
       </c>
       <c r="I675" s="7">
-        <v>0.374442</v>
+        <v>0.374429</v>
       </c>
       <c r="J675" s="7">
-        <v>1.8577789999999998</v>
+        <v>1.8577510000000002</v>
       </c>
       <c r="K675" s="7">
-        <v>5.23019</v>
+        <v>5.23013</v>
       </c>
     </row>
     <row r="676" spans="1:11" x14ac:dyDescent="0.25">
@@ -28458,10 +28458,10 @@
         <v>3</v>
       </c>
       <c r="E677" s="7">
-        <v>0.002948</v>
+        <v>0.002946</v>
       </c>
       <c r="F677" s="7">
-        <v>0.060956</v>
+        <v>0.060953999999999994</v>
       </c>
       <c r="G677" s="7"/>
       <c r="H677" s="7"/>
@@ -28549,25 +28549,25 @@
         <v>5</v>
       </c>
       <c r="E680" s="7">
-        <v>0</v>
+        <v>-0.025002</v>
       </c>
       <c r="F680" s="7">
-        <v>0</v>
+        <v>-0.023072</v>
       </c>
       <c r="G680" s="7">
-        <v>0</v>
+        <v>0.011126</v>
       </c>
       <c r="H680" s="7">
-        <v>0</v>
+        <v>0.119132</v>
       </c>
       <c r="I680" s="7">
-        <v>0</v>
+        <v>0.215979</v>
       </c>
       <c r="J680" s="7">
-        <v>0</v>
+        <v>1.5091970000000001</v>
       </c>
       <c r="K680" s="7">
-        <v>0</v>
+        <v>6.398078000000001</v>
       </c>
     </row>
     <row r="681" spans="1:11" x14ac:dyDescent="0.25">
@@ -28582,22 +28582,22 @@
       </c>
       <c r="D681" s="6"/>
       <c r="E681" s="7">
-        <v>0.013491</v>
+        <v>0.013833999999999999</v>
       </c>
       <c r="F681" s="7">
-        <v>0.048875</v>
+        <v>0.04923</v>
       </c>
       <c r="G681" s="7">
-        <v>0.135205</v>
+        <v>0.135589</v>
       </c>
       <c r="H681" s="7">
-        <v>0.21412299999999998</v>
+        <v>0.21453399999999997</v>
       </c>
       <c r="I681" s="7">
-        <v>0.319501</v>
+        <v>0.319948</v>
       </c>
       <c r="J681" s="7">
-        <v>1.4325040000000002</v>
+        <v>1.433328</v>
       </c>
       <c r="K681" s="7"/>
     </row>
@@ -28615,25 +28615,25 @@
         <v>4</v>
       </c>
       <c r="E682" s="7">
-        <v>0.022887</v>
+        <v>0.022888000000000002</v>
       </c>
       <c r="F682" s="7">
-        <v>0.061883999999999995</v>
+        <v>0.061886000000000004</v>
       </c>
       <c r="G682" s="7">
-        <v>0.119746</v>
+        <v>0.11974800000000001</v>
       </c>
       <c r="H682" s="7">
-        <v>0.20607199999999998</v>
+        <v>0.20607399999999998</v>
       </c>
       <c r="I682" s="7">
-        <v>0.342078</v>
+        <v>0.342081</v>
       </c>
       <c r="J682" s="7">
-        <v>1.736404</v>
+        <v>1.73641</v>
       </c>
       <c r="K682" s="7">
-        <v>6.455075000000001</v>
+        <v>6.455089</v>
       </c>
     </row>
     <row r="683" spans="1:11" x14ac:dyDescent="0.25">
@@ -28753,22 +28753,22 @@
         <v>6</v>
       </c>
       <c r="E686" s="7">
-        <v>0.002302</v>
+        <v>-0.002781</v>
       </c>
       <c r="F686" s="7">
-        <v>0.037811</v>
+        <v>0.032548</v>
       </c>
       <c r="G686" s="7">
-        <v>-0.013111</v>
+        <v>-0.018115000000000003</v>
       </c>
       <c r="H686" s="7">
-        <v>0.126843</v>
+        <v>0.121129</v>
       </c>
       <c r="I686" s="7">
-        <v>0.170579</v>
+        <v>0.164644</v>
       </c>
       <c r="J686" s="7">
-        <v>0.684442</v>
+        <v>0.6759010000000001</v>
       </c>
       <c r="K686" s="7"/>
     </row>
@@ -28786,22 +28786,22 @@
         <v>3</v>
       </c>
       <c r="E687" s="7">
-        <v>0.018453</v>
+        <v>0.010945</v>
       </c>
       <c r="F687" s="7">
-        <v>0.06132</v>
+        <v>0.053495</v>
       </c>
       <c r="G687" s="7">
-        <v>0.14654</v>
+        <v>0.138088</v>
       </c>
       <c r="H687" s="7">
-        <v>0.250586</v>
+        <v>0.241367</v>
       </c>
       <c r="I687" s="7">
-        <v>0.412409</v>
+        <v>0.40199599999999996</v>
       </c>
       <c r="J687" s="7">
-        <v>2.195872</v>
+        <v>2.172312</v>
       </c>
       <c r="K687" s="7"/>
     </row>
@@ -28887,25 +28887,25 @@
         <v>6</v>
       </c>
       <c r="E690" s="7">
-        <v>-0.029039000000000002</v>
+        <v>-0.029853</v>
       </c>
       <c r="F690" s="7">
-        <v>-0.0029360000000000002</v>
+        <v>-0.0037719999999999997</v>
       </c>
       <c r="G690" s="7">
-        <v>0.363119</v>
+        <v>0.361976</v>
       </c>
       <c r="H690" s="7">
-        <v>0.39785200000000004</v>
+        <v>0.39668</v>
       </c>
       <c r="I690" s="7">
-        <v>0.51298</v>
+        <v>0.511711</v>
       </c>
       <c r="J690" s="7">
-        <v>2.6288350000000005</v>
+        <v>2.625793</v>
       </c>
       <c r="K690" s="7">
-        <v>10.497402999999998</v>
+        <v>10.487764</v>
       </c>
     </row>
     <row r="691" spans="1:11" x14ac:dyDescent="0.25">
@@ -28957,25 +28957,25 @@
         <v>2</v>
       </c>
       <c r="E692" s="7">
-        <v>0.0302</v>
+        <v>0.030196</v>
       </c>
       <c r="F692" s="7">
-        <v>0.098996</v>
+        <v>0.09899200000000001</v>
       </c>
       <c r="G692" s="7">
-        <v>0.20924600000000002</v>
+        <v>0.20924199999999998</v>
       </c>
       <c r="H692" s="7">
-        <v>0.298257</v>
+        <v>0.298253</v>
       </c>
       <c r="I692" s="7">
-        <v>0.45445500000000005</v>
+        <v>0.454449</v>
       </c>
       <c r="J692" s="7">
-        <v>2.522175</v>
+        <v>2.522163</v>
       </c>
       <c r="K692" s="7">
-        <v>4.091279</v>
+        <v>4.09126</v>
       </c>
     </row>
     <row r="693" spans="1:11" x14ac:dyDescent="0.25">
@@ -28992,25 +28992,25 @@
         <v>3</v>
       </c>
       <c r="E693" s="7">
-        <v>0.030302</v>
+        <v>0.030296</v>
       </c>
       <c r="F693" s="7">
-        <v>0.09955299999999999</v>
+        <v>0.099546</v>
       </c>
       <c r="G693" s="7">
-        <v>0.209362</v>
+        <v>0.209355</v>
       </c>
       <c r="H693" s="7">
-        <v>0.302022</v>
+        <v>0.302014</v>
       </c>
       <c r="I693" s="7">
-        <v>0.455362</v>
+        <v>0.45535400000000004</v>
       </c>
       <c r="J693" s="7">
-        <v>2.500136</v>
+        <v>2.500115</v>
       </c>
       <c r="K693" s="7">
-        <v>4.4124099999999995</v>
+        <v>4.412377</v>
       </c>
     </row>
     <row r="694" spans="1:11" x14ac:dyDescent="0.25">
@@ -29091,22 +29091,22 @@
         <v>2</v>
       </c>
       <c r="E696" s="7">
-        <v>0.031027999999999997</v>
+        <v>0.031859</v>
       </c>
       <c r="F696" s="7">
-        <v>0.10191499999999999</v>
+        <v>0.102803</v>
       </c>
       <c r="G696" s="7">
-        <v>0.222192</v>
+        <v>0.223177</v>
       </c>
       <c r="H696" s="7">
-        <v>0.318959</v>
+        <v>0.32002200000000003</v>
       </c>
       <c r="I696" s="7">
-        <v>0.482179</v>
+        <v>0.483373</v>
       </c>
       <c r="J696" s="7">
-        <v>2.521665</v>
+        <v>2.524504</v>
       </c>
       <c r="K696" s="7"/>
     </row>
@@ -29611,22 +29611,22 @@
         <v>6</v>
       </c>
       <c r="E712" s="7">
-        <v>-0.003715</v>
+        <v>-0.003636</v>
       </c>
       <c r="F712" s="7">
-        <v>-0.015913</v>
+        <v>-0.015835</v>
       </c>
       <c r="G712" s="7">
-        <v>-0.090621</v>
+        <v>-0.090549</v>
       </c>
       <c r="H712" s="7">
-        <v>0.021692999999999997</v>
+        <v>0.021774</v>
       </c>
       <c r="I712" s="7">
-        <v>0.503781</v>
+        <v>0.5039009999999999</v>
       </c>
       <c r="J712" s="7">
-        <v>2.6801389999999996</v>
+        <v>2.680431</v>
       </c>
       <c r="K712" s="7"/>
     </row>
@@ -29642,25 +29642,25 @@
       </c>
       <c r="D713" s="6"/>
       <c r="E713" s="7">
-        <v>0.028002</v>
+        <v>0.027997</v>
       </c>
       <c r="F713" s="7">
-        <v>0.09294000000000001</v>
+        <v>0.092935</v>
       </c>
       <c r="G713" s="7">
-        <v>0.197469</v>
+        <v>0.19746300000000003</v>
       </c>
       <c r="H713" s="7">
-        <v>0.28027799999999997</v>
+        <v>0.280271</v>
       </c>
       <c r="I713" s="7">
-        <v>0.417384</v>
+        <v>0.41737699999999994</v>
       </c>
       <c r="J713" s="7">
-        <v>1.5799029999999998</v>
+        <v>1.57989</v>
       </c>
       <c r="K713" s="7">
-        <v>3.7968990000000002</v>
+        <v>3.796875</v>
       </c>
     </row>
     <row r="714" spans="1:11" x14ac:dyDescent="0.25">
@@ -29741,22 +29741,22 @@
         <v>6</v>
       </c>
       <c r="E716" s="7">
-        <v>0.074718</v>
+        <v>0.074368</v>
       </c>
       <c r="F716" s="7">
-        <v>0.156662</v>
+        <v>0.156286</v>
       </c>
       <c r="G716" s="7">
-        <v>0.156728</v>
+        <v>0.156351</v>
       </c>
       <c r="H716" s="7">
-        <v>0.38738100000000003</v>
+        <v>0.386929</v>
       </c>
       <c r="I716" s="7">
-        <v>0.594059</v>
+        <v>0.59354</v>
       </c>
       <c r="J716" s="7">
-        <v>1.611175</v>
+        <v>1.610325</v>
       </c>
       <c r="K716" s="7"/>
     </row>
@@ -29952,19 +29952,19 @@
         <v>4</v>
       </c>
       <c r="E723" s="7">
-        <v>0.015463</v>
+        <v>0.00063</v>
       </c>
       <c r="F723" s="7">
-        <v>0.08137499999999999</v>
+        <v>0.065579</v>
       </c>
       <c r="G723" s="7">
-        <v>0.25733</v>
+        <v>0.238964</v>
       </c>
       <c r="H723" s="7">
-        <v>0.447562</v>
+        <v>0.426417</v>
       </c>
       <c r="I723" s="7">
-        <v>0.608564</v>
+        <v>0.585067</v>
       </c>
       <c r="J723" s="7"/>
       <c r="K723" s="7"/>
@@ -30243,22 +30243,22 @@
         <v>4</v>
       </c>
       <c r="E732" s="7">
-        <v>-0.043602</v>
+        <v>-0.04697199999999999</v>
       </c>
       <c r="F732" s="7">
-        <v>0.001399</v>
+        <v>-0.0021290000000000002</v>
       </c>
       <c r="G732" s="7">
-        <v>0.118127</v>
+        <v>0.114188</v>
       </c>
       <c r="H732" s="7">
-        <v>0.215258</v>
+        <v>0.210977</v>
       </c>
       <c r="I732" s="7">
-        <v>0.364475</v>
+        <v>0.359668</v>
       </c>
       <c r="J732" s="7">
-        <v>1.8403530000000001</v>
+        <v>1.830347</v>
       </c>
       <c r="K732" s="7"/>
     </row>
@@ -30491,22 +30491,22 @@
         <v>6</v>
       </c>
       <c r="E740" s="7">
-        <v>-0.049082</v>
+        <v>-0.050469</v>
       </c>
       <c r="F740" s="7">
-        <v>-0.08877800000000001</v>
+        <v>-0.090106</v>
       </c>
       <c r="G740" s="7">
-        <v>0.07653599999999999</v>
+        <v>0.074966</v>
       </c>
       <c r="H740" s="7">
-        <v>0.228548</v>
+        <v>0.226757</v>
       </c>
       <c r="I740" s="7">
-        <v>0.577894</v>
+        <v>0.575593</v>
       </c>
       <c r="J740" s="7">
-        <v>1.852948</v>
+        <v>1.848788</v>
       </c>
       <c r="K740" s="7"/>
     </row>
@@ -32727,7 +32727,7 @@
         <v>6</v>
       </c>
       <c r="E812" s="7">
-        <v>0.071627</v>
+        <v>0.071406</v>
       </c>
       <c r="F812" s="7"/>
       <c r="G812" s="7"/>
@@ -33184,22 +33184,22 @@
         <v>6</v>
       </c>
       <c r="E827" s="7">
-        <v>-0.042030000000000005</v>
+        <v>-0.032582</v>
       </c>
       <c r="F827" s="7">
-        <v>0.006226000000000001</v>
+        <v>0.016151</v>
       </c>
       <c r="G827" s="7">
-        <v>0.151657</v>
+        <v>0.163016</v>
       </c>
       <c r="H827" s="7">
-        <v>0.273951</v>
+        <v>0.28651499999999996</v>
       </c>
       <c r="I827" s="7">
-        <v>0.472916</v>
+        <v>0.487443</v>
       </c>
       <c r="J827" s="7">
-        <v>1.6438560000000002</v>
+        <v>1.669932</v>
       </c>
       <c r="K827" s="7"/>
     </row>
@@ -33316,19 +33316,19 @@
         <v>2</v>
       </c>
       <c r="E831" s="7">
-        <v>0.020349</v>
+        <v>0.020352000000000002</v>
       </c>
       <c r="F831" s="7">
-        <v>0.076464</v>
+        <v>0.07646700000000001</v>
       </c>
       <c r="G831" s="7">
-        <v>0.185061</v>
+        <v>0.185064</v>
       </c>
       <c r="H831" s="7">
-        <v>0.26672</v>
+        <v>0.266723</v>
       </c>
       <c r="I831" s="7">
-        <v>0.38608600000000004</v>
+        <v>0.38609000000000004</v>
       </c>
       <c r="J831" s="7"/>
       <c r="K831" s="7"/>
@@ -33347,22 +33347,22 @@
         <v>6</v>
       </c>
       <c r="E832" s="7">
-        <v>0.010249</v>
+        <v>0.010447999999999999</v>
       </c>
       <c r="F832" s="7">
-        <v>0.14075</v>
+        <v>0.140975</v>
       </c>
       <c r="G832" s="7">
-        <v>0.22075199999999998</v>
+        <v>0.220993</v>
       </c>
       <c r="H832" s="7">
-        <v>0.31015899999999996</v>
+        <v>0.310417</v>
       </c>
       <c r="I832" s="7">
-        <v>0.6557729999999999</v>
+        <v>0.656099</v>
       </c>
       <c r="J832" s="7">
-        <v>1.369765</v>
+        <v>1.3702320000000001</v>
       </c>
       <c r="K832" s="7"/>
     </row>
@@ -33890,19 +33890,19 @@
         <v>6</v>
       </c>
       <c r="E849" s="7">
-        <v>0</v>
+        <v>-0.09763999999999999</v>
       </c>
       <c r="F849" s="7">
-        <v>0</v>
+        <v>-0.132371</v>
       </c>
       <c r="G849" s="7">
-        <v>0</v>
+        <v>-0.037897</v>
       </c>
       <c r="H849" s="7">
-        <v>0</v>
+        <v>0.119342</v>
       </c>
       <c r="I849" s="7">
-        <v>0</v>
+        <v>0.3189</v>
       </c>
       <c r="J849" s="7"/>
       <c r="K849" s="7"/>
@@ -33921,7 +33921,7 @@
         <v>5</v>
       </c>
       <c r="E850" s="7">
-        <v>0</v>
+        <v>-0.018874</v>
       </c>
       <c r="F850" s="7"/>
       <c r="G850" s="7"/>
@@ -33944,19 +33944,19 @@
         <v>5</v>
       </c>
       <c r="E851" s="7">
-        <v>0.017967</v>
+        <v>0.008482</v>
       </c>
       <c r="F851" s="7">
-        <v>0.044049</v>
+        <v>0.034321000000000004</v>
       </c>
       <c r="G851" s="7">
-        <v>0.139568</v>
+        <v>0.12895</v>
       </c>
       <c r="H851" s="7">
-        <v>0.288711</v>
+        <v>0.27670300000000003</v>
       </c>
       <c r="I851" s="7">
-        <v>0.416543</v>
+        <v>0.403345</v>
       </c>
       <c r="J851" s="7"/>
       <c r="K851" s="7"/>
@@ -34083,16 +34083,16 @@
         <v>6</v>
       </c>
       <c r="E856" s="7">
-        <v>0</v>
+        <v>0.011291</v>
       </c>
       <c r="F856" s="7">
-        <v>0</v>
+        <v>0.011733</v>
       </c>
       <c r="G856" s="7">
-        <v>0</v>
+        <v>0.087171</v>
       </c>
       <c r="H856" s="7">
-        <v>0</v>
+        <v>0.43857300000000005</v>
       </c>
       <c r="I856" s="7"/>
       <c r="J856" s="7"/>
@@ -34393,19 +34393,19 @@
         <v>4</v>
       </c>
       <c r="E866" s="7">
-        <v>0.017286</v>
+        <v>0.011704</v>
       </c>
       <c r="F866" s="7">
-        <v>0.054675</v>
+        <v>0.048888</v>
       </c>
       <c r="G866" s="7">
-        <v>0.152083</v>
+        <v>0.145761</v>
       </c>
       <c r="H866" s="7">
-        <v>0.275522</v>
+        <v>0.268523</v>
       </c>
       <c r="I866" s="7">
-        <v>0.48184399999999994</v>
+        <v>0.473713</v>
       </c>
       <c r="J866" s="7"/>
       <c r="K866" s="7"/>
@@ -34550,19 +34550,19 @@
         <v>6</v>
       </c>
       <c r="E871" s="7">
-        <v>0.129819</v>
+        <v>0.12783899999999998</v>
       </c>
       <c r="F871" s="7">
-        <v>0.152361</v>
+        <v>0.150342</v>
       </c>
       <c r="G871" s="7">
-        <v>0.221335</v>
+        <v>0.219196</v>
       </c>
       <c r="H871" s="7">
-        <v>0.42355</v>
+        <v>0.42105600000000004</v>
       </c>
       <c r="I871" s="7">
-        <v>0.180507</v>
+        <v>0.178438</v>
       </c>
       <c r="J871" s="7"/>
       <c r="K871" s="7"/>
@@ -35057,22 +35057,22 @@
         <v>3</v>
       </c>
       <c r="E886" s="7">
-        <v>0</v>
+        <v>0.029618000000000002</v>
       </c>
       <c r="F886" s="7">
-        <v>0</v>
+        <v>0.09429</v>
       </c>
       <c r="G886" s="7">
-        <v>0</v>
+        <v>0.19759000000000002</v>
       </c>
       <c r="H886" s="7">
-        <v>0</v>
+        <v>0.296523</v>
       </c>
       <c r="I886" s="7">
-        <v>0</v>
+        <v>0.453854</v>
       </c>
       <c r="J886" s="7">
-        <v>0</v>
+        <v>2.367431</v>
       </c>
       <c r="K886" s="7"/>
     </row>
@@ -35193,19 +35193,19 @@
         <v>6</v>
       </c>
       <c r="E890" s="7">
-        <v>-0.029676</v>
+        <v>-0.030229</v>
       </c>
       <c r="F890" s="7">
-        <v>0.00038899999999999997</v>
+        <v>-0.000181</v>
       </c>
       <c r="G890" s="7">
-        <v>0.405076</v>
+        <v>0.40427599999999997</v>
       </c>
       <c r="H890" s="7">
-        <v>0.457159</v>
+        <v>0.456329</v>
       </c>
       <c r="I890" s="7">
-        <v>0.588465</v>
+        <v>0.58756</v>
       </c>
       <c r="J890" s="7"/>
       <c r="K890" s="7"/>
@@ -35762,25 +35762,25 @@
         <v>6</v>
       </c>
       <c r="E907" s="7">
-        <v>0</v>
+        <v>-0.009142</v>
       </c>
       <c r="F907" s="7">
-        <v>0</v>
+        <v>-0.015497</v>
       </c>
       <c r="G907" s="7">
-        <v>0</v>
+        <v>0.108151</v>
       </c>
       <c r="H907" s="7">
-        <v>0</v>
+        <v>0.22031199999999998</v>
       </c>
       <c r="I907" s="7">
-        <v>0</v>
+        <v>0.284126</v>
       </c>
       <c r="J907" s="7">
-        <v>0</v>
+        <v>1.157349</v>
       </c>
       <c r="K907" s="7">
-        <v>0</v>
+        <v>4.420669</v>
       </c>
     </row>
     <row r="908" spans="1:11" x14ac:dyDescent="0.25">
@@ -35797,22 +35797,22 @@
         <v>4</v>
       </c>
       <c r="E908" s="7">
-        <v>0</v>
+        <v>0.0066359999999999995</v>
       </c>
       <c r="F908" s="7">
-        <v>0</v>
+        <v>0.021165</v>
       </c>
       <c r="G908" s="7">
-        <v>0</v>
+        <v>0.103613</v>
       </c>
       <c r="H908" s="7">
-        <v>0</v>
+        <v>0.21609</v>
       </c>
       <c r="I908" s="7">
-        <v>0</v>
+        <v>0.365007</v>
       </c>
       <c r="J908" s="7">
-        <v>0</v>
+        <v>1.6770249999999998</v>
       </c>
       <c r="K908" s="7"/>
     </row>
@@ -36197,19 +36197,19 @@
         <v>2</v>
       </c>
       <c r="E920" s="7">
-        <v>0.026394</v>
+        <v>0.022947000000000002</v>
       </c>
       <c r="F920" s="7">
-        <v>0.073451</v>
+        <v>0.069846</v>
       </c>
       <c r="G920" s="7">
-        <v>0.170114</v>
+        <v>0.166184</v>
       </c>
       <c r="H920" s="7">
-        <v>0.277163</v>
+        <v>0.272873</v>
       </c>
       <c r="I920" s="7">
-        <v>0.42965200000000003</v>
+        <v>0.42485</v>
       </c>
       <c r="J920" s="7"/>
       <c r="K920" s="7"/>
@@ -36356,25 +36356,25 @@
         <v>6</v>
       </c>
       <c r="E925" s="7">
-        <v>0</v>
+        <v>-0.00295</v>
       </c>
       <c r="F925" s="7">
-        <v>0</v>
+        <v>-0.01213</v>
       </c>
       <c r="G925" s="7">
-        <v>0</v>
+        <v>-0.070884</v>
       </c>
       <c r="H925" s="7">
-        <v>0</v>
+        <v>0.03764</v>
       </c>
       <c r="I925" s="7">
-        <v>0</v>
+        <v>0.327538</v>
       </c>
       <c r="J925" s="7">
-        <v>0</v>
+        <v>1.7292679999999998</v>
       </c>
       <c r="K925" s="7">
-        <v>0</v>
+        <v>6.066307</v>
       </c>
     </row>
     <row r="926" spans="1:11" x14ac:dyDescent="0.25">
@@ -36890,22 +36890,22 @@
         <v>5</v>
       </c>
       <c r="E941" s="7">
-        <v>0.032751</v>
+        <v>0.031045</v>
       </c>
       <c r="F941" s="7">
-        <v>0.107683</v>
+        <v>0.105853</v>
       </c>
       <c r="G941" s="7">
-        <v>0.24668900000000002</v>
+        <v>0.24463000000000001</v>
       </c>
       <c r="H941" s="7">
-        <v>0.339991</v>
+        <v>0.33777799999999997</v>
       </c>
       <c r="I941" s="7">
-        <v>0.517802</v>
+        <v>0.515295</v>
       </c>
       <c r="J941" s="7">
-        <v>1.8214650000000001</v>
+        <v>1.816805</v>
       </c>
       <c r="K941" s="7"/>
     </row>
@@ -37807,25 +37807,25 @@
         <v>5</v>
       </c>
       <c r="E972" s="7">
-        <v>0</v>
+        <v>0.008228</v>
       </c>
       <c r="F972" s="7">
-        <v>0</v>
+        <v>0.03891</v>
       </c>
       <c r="G972" s="7">
-        <v>0</v>
+        <v>0.097545</v>
       </c>
       <c r="H972" s="7">
-        <v>0</v>
+        <v>0.18296099999999998</v>
       </c>
       <c r="I972" s="7">
-        <v>0</v>
+        <v>0.295056</v>
       </c>
       <c r="J972" s="7">
-        <v>0</v>
+        <v>1.40602</v>
       </c>
       <c r="K972" s="7">
-        <v>0</v>
+        <v>5.890713</v>
       </c>
     </row>
     <row r="973" spans="1:11" x14ac:dyDescent="0.25">
@@ -37904,25 +37904,25 @@
         <v>4</v>
       </c>
       <c r="E975" s="7">
-        <v>0</v>
+        <v>0.028974000000000003</v>
       </c>
       <c r="F975" s="7">
-        <v>0</v>
+        <v>0.083669</v>
       </c>
       <c r="G975" s="7">
-        <v>0</v>
+        <v>0.169928</v>
       </c>
       <c r="H975" s="7">
-        <v>0</v>
+        <v>0.248035</v>
       </c>
       <c r="I975" s="7">
-        <v>0</v>
+        <v>0.359933</v>
       </c>
       <c r="J975" s="7">
-        <v>0</v>
+        <v>1.2704900000000001</v>
       </c>
       <c r="K975" s="7">
-        <v>0</v>
+        <v>4.900521</v>
       </c>
     </row>
     <row r="976" spans="1:11" x14ac:dyDescent="0.25">
@@ -38205,22 +38205,22 @@
         <v>2</v>
       </c>
       <c r="E984" s="7">
-        <v>0</v>
+        <v>0.024338000000000002</v>
       </c>
       <c r="F984" s="7">
-        <v>0</v>
+        <v>0.08373100000000001</v>
       </c>
       <c r="G984" s="7">
-        <v>0</v>
+        <v>0.182711</v>
       </c>
       <c r="H984" s="7">
-        <v>0</v>
+        <v>0.279905</v>
       </c>
       <c r="I984" s="7">
-        <v>0</v>
+        <v>0.418063</v>
       </c>
       <c r="J984" s="7">
-        <v>0</v>
+        <v>1.801012</v>
       </c>
       <c r="K984" s="7"/>
     </row>
@@ -38737,22 +38737,22 @@
         <v>5</v>
       </c>
       <c r="E1000" s="7">
-        <v>0</v>
+        <v>-0.056928</v>
       </c>
       <c r="F1000" s="7">
-        <v>0</v>
+        <v>-0.04848499999999999</v>
       </c>
       <c r="G1000" s="7">
-        <v>0</v>
+        <v>0.34283499999999995</v>
       </c>
       <c r="H1000" s="7">
-        <v>0</v>
+        <v>0.435715</v>
       </c>
       <c r="I1000" s="7">
-        <v>0</v>
+        <v>0.610191</v>
       </c>
       <c r="J1000" s="7">
-        <v>0</v>
+        <v>2.2532490000000003</v>
       </c>
       <c r="K1000" s="7"/>
     </row>
@@ -39360,25 +39360,25 @@
         <v>5</v>
       </c>
       <c r="E1019" s="7">
-        <v>0</v>
+        <v>0.002559</v>
       </c>
       <c r="F1019" s="7">
-        <v>0</v>
+        <v>0.021568</v>
       </c>
       <c r="G1019" s="7">
-        <v>0</v>
+        <v>0.08109999999999999</v>
       </c>
       <c r="H1019" s="7">
-        <v>0</v>
+        <v>0.177004</v>
       </c>
       <c r="I1019" s="7">
-        <v>0</v>
+        <v>0.210788</v>
       </c>
       <c r="J1019" s="7">
-        <v>0</v>
+        <v>1.091612</v>
       </c>
       <c r="K1019" s="7">
-        <v>0</v>
+        <v>4.577297</v>
       </c>
     </row>
     <row r="1020" spans="1:11" x14ac:dyDescent="0.25">
@@ -39542,25 +39542,25 @@
         <v>6</v>
       </c>
       <c r="E1025" s="7">
-        <v>0</v>
+        <v>-0.032023</v>
       </c>
       <c r="F1025" s="7">
-        <v>0</v>
+        <v>-0.017807</v>
       </c>
       <c r="G1025" s="7">
-        <v>0</v>
+        <v>0.234899</v>
       </c>
       <c r="H1025" s="7">
-        <v>0</v>
+        <v>0.19411899999999999</v>
       </c>
       <c r="I1025" s="7">
-        <v>0</v>
+        <v>0.34863999999999995</v>
       </c>
       <c r="J1025" s="7">
-        <v>0</v>
+        <v>2.021085</v>
       </c>
       <c r="K1025" s="7">
-        <v>0</v>
+        <v>8.217224</v>
       </c>
     </row>
     <row r="1026" spans="1:11" x14ac:dyDescent="0.25">
@@ -39829,25 +39829,25 @@
         <v>7</v>
       </c>
       <c r="E1034" s="7">
-        <v>0</v>
+        <v>-0.013456</v>
       </c>
       <c r="F1034" s="7">
-        <v>0</v>
+        <v>-0.06983</v>
       </c>
       <c r="G1034" s="7">
-        <v>0</v>
+        <v>-0.17445799999999997</v>
       </c>
       <c r="H1034" s="7">
-        <v>0</v>
+        <v>-0.038873000000000005</v>
       </c>
       <c r="I1034" s="7">
-        <v>0</v>
+        <v>0.669873</v>
       </c>
       <c r="J1034" s="7">
-        <v>0</v>
+        <v>3.480153</v>
       </c>
       <c r="K1034" s="7">
-        <v>0</v>
+        <v>11.525682999999999</v>
       </c>
     </row>
     <row r="1035" spans="1:11" x14ac:dyDescent="0.25">
@@ -40153,22 +40153,22 @@
         <v>6</v>
       </c>
       <c r="E1044" s="7">
-        <v>0.036782</v>
+        <v>0.035011</v>
       </c>
       <c r="F1044" s="7">
-        <v>0.07569</v>
+        <v>0.073852</v>
       </c>
       <c r="G1044" s="7">
-        <v>0.093109</v>
+        <v>0.091242</v>
       </c>
       <c r="H1044" s="7">
-        <v>0.250344</v>
+        <v>0.24820799999999998</v>
       </c>
       <c r="I1044" s="7">
-        <v>0.439598</v>
+        <v>0.437139</v>
       </c>
       <c r="J1044" s="7">
-        <v>1.7307560000000002</v>
+        <v>1.726091</v>
       </c>
       <c r="K1044" s="7"/>
     </row>
@@ -40716,25 +40716,25 @@
         <v>5</v>
       </c>
       <c r="E1061" s="7">
-        <v>0.014397</v>
+        <v>0.014308000000000001</v>
       </c>
       <c r="F1061" s="7">
-        <v>0.014372000000000001</v>
+        <v>0.014282999999999999</v>
       </c>
       <c r="G1061" s="7">
-        <v>0.093622</v>
+        <v>0.093525</v>
       </c>
       <c r="H1061" s="7">
-        <v>0.151447</v>
+        <v>0.151346</v>
       </c>
       <c r="I1061" s="7">
-        <v>0.19872800000000002</v>
+        <v>0.19862300000000002</v>
       </c>
       <c r="J1061" s="7">
-        <v>1.199126</v>
+        <v>1.198933</v>
       </c>
       <c r="K1061" s="7">
-        <v>7.0911919999999995</v>
+        <v>7.09048</v>
       </c>
     </row>
     <row r="1062" spans="1:11" x14ac:dyDescent="0.25">
@@ -40941,22 +40941,22 @@
         <v>6</v>
       </c>
       <c r="E1068" s="7">
-        <v>0.004599</v>
+        <v>0.00091</v>
       </c>
       <c r="F1068" s="7">
-        <v>-0.0016359999999999999</v>
+        <v>-0.005302</v>
       </c>
       <c r="G1068" s="7">
-        <v>0.149406</v>
+        <v>0.14518599999999998</v>
       </c>
       <c r="H1068" s="7">
-        <v>0.25153</v>
+        <v>0.24693400000000001</v>
       </c>
       <c r="I1068" s="7">
-        <v>0.350319</v>
+        <v>0.345361</v>
       </c>
       <c r="J1068" s="7">
-        <v>1.3890149999999999</v>
+        <v>1.380243</v>
       </c>
       <c r="K1068" s="7"/>
     </row>
@@ -40974,19 +40974,19 @@
         <v>5</v>
       </c>
       <c r="E1069" s="7">
-        <v>0.04605000000000001</v>
+        <v>0.042255</v>
       </c>
       <c r="F1069" s="7">
-        <v>0.146927</v>
+        <v>0.142767</v>
       </c>
       <c r="G1069" s="7">
-        <v>0.193693</v>
+        <v>0.189363</v>
       </c>
       <c r="H1069" s="7">
-        <v>0.287261</v>
+        <v>0.282592</v>
       </c>
       <c r="I1069" s="7">
-        <v>0.312417</v>
+        <v>0.307657</v>
       </c>
       <c r="J1069" s="7"/>
       <c r="K1069" s="7"/>

</xml_diff>

<commit_message>
Site guncellemesi - 17.09.2026 11:26
</commit_message>
<xml_diff>
--- a/app/fonlar/getiri/menkul-kiymet-yatirim-fonlari/data/menkul-kiymet-yatirim-fonlari-getiri.xlsx
+++ b/app/fonlar/getiri/menkul-kiymet-yatirim-fonlari/data/menkul-kiymet-yatirim-fonlari-getiri.xlsx
@@ -19,7 +19,7 @@
     <t>Dışa Aktarım Tarihi:</t>
   </si>
   <si>
-    <t>17.09.2026 10:05:35</t>
+    <t>17.09.2026 10:21:07</t>
   </si>
   <si>
     <t>Toplam Kayıt Sayısı:</t>
@@ -7287,7 +7287,7 @@
         <v>1.6490129999999998</v>
       </c>
       <c r="K14" s="7">
-        <v>11.791252</v>
+        <v>11.79125</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -11463,22 +11463,22 @@
         <v>7</v>
       </c>
       <c r="E146" s="7">
-        <v>0</v>
+        <v>0.118986</v>
       </c>
       <c r="F146" s="7">
-        <v>0</v>
+        <v>0.463362</v>
       </c>
       <c r="G146" s="7">
-        <v>0</v>
+        <v>0.832381</v>
       </c>
       <c r="H146" s="7">
-        <v>0</v>
+        <v>1.260772</v>
       </c>
       <c r="I146" s="7">
-        <v>0</v>
+        <v>5.4226</v>
       </c>
       <c r="J146" s="7">
-        <v>0</v>
+        <v>23.397871</v>
       </c>
       <c r="K146" s="7"/>
     </row>
@@ -12089,19 +12089,19 @@
         <v>6</v>
       </c>
       <c r="E166" s="7">
-        <v>-0.069521</v>
+        <v>-0.069519</v>
       </c>
       <c r="F166" s="7">
-        <v>-0.067827</v>
+        <v>-0.067826</v>
       </c>
       <c r="G166" s="7">
-        <v>-0.05404899999999999</v>
+        <v>-0.054047</v>
       </c>
       <c r="H166" s="7">
-        <v>0.155214</v>
+        <v>0.155216</v>
       </c>
       <c r="I166" s="7">
-        <v>0.277839</v>
+        <v>0.277841</v>
       </c>
       <c r="J166" s="7"/>
       <c r="K166" s="7"/>
@@ -14236,25 +14236,25 @@
         <v>4</v>
       </c>
       <c r="E235" s="7">
-        <v>0.015621000000000001</v>
+        <v>0.007466</v>
       </c>
       <c r="F235" s="7">
-        <v>0.041985</v>
+        <v>0.033618</v>
       </c>
       <c r="G235" s="7">
-        <v>0.080659</v>
+        <v>0.071982</v>
       </c>
       <c r="H235" s="7">
-        <v>0.16375399999999998</v>
+        <v>0.15441000000000002</v>
       </c>
       <c r="I235" s="7">
-        <v>0.35545499999999997</v>
+        <v>0.34457099999999996</v>
       </c>
       <c r="J235" s="7">
-        <v>1.9260570000000001</v>
+        <v>1.902563</v>
       </c>
       <c r="K235" s="7">
-        <v>5.736673</v>
+        <v>5.682582</v>
       </c>
     </row>
     <row r="236" spans="1:11" x14ac:dyDescent="0.25">
@@ -14964,25 +14964,25 @@
       </c>
       <c r="D257" s="6"/>
       <c r="E257" s="7">
-        <v>0.021091000000000002</v>
+        <v>0.020939</v>
       </c>
       <c r="F257" s="7">
-        <v>0.060445</v>
+        <v>0.060287</v>
       </c>
       <c r="G257" s="7">
-        <v>0.12061899999999999</v>
+        <v>0.12045299999999999</v>
       </c>
       <c r="H257" s="7">
-        <v>0.16194</v>
+        <v>0.161768</v>
       </c>
       <c r="I257" s="7">
-        <v>0.22053899999999999</v>
+        <v>0.220357</v>
       </c>
       <c r="J257" s="7">
-        <v>1.049633</v>
+        <v>1.049328</v>
       </c>
       <c r="K257" s="7">
-        <v>5.831192</v>
+        <v>5.830176</v>
       </c>
     </row>
     <row r="258" spans="1:11" x14ac:dyDescent="0.25">
@@ -16434,25 +16434,25 @@
         <v>6</v>
       </c>
       <c r="E301" s="7">
-        <v>-0.042962999999999994</v>
+        <v>-0.042962</v>
       </c>
       <c r="F301" s="7">
-        <v>-0.027659</v>
+        <v>-0.027658000000000002</v>
       </c>
       <c r="G301" s="7">
-        <v>0.070826</v>
+        <v>0.070827</v>
       </c>
       <c r="H301" s="7">
         <v>0.196904</v>
       </c>
       <c r="I301" s="7">
-        <v>0.309077</v>
+        <v>0.309078</v>
       </c>
       <c r="J301" s="7">
-        <v>1.274197</v>
+        <v>1.274199</v>
       </c>
       <c r="K301" s="7">
-        <v>12.735626</v>
+        <v>12.735636</v>
       </c>
     </row>
     <row r="302" spans="1:11" x14ac:dyDescent="0.25">
@@ -18673,22 +18673,22 @@
       </c>
       <c r="D370" s="6"/>
       <c r="E370" s="7">
-        <v>0</v>
+        <v>0.004112</v>
       </c>
       <c r="F370" s="7">
-        <v>0</v>
+        <v>0.032078</v>
       </c>
       <c r="G370" s="7">
-        <v>0</v>
+        <v>0.122398</v>
       </c>
       <c r="H370" s="7">
-        <v>0</v>
+        <v>0.21668700000000002</v>
       </c>
       <c r="I370" s="7">
-        <v>0</v>
+        <v>0.281155</v>
       </c>
       <c r="J370" s="7">
-        <v>0</v>
+        <v>1.5306870000000001</v>
       </c>
       <c r="K370" s="7"/>
     </row>
@@ -19250,19 +19250,19 @@
         <v>6</v>
       </c>
       <c r="E389" s="7">
-        <v>-0.030061</v>
+        <v>-0.027886</v>
       </c>
       <c r="F389" s="7">
-        <v>0.019686</v>
+        <v>0.021972000000000002</v>
       </c>
       <c r="G389" s="7">
-        <v>0.111078</v>
+        <v>0.11356899999999999</v>
       </c>
       <c r="H389" s="7">
-        <v>0.200133</v>
+        <v>0.20282499999999998</v>
       </c>
       <c r="I389" s="7">
-        <v>0.270368</v>
+        <v>0.273217</v>
       </c>
       <c r="J389" s="7"/>
       <c r="K389" s="7"/>
@@ -19564,25 +19564,25 @@
       </c>
       <c r="D399" s="6"/>
       <c r="E399" s="7">
-        <v>-0.00607</v>
+        <v>-0.006102</v>
       </c>
       <c r="F399" s="7">
-        <v>0.026184</v>
+        <v>0.026151</v>
       </c>
       <c r="G399" s="7">
-        <v>0.189164</v>
+        <v>0.18912500000000002</v>
       </c>
       <c r="H399" s="7">
-        <v>0.229246</v>
+        <v>0.229206</v>
       </c>
       <c r="I399" s="7">
-        <v>0.308019</v>
+        <v>0.307977</v>
       </c>
       <c r="J399" s="7">
-        <v>1.536249</v>
+        <v>1.5361660000000001</v>
       </c>
       <c r="K399" s="7">
-        <v>6.4670060000000005</v>
+        <v>6.466762</v>
       </c>
     </row>
     <row r="400" spans="1:11" x14ac:dyDescent="0.25">
@@ -19950,10 +19950,10 @@
         <v>6</v>
       </c>
       <c r="E411" s="7">
-        <v>-0.103535</v>
+        <v>-0.106822</v>
       </c>
       <c r="F411" s="7">
-        <v>-0.03058</v>
+        <v>-0.034135</v>
       </c>
       <c r="G411" s="7"/>
       <c r="H411" s="7"/>
@@ -20297,19 +20297,19 @@
         <v>5</v>
       </c>
       <c r="E422" s="7">
-        <v>-0.028127</v>
+        <v>-0.028130000000000002</v>
       </c>
       <c r="F422" s="7">
-        <v>0.013388</v>
+        <v>0.013384</v>
       </c>
       <c r="G422" s="7">
-        <v>0.129524</v>
+        <v>0.129521</v>
       </c>
       <c r="H422" s="7">
-        <v>0.468198</v>
+        <v>0.46819299999999997</v>
       </c>
       <c r="I422" s="7">
-        <v>0.42545099999999997</v>
+        <v>0.42544699999999996</v>
       </c>
       <c r="J422" s="7"/>
       <c r="K422" s="7"/>
@@ -20889,25 +20889,25 @@
       </c>
       <c r="D440" s="6"/>
       <c r="E440" s="7">
-        <v>0</v>
+        <v>0.015024</v>
       </c>
       <c r="F440" s="7">
-        <v>0</v>
+        <v>0.058993000000000004</v>
       </c>
       <c r="G440" s="7">
-        <v>0</v>
+        <v>0.124774</v>
       </c>
       <c r="H440" s="7">
-        <v>0</v>
+        <v>0.15967399999999998</v>
       </c>
       <c r="I440" s="7">
-        <v>0</v>
+        <v>0.23738499999999998</v>
       </c>
       <c r="J440" s="7">
-        <v>0</v>
+        <v>1.260678</v>
       </c>
       <c r="K440" s="7">
-        <v>0</v>
+        <v>6.76764</v>
       </c>
     </row>
     <row r="441" spans="1:11" x14ac:dyDescent="0.25">
@@ -21397,19 +21397,19 @@
         <v>6</v>
       </c>
       <c r="E456" s="7">
-        <v>-0.152279</v>
+        <v>-0.152294</v>
       </c>
       <c r="F456" s="7">
-        <v>-0.126604</v>
+        <v>-0.12661899999999998</v>
       </c>
       <c r="G456" s="7">
-        <v>-0.006836999999999999</v>
+        <v>-0.006854</v>
       </c>
       <c r="H456" s="7">
-        <v>0.12152400000000001</v>
+        <v>0.12150499999999999</v>
       </c>
       <c r="I456" s="7">
-        <v>0.09003</v>
+        <v>0.09001200000000001</v>
       </c>
       <c r="J456" s="7"/>
       <c r="K456" s="7"/>
@@ -21760,22 +21760,22 @@
         <v>7</v>
       </c>
       <c r="E467" s="7">
-        <v>-0.074325</v>
+        <v>-0.074328</v>
       </c>
       <c r="F467" s="7">
-        <v>-0.047857000000000004</v>
+        <v>-0.047861</v>
       </c>
       <c r="G467" s="7">
-        <v>0.385471</v>
+        <v>0.385465</v>
       </c>
       <c r="H467" s="7">
-        <v>0.426709</v>
+        <v>0.426703</v>
       </c>
       <c r="I467" s="7">
-        <v>0.66769</v>
+        <v>0.6676829999999999</v>
       </c>
       <c r="J467" s="7">
-        <v>2.104098</v>
+        <v>2.104085</v>
       </c>
       <c r="K467" s="7"/>
     </row>
@@ -21863,25 +21863,25 @@
         <v>1</v>
       </c>
       <c r="E470" s="7">
-        <v>0.03339</v>
+        <v>0.033396</v>
       </c>
       <c r="F470" s="7">
-        <v>0.103422</v>
+        <v>0.10342900000000001</v>
       </c>
       <c r="G470" s="7">
-        <v>0.21604800000000002</v>
+        <v>0.216055</v>
       </c>
       <c r="H470" s="7">
-        <v>0.31149899999999997</v>
+        <v>0.311507</v>
       </c>
       <c r="I470" s="7">
-        <v>0.47323</v>
+        <v>0.473239</v>
       </c>
       <c r="J470" s="7">
-        <v>2.643686</v>
+        <v>2.6437079999999997</v>
       </c>
       <c r="K470" s="7">
-        <v>4.4795620000000005</v>
+        <v>4.479595</v>
       </c>
     </row>
     <row r="471" spans="1:11" x14ac:dyDescent="0.25">
@@ -21968,25 +21968,25 @@
         <v>6</v>
       </c>
       <c r="E473" s="7">
-        <v>-0.033974000000000004</v>
+        <v>-0.033933</v>
       </c>
       <c r="F473" s="7">
-        <v>-0.035594</v>
+        <v>-0.035553</v>
       </c>
       <c r="G473" s="7">
-        <v>0.13627599999999998</v>
+        <v>0.136325</v>
       </c>
       <c r="H473" s="7">
-        <v>0.305093</v>
+        <v>0.30514800000000003</v>
       </c>
       <c r="I473" s="7">
-        <v>0.45781700000000003</v>
+        <v>0.45787799999999995</v>
       </c>
       <c r="J473" s="7">
-        <v>1.9944909999999998</v>
+        <v>1.994618</v>
       </c>
       <c r="K473" s="7">
-        <v>6.918654</v>
+        <v>6.91899</v>
       </c>
     </row>
     <row r="474" spans="1:11" x14ac:dyDescent="0.25">
@@ -22529,22 +22529,22 @@
         <v>3</v>
       </c>
       <c r="E490" s="7">
-        <v>0.037586</v>
+        <v>0.037592</v>
       </c>
       <c r="F490" s="7">
-        <v>0.113691</v>
+        <v>0.113698</v>
       </c>
       <c r="G490" s="7">
-        <v>0.19375499999999998</v>
+        <v>0.19376300000000002</v>
       </c>
       <c r="H490" s="7">
-        <v>0.275096</v>
+        <v>0.275104</v>
       </c>
       <c r="I490" s="7">
-        <v>0.402958</v>
+        <v>0.402967</v>
       </c>
       <c r="J490" s="7">
-        <v>2.0356739999999998</v>
+        <v>2.035693</v>
       </c>
       <c r="K490" s="7"/>
     </row>
@@ -22948,22 +22948,22 @@
         <v>5</v>
       </c>
       <c r="E503" s="7">
-        <v>0.025977</v>
+        <v>0.026442999999999998</v>
       </c>
       <c r="F503" s="7">
-        <v>0.109232</v>
+        <v>0.109735</v>
       </c>
       <c r="G503" s="7">
-        <v>0.349037</v>
+        <v>0.349649</v>
       </c>
       <c r="H503" s="7">
-        <v>0.43306199999999995</v>
+        <v>0.43371200000000004</v>
       </c>
       <c r="I503" s="7">
-        <v>0.5380590000000001</v>
+        <v>0.538756</v>
       </c>
       <c r="J503" s="7">
-        <v>1.7173679999999998</v>
+        <v>1.7186009999999998</v>
       </c>
       <c r="K503" s="7"/>
     </row>
@@ -22981,25 +22981,25 @@
         <v>7</v>
       </c>
       <c r="E504" s="7">
-        <v>0.084588</v>
+        <v>0.08458500000000001</v>
       </c>
       <c r="F504" s="7">
-        <v>0.28968499999999997</v>
+        <v>0.289682</v>
       </c>
       <c r="G504" s="7">
-        <v>0.304632</v>
+        <v>0.30462900000000004</v>
       </c>
       <c r="H504" s="7">
-        <v>0.17554999999999998</v>
+        <v>0.175547</v>
       </c>
       <c r="I504" s="7">
-        <v>0.174435</v>
+        <v>0.174432</v>
       </c>
       <c r="J504" s="7">
-        <v>1.4717879999999999</v>
+        <v>1.4717820000000001</v>
       </c>
       <c r="K504" s="7">
-        <v>6.551005</v>
+        <v>6.550987</v>
       </c>
     </row>
     <row r="505" spans="1:11" x14ac:dyDescent="0.25">
@@ -23163,22 +23163,22 @@
         <v>2</v>
       </c>
       <c r="E510" s="7">
-        <v>0.010462</v>
+        <v>0.010428999999999999</v>
       </c>
       <c r="F510" s="7">
-        <v>0.046128999999999996</v>
+        <v>0.046095</v>
       </c>
       <c r="G510" s="7">
-        <v>0.203645</v>
+        <v>0.203606</v>
       </c>
       <c r="H510" s="7">
-        <v>0.340221</v>
+        <v>0.34017699999999995</v>
       </c>
       <c r="I510" s="7">
-        <v>0.49741</v>
+        <v>0.497361</v>
       </c>
       <c r="J510" s="7">
-        <v>2.297962</v>
+        <v>2.297854</v>
       </c>
       <c r="K510" s="7"/>
     </row>
@@ -23983,19 +23983,19 @@
         <v>6</v>
       </c>
       <c r="E536" s="7">
-        <v>0.005447</v>
+        <v>0.005506</v>
       </c>
       <c r="F536" s="7">
-        <v>0.029405</v>
+        <v>0.029464999999999998</v>
       </c>
       <c r="G536" s="7">
-        <v>-0.04762400000000001</v>
+        <v>-0.047568</v>
       </c>
       <c r="H536" s="7">
-        <v>0.115898</v>
+        <v>0.115964</v>
       </c>
       <c r="I536" s="7">
-        <v>0.345672</v>
+        <v>0.345751</v>
       </c>
       <c r="J536" s="7"/>
       <c r="K536" s="7"/>
@@ -24640,19 +24640,19 @@
         <v>2</v>
       </c>
       <c r="E557" s="7">
-        <v>0.03195</v>
+        <v>0.03199</v>
       </c>
       <c r="F557" s="7">
-        <v>0.10192</v>
+        <v>0.101962</v>
       </c>
       <c r="G557" s="7">
-        <v>0.215303</v>
+        <v>0.215349</v>
       </c>
       <c r="H557" s="7">
-        <v>0.309985</v>
+        <v>0.310035</v>
       </c>
       <c r="I557" s="7">
-        <v>0.463218</v>
+        <v>0.46327399999999996</v>
       </c>
       <c r="J557" s="7"/>
       <c r="K557" s="7"/>
@@ -25253,22 +25253,22 @@
         <v>2</v>
       </c>
       <c r="E576" s="7">
-        <v>0.033714</v>
+        <v>0.033733</v>
       </c>
       <c r="F576" s="7">
-        <v>0.107015</v>
+        <v>0.107035</v>
       </c>
       <c r="G576" s="7">
-        <v>0.22608</v>
+        <v>0.226103</v>
       </c>
       <c r="H576" s="7">
-        <v>0.32480800000000004</v>
+        <v>0.324833</v>
       </c>
       <c r="I576" s="7">
-        <v>0.489907</v>
+        <v>0.48993400000000004</v>
       </c>
       <c r="J576" s="7">
-        <v>2.526227</v>
+        <v>2.526293</v>
       </c>
       <c r="K576" s="7"/>
     </row>
@@ -27035,19 +27035,19 @@
         <v>2</v>
       </c>
       <c r="E632" s="7">
-        <v>0</v>
+        <v>0.031934</v>
       </c>
       <c r="F632" s="7">
-        <v>0</v>
+        <v>0.10345399999999999</v>
       </c>
       <c r="G632" s="7">
-        <v>0</v>
+        <v>0.22684300000000002</v>
       </c>
       <c r="H632" s="7">
-        <v>0</v>
+        <v>0.341056</v>
       </c>
       <c r="I632" s="7">
-        <v>0</v>
+        <v>0.535728</v>
       </c>
       <c r="J632" s="7"/>
       <c r="K632" s="7"/>
@@ -28889,25 +28889,25 @@
         <v>6</v>
       </c>
       <c r="E690" s="7">
-        <v>-0.033599000000000004</v>
+        <v>-0.035837</v>
       </c>
       <c r="F690" s="7">
-        <v>-0.013040000000000001</v>
+        <v>-0.015325</v>
       </c>
       <c r="G690" s="7">
-        <v>0.353694</v>
+        <v>0.350559</v>
       </c>
       <c r="H690" s="7">
-        <v>0.39128599999999997</v>
+        <v>0.38806399999999996</v>
       </c>
       <c r="I690" s="7">
-        <v>0.48885</v>
+        <v>0.48540300000000003</v>
       </c>
       <c r="J690" s="7">
-        <v>2.6117899999999996</v>
+        <v>2.6034260000000002</v>
       </c>
       <c r="K690" s="7">
-        <v>10.403127999999999</v>
+        <v>10.376723</v>
       </c>
     </row>
     <row r="691" spans="1:11" x14ac:dyDescent="0.25">
@@ -29743,22 +29743,22 @@
         <v>6</v>
       </c>
       <c r="E716" s="7">
-        <v>0.082138</v>
+        <v>0.082558</v>
       </c>
       <c r="F716" s="7">
-        <v>0.168117</v>
+        <v>0.168569</v>
       </c>
       <c r="G716" s="7">
-        <v>0.16325099999999998</v>
+        <v>0.16370200000000001</v>
       </c>
       <c r="H716" s="7">
-        <v>0.39696</v>
+        <v>0.397502</v>
       </c>
       <c r="I716" s="7">
-        <v>0.5923940000000001</v>
+        <v>0.593011</v>
       </c>
       <c r="J716" s="7">
-        <v>1.629205</v>
+        <v>1.6302240000000001</v>
       </c>
       <c r="K716" s="7"/>
     </row>
@@ -30214,19 +30214,19 @@
         <v>4</v>
       </c>
       <c r="E731" s="7">
-        <v>0.039671</v>
+        <v>0.024792</v>
       </c>
       <c r="F731" s="7">
-        <v>0.063025</v>
+        <v>0.047813</v>
       </c>
       <c r="G731" s="7">
-        <v>0.083314</v>
+        <v>0.06781100000000001</v>
       </c>
       <c r="H731" s="7">
-        <v>0.210791</v>
+        <v>0.193464</v>
       </c>
       <c r="I731" s="7">
-        <v>0.32449300000000003</v>
+        <v>0.305538</v>
       </c>
       <c r="J731" s="7"/>
       <c r="K731" s="7"/>
@@ -30309,19 +30309,19 @@
         <v>6</v>
       </c>
       <c r="E734" s="7">
-        <v>-0.049525</v>
+        <v>-0.050174</v>
       </c>
       <c r="F734" s="7">
-        <v>-0.104938</v>
+        <v>-0.105549</v>
       </c>
       <c r="G734" s="7">
-        <v>0.044538</v>
+        <v>0.043825</v>
       </c>
       <c r="H734" s="7">
-        <v>0.13661500000000001</v>
+        <v>0.135839</v>
       </c>
       <c r="I734" s="7">
-        <v>0.09920899999999999</v>
+        <v>0.098459</v>
       </c>
       <c r="J734" s="7"/>
       <c r="K734" s="7"/>
@@ -30431,7 +30431,7 @@
         <v>6</v>
       </c>
       <c r="E738" s="7">
-        <v>-0.026358000000000003</v>
+        <v>-0.026359</v>
       </c>
       <c r="F738" s="7">
         <v>-0.044236000000000004</v>
@@ -30440,10 +30440,10 @@
         <v>0.12313800000000001</v>
       </c>
       <c r="H738" s="7">
-        <v>0.311885</v>
+        <v>0.311884</v>
       </c>
       <c r="I738" s="7">
-        <v>0.25125800000000004</v>
+        <v>0.251257</v>
       </c>
       <c r="J738" s="7"/>
       <c r="K738" s="7"/>
@@ -31442,22 +31442,22 @@
         <v>7</v>
       </c>
       <c r="E771" s="7">
-        <v>0.295788</v>
+        <v>0.295787</v>
       </c>
       <c r="F771" s="7">
-        <v>0.39861199999999997</v>
+        <v>0.398611</v>
       </c>
       <c r="G771" s="7">
-        <v>-0.074325</v>
+        <v>-0.074326</v>
       </c>
       <c r="H771" s="7">
-        <v>0.13637</v>
+        <v>0.13636900000000002</v>
       </c>
       <c r="I771" s="7">
-        <v>0.34647300000000003</v>
+        <v>0.346472</v>
       </c>
       <c r="J771" s="7">
-        <v>2.233235</v>
+        <v>2.233233</v>
       </c>
       <c r="K771" s="7"/>
     </row>
@@ -33155,19 +33155,19 @@
         <v>7</v>
       </c>
       <c r="E826" s="7">
-        <v>0</v>
+        <v>-0.037290000000000004</v>
       </c>
       <c r="F826" s="7">
-        <v>0</v>
+        <v>-0.14177</v>
       </c>
       <c r="G826" s="7">
-        <v>0</v>
+        <v>0.025736</v>
       </c>
       <c r="H826" s="7">
-        <v>0</v>
+        <v>0.132304</v>
       </c>
       <c r="I826" s="7">
-        <v>0</v>
+        <v>0.741221</v>
       </c>
       <c r="J826" s="7"/>
       <c r="K826" s="7"/>
@@ -34457,19 +34457,19 @@
         <v>5</v>
       </c>
       <c r="E868" s="7">
-        <v>0.011720999999999999</v>
+        <v>0.011562</v>
       </c>
       <c r="F868" s="7">
-        <v>0.127958</v>
+        <v>0.127781</v>
       </c>
       <c r="G868" s="7">
-        <v>0.213646</v>
+        <v>0.213456</v>
       </c>
       <c r="H868" s="7">
-        <v>0.23613800000000001</v>
+        <v>0.23594400000000001</v>
       </c>
       <c r="I868" s="7">
-        <v>0.419619</v>
+        <v>0.419396</v>
       </c>
       <c r="J868" s="7"/>
       <c r="K868" s="7"/>
@@ -36230,19 +36230,19 @@
         <v>5</v>
       </c>
       <c r="E921" s="7">
-        <v>0.014711</v>
+        <v>0.014716</v>
       </c>
       <c r="F921" s="7">
-        <v>0.062566</v>
+        <v>0.062572</v>
       </c>
       <c r="G921" s="7">
-        <v>0.150802</v>
+        <v>0.150809</v>
       </c>
       <c r="H921" s="7">
-        <v>0.22830899999999998</v>
+        <v>0.22831600000000002</v>
       </c>
       <c r="I921" s="7">
-        <v>0.287613</v>
+        <v>0.28762</v>
       </c>
       <c r="J921" s="7"/>
       <c r="K921" s="7"/>
@@ -36758,25 +36758,25 @@
         <v>7</v>
       </c>
       <c r="E937" s="7">
-        <v>-0.032639</v>
+        <v>-0.032615</v>
       </c>
       <c r="F937" s="7">
-        <v>-0.0537</v>
+        <v>-0.053676</v>
       </c>
       <c r="G937" s="7">
-        <v>0.129491</v>
+        <v>0.129519</v>
       </c>
       <c r="H937" s="7">
-        <v>0.245658</v>
+        <v>0.245689</v>
       </c>
       <c r="I937" s="7">
-        <v>0.265025</v>
+        <v>0.265056</v>
       </c>
       <c r="J937" s="7">
-        <v>3.2069650000000003</v>
+        <v>3.207069</v>
       </c>
       <c r="K937" s="7">
-        <v>17.631603</v>
+        <v>17.632064</v>
       </c>
     </row>
     <row r="938" spans="1:11" x14ac:dyDescent="0.25">
@@ -39959,25 +39959,25 @@
         <v>6</v>
       </c>
       <c r="E1038" s="7">
-        <v>-0.012056</v>
+        <v>-0.011861</v>
       </c>
       <c r="F1038" s="7">
-        <v>-0.024535</v>
+        <v>-0.024343</v>
       </c>
       <c r="G1038" s="7">
-        <v>0.077459</v>
+        <v>0.077671</v>
       </c>
       <c r="H1038" s="7">
-        <v>0.126358</v>
+        <v>0.12658</v>
       </c>
       <c r="I1038" s="7">
-        <v>0.19103799999999999</v>
+        <v>0.19127300000000003</v>
       </c>
       <c r="J1038" s="7">
-        <v>1.024308</v>
+        <v>1.024708</v>
       </c>
       <c r="K1038" s="7">
-        <v>5.135193</v>
+        <v>5.1364030000000005</v>
       </c>
     </row>
     <row r="1039" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Site guncellemesi - 01.10.2026 10:33
</commit_message>
<xml_diff>
--- a/app/fonlar/getiri/menkul-kiymet-yatirim-fonlari/data/menkul-kiymet-yatirim-fonlari-getiri.xlsx
+++ b/app/fonlar/getiri/menkul-kiymet-yatirim-fonlari/data/menkul-kiymet-yatirim-fonlari-getiri.xlsx
@@ -19,7 +19,7 @@
     <t>Dışa Aktarım Tarihi:</t>
   </si>
   <si>
-    <t>01.10.2026 08:50:49</t>
+    <t>01.10.2026 10:17:57</t>
   </si>
   <si>
     <t>Toplam Kayıt Sayısı:</t>
@@ -7056,25 +7056,25 @@
         <v>5</v>
       </c>
       <c r="E7" s="7">
-        <v>0.016356</v>
+        <v>0.016348</v>
       </c>
       <c r="F7" s="7">
-        <v>0.090489</v>
+        <v>0.09048199999999999</v>
       </c>
       <c r="G7" s="7">
-        <v>0.28194199999999997</v>
+        <v>0.281932</v>
       </c>
       <c r="H7" s="7">
-        <v>0.256618</v>
+        <v>0.25660900000000003</v>
       </c>
       <c r="I7" s="7">
-        <v>0.35336799999999996</v>
+        <v>0.35335900000000003</v>
       </c>
       <c r="J7" s="7">
-        <v>1.296649</v>
+        <v>1.2966319999999998</v>
       </c>
       <c r="K7" s="7">
-        <v>2.680945</v>
+        <v>2.6809179999999997</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -7192,22 +7192,22 @@
         <v>3</v>
       </c>
       <c r="E11" s="7">
-        <v>0</v>
+        <v>0.034414</v>
       </c>
       <c r="F11" s="7">
-        <v>0</v>
+        <v>0.087742</v>
       </c>
       <c r="G11" s="7">
-        <v>0</v>
+        <v>0.16007200000000002</v>
       </c>
       <c r="H11" s="7">
-        <v>0</v>
+        <v>0.252445</v>
       </c>
       <c r="I11" s="7">
-        <v>0</v>
+        <v>0.35369500000000004</v>
       </c>
       <c r="J11" s="7">
-        <v>0</v>
+        <v>1.704418</v>
       </c>
       <c r="K11" s="7"/>
     </row>
@@ -7258,25 +7258,25 @@
         <v>6</v>
       </c>
       <c r="E13" s="7">
-        <v>0</v>
+        <v>-0.08133800000000001</v>
       </c>
       <c r="F13" s="7">
-        <v>0</v>
+        <v>-0.110687</v>
       </c>
       <c r="G13" s="7">
-        <v>0</v>
+        <v>0.010074000000000001</v>
       </c>
       <c r="H13" s="7">
-        <v>0</v>
+        <v>0.184243</v>
       </c>
       <c r="I13" s="7">
-        <v>0</v>
+        <v>0.22937100000000002</v>
       </c>
       <c r="J13" s="7">
-        <v>0</v>
+        <v>1.087785</v>
       </c>
       <c r="K13" s="7">
-        <v>0</v>
+        <v>13.195473</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -7328,25 +7328,25 @@
         <v>5</v>
       </c>
       <c r="E15" s="7">
-        <v>0</v>
+        <v>0.019938</v>
       </c>
       <c r="F15" s="7">
-        <v>0</v>
+        <v>0.06317</v>
       </c>
       <c r="G15" s="7">
-        <v>0</v>
+        <v>0.128808</v>
       </c>
       <c r="H15" s="7">
-        <v>0</v>
+        <v>0.183718</v>
       </c>
       <c r="I15" s="7">
-        <v>0</v>
+        <v>0.246095</v>
       </c>
       <c r="J15" s="7">
-        <v>0</v>
+        <v>1.136634</v>
       </c>
       <c r="K15" s="7">
-        <v>0</v>
+        <v>4.415723</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -7917,19 +7917,19 @@
         <v>2</v>
       </c>
       <c r="E32" s="7">
-        <v>0</v>
+        <v>0.023813</v>
       </c>
       <c r="F32" s="7">
-        <v>0</v>
+        <v>0.080656</v>
       </c>
       <c r="G32" s="7">
-        <v>0</v>
+        <v>0.168676</v>
       </c>
       <c r="H32" s="7">
-        <v>0</v>
+        <v>0.238141</v>
       </c>
       <c r="I32" s="7">
-        <v>0</v>
+        <v>0.34862000000000004</v>
       </c>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
@@ -8321,19 +8321,19 @@
         <v>3</v>
       </c>
       <c r="E44" s="7">
-        <v>0</v>
+        <v>0.026969</v>
       </c>
       <c r="F44" s="7">
-        <v>0</v>
+        <v>0.09228199999999999</v>
       </c>
       <c r="G44" s="7">
-        <v>0</v>
+        <v>0.223132</v>
       </c>
       <c r="H44" s="7">
-        <v>0</v>
+        <v>0.336253</v>
       </c>
       <c r="I44" s="7">
-        <v>0</v>
+        <v>0.453989</v>
       </c>
       <c r="J44" s="7"/>
       <c r="K44" s="7"/>
@@ -8622,16 +8622,16 @@
         <v>6</v>
       </c>
       <c r="E53" s="7">
-        <v>0</v>
+        <v>-0.044295999999999995</v>
       </c>
       <c r="F53" s="7">
-        <v>0</v>
+        <v>0.096921</v>
       </c>
       <c r="G53" s="7">
-        <v>0</v>
+        <v>0.008075</v>
       </c>
       <c r="H53" s="7">
-        <v>0</v>
+        <v>0.093618</v>
       </c>
       <c r="I53" s="7"/>
       <c r="J53" s="7"/>
@@ -8982,22 +8982,22 @@
         <v>5</v>
       </c>
       <c r="E65" s="7">
-        <v>0</v>
+        <v>-0.009931</v>
       </c>
       <c r="F65" s="7">
-        <v>0</v>
+        <v>0.046954</v>
       </c>
       <c r="G65" s="7">
-        <v>0</v>
+        <v>0.11036</v>
       </c>
       <c r="H65" s="7">
-        <v>0</v>
+        <v>-0.057239000000000005</v>
       </c>
       <c r="I65" s="7">
-        <v>0</v>
+        <v>0.025039</v>
       </c>
       <c r="J65" s="7">
-        <v>0</v>
+        <v>1.975417</v>
       </c>
       <c r="K65" s="7"/>
     </row>
@@ -9838,16 +9838,16 @@
         <v>5</v>
       </c>
       <c r="E93" s="7">
-        <v>0</v>
+        <v>0.010003</v>
       </c>
       <c r="F93" s="7">
-        <v>0</v>
+        <v>0.11838699999999999</v>
       </c>
       <c r="G93" s="7">
-        <v>0</v>
+        <v>0.221365</v>
       </c>
       <c r="H93" s="7">
-        <v>0</v>
+        <v>0.202926</v>
       </c>
       <c r="I93" s="7"/>
       <c r="J93" s="7"/>
@@ -10188,22 +10188,22 @@
         <v>7</v>
       </c>
       <c r="E105" s="7">
-        <v>-0.027957999999999997</v>
+        <v>-0.027969</v>
       </c>
       <c r="F105" s="7">
-        <v>-0.003017</v>
+        <v>-0.0030280000000000003</v>
       </c>
       <c r="G105" s="7">
-        <v>0.053753999999999996</v>
+        <v>0.053742</v>
       </c>
       <c r="H105" s="7">
-        <v>0.170969</v>
+        <v>0.170956</v>
       </c>
       <c r="I105" s="7">
-        <v>0.208232</v>
+        <v>0.208219</v>
       </c>
       <c r="J105" s="7">
-        <v>1.321659</v>
+        <v>1.3216329999999998</v>
       </c>
       <c r="K105" s="7"/>
     </row>
@@ -10439,16 +10439,16 @@
         <v>-0.121952</v>
       </c>
       <c r="F113" s="7">
-        <v>-0.040384</v>
+        <v>-0.040385</v>
       </c>
       <c r="G113" s="7">
-        <v>0.047026000000000005</v>
+        <v>0.047025</v>
       </c>
       <c r="H113" s="7">
-        <v>0.134762</v>
+        <v>0.13476100000000002</v>
       </c>
       <c r="I113" s="7">
-        <v>0.33204999999999996</v>
+        <v>0.33204900000000004</v>
       </c>
       <c r="J113" s="7"/>
       <c r="K113" s="7"/>
@@ -10678,19 +10678,19 @@
         <v>2</v>
       </c>
       <c r="E121" s="7">
-        <v>0</v>
+        <v>0.029977</v>
       </c>
       <c r="F121" s="7">
-        <v>0</v>
+        <v>0.100555</v>
       </c>
       <c r="G121" s="7">
-        <v>0</v>
+        <v>0.21494</v>
       </c>
       <c r="H121" s="7">
-        <v>0</v>
+        <v>0.330276</v>
       </c>
       <c r="I121" s="7">
-        <v>0</v>
+        <v>0.46816</v>
       </c>
       <c r="J121" s="7"/>
       <c r="K121" s="7"/>
@@ -10928,16 +10928,16 @@
         <v>4</v>
       </c>
       <c r="E129" s="7">
-        <v>0</v>
+        <v>-0.03603</v>
       </c>
       <c r="F129" s="7">
-        <v>0</v>
+        <v>0.20071000000000003</v>
       </c>
       <c r="G129" s="7">
-        <v>0</v>
+        <v>0.345503</v>
       </c>
       <c r="H129" s="7">
-        <v>0</v>
+        <v>0.46444899999999995</v>
       </c>
       <c r="I129" s="7"/>
       <c r="J129" s="7"/>
@@ -11046,22 +11046,22 @@
         <v>5</v>
       </c>
       <c r="E133" s="7">
-        <v>0.018964</v>
+        <v>0.018965</v>
       </c>
       <c r="F133" s="7">
-        <v>0.061207000000000004</v>
+        <v>0.061208</v>
       </c>
       <c r="G133" s="7">
-        <v>0.12382699999999999</v>
+        <v>0.123828</v>
       </c>
       <c r="H133" s="7">
-        <v>0.17420000000000002</v>
+        <v>0.17420100000000002</v>
       </c>
       <c r="I133" s="7">
-        <v>0.223572</v>
+        <v>0.223573</v>
       </c>
       <c r="J133" s="7">
-        <v>1.0174320000000001</v>
+        <v>1.017434</v>
       </c>
       <c r="K133" s="7"/>
     </row>
@@ -11322,25 +11322,25 @@
         <v>7</v>
       </c>
       <c r="E141" s="7">
-        <v>-0.052523999999999994</v>
+        <v>-0.052513</v>
       </c>
       <c r="F141" s="7">
-        <v>-0.136656</v>
+        <v>-0.13664500000000002</v>
       </c>
       <c r="G141" s="7">
-        <v>0.012830999999999999</v>
+        <v>0.012843</v>
       </c>
       <c r="H141" s="7">
-        <v>-0.04369</v>
+        <v>-0.043678999999999996</v>
       </c>
       <c r="I141" s="7">
-        <v>-0.007652</v>
+        <v>-0.007641</v>
       </c>
       <c r="J141" s="7">
-        <v>0.671357</v>
+        <v>0.671377</v>
       </c>
       <c r="K141" s="7">
-        <v>8.896251999999999</v>
+        <v>8.896367</v>
       </c>
     </row>
     <row r="142" spans="1:11" x14ac:dyDescent="0.25">
@@ -12169,19 +12169,19 @@
       </c>
       <c r="D168" s="6"/>
       <c r="E168" s="7">
-        <v>-0.005778</v>
+        <v>-0.006902</v>
       </c>
       <c r="F168" s="7">
-        <v>0.061133</v>
+        <v>0.05993299999999999</v>
       </c>
       <c r="G168" s="7">
-        <v>0.12044600000000001</v>
+        <v>0.119179</v>
       </c>
       <c r="H168" s="7">
-        <v>0.129703</v>
+        <v>0.12842599999999998</v>
       </c>
       <c r="I168" s="7">
-        <v>0.21931799999999999</v>
+        <v>0.217939</v>
       </c>
       <c r="J168" s="7"/>
       <c r="K168" s="7"/>
@@ -12592,16 +12592,16 @@
         <v>6</v>
       </c>
       <c r="E181" s="7">
-        <v>-0.16458899999999999</v>
+        <v>-0.16397099999999998</v>
       </c>
       <c r="F181" s="7">
-        <v>-0.159244</v>
+        <v>-0.158623</v>
       </c>
       <c r="G181" s="7">
-        <v>0.014865</v>
+        <v>0.015615</v>
       </c>
       <c r="H181" s="7">
-        <v>0.128392</v>
+        <v>0.129227</v>
       </c>
       <c r="I181" s="7"/>
       <c r="J181" s="7"/>
@@ -12749,19 +12749,19 @@
         <v>6</v>
       </c>
       <c r="E186" s="7">
-        <v>0</v>
+        <v>-0.089765</v>
       </c>
       <c r="F186" s="7">
-        <v>0</v>
+        <v>-0.14530200000000001</v>
       </c>
       <c r="G186" s="7">
-        <v>0</v>
+        <v>-0.031385</v>
       </c>
       <c r="H186" s="7">
-        <v>0</v>
+        <v>-0.214047</v>
       </c>
       <c r="I186" s="7">
-        <v>0</v>
+        <v>-0.195686</v>
       </c>
       <c r="J186" s="7"/>
       <c r="K186" s="7"/>
@@ -13278,10 +13278,10 @@
         <v>6</v>
       </c>
       <c r="E203" s="7">
-        <v>-0.040455</v>
+        <v>-0.040397999999999996</v>
       </c>
       <c r="F203" s="7">
-        <v>0.018484</v>
+        <v>0.018545</v>
       </c>
       <c r="G203" s="7"/>
       <c r="H203" s="7"/>
@@ -13590,16 +13590,16 @@
         <v>5</v>
       </c>
       <c r="E213" s="7">
-        <v>-0.105194</v>
+        <v>-0.104643</v>
       </c>
       <c r="F213" s="7">
-        <v>-0.114716</v>
+        <v>-0.114171</v>
       </c>
       <c r="G213" s="7">
-        <v>-0.033902</v>
+        <v>-0.033307</v>
       </c>
       <c r="H213" s="7">
-        <v>0.013485</v>
+        <v>0.014109</v>
       </c>
       <c r="I213" s="7"/>
       <c r="J213" s="7"/>
@@ -13619,16 +13619,16 @@
         <v>6</v>
       </c>
       <c r="E214" s="7">
-        <v>-0.057676</v>
+        <v>-0.057627</v>
       </c>
       <c r="F214" s="7">
-        <v>0.061288999999999996</v>
+        <v>0.061345000000000004</v>
       </c>
       <c r="G214" s="7">
-        <v>-0.063777</v>
+        <v>-0.063729</v>
       </c>
       <c r="H214" s="7">
-        <v>0.0015379999999999999</v>
+        <v>0.001591</v>
       </c>
       <c r="I214" s="7"/>
       <c r="J214" s="7"/>
@@ -14105,19 +14105,19 @@
         <v>0.072307</v>
       </c>
       <c r="G230" s="7">
-        <v>0.43056399999999995</v>
+        <v>0.430565</v>
       </c>
       <c r="H230" s="7">
-        <v>0.32445799999999997</v>
+        <v>0.324459</v>
       </c>
       <c r="I230" s="7">
-        <v>0.410322</v>
+        <v>0.410323</v>
       </c>
       <c r="J230" s="7">
-        <v>1.983308</v>
+        <v>1.98331</v>
       </c>
       <c r="K230" s="7">
-        <v>3.2885860000000005</v>
+        <v>3.288589</v>
       </c>
     </row>
     <row r="231" spans="1:11" x14ac:dyDescent="0.25">
@@ -14295,25 +14295,25 @@
         <v>4</v>
       </c>
       <c r="E236" s="7">
-        <v>-0.0088</v>
+        <v>-0.011195</v>
       </c>
       <c r="F236" s="7">
-        <v>0.052403000000000005</v>
+        <v>0.049859999999999995</v>
       </c>
       <c r="G236" s="7">
-        <v>0.091242</v>
+        <v>0.088605</v>
       </c>
       <c r="H236" s="7">
-        <v>0.15798500000000001</v>
+        <v>0.15518700000000002</v>
       </c>
       <c r="I236" s="7">
-        <v>0.326229</v>
+        <v>0.323024</v>
       </c>
       <c r="J236" s="7">
-        <v>1.884286</v>
+        <v>1.877317</v>
       </c>
       <c r="K236" s="7">
-        <v>5.638155</v>
+        <v>5.622115</v>
       </c>
     </row>
     <row r="237" spans="1:11" x14ac:dyDescent="0.25">
@@ -14726,25 +14726,25 @@
         <v>4</v>
       </c>
       <c r="E249" s="7">
-        <v>-0.017236</v>
+        <v>-0.017809</v>
       </c>
       <c r="F249" s="7">
-        <v>0.037721</v>
+        <v>0.037117</v>
       </c>
       <c r="G249" s="7">
-        <v>0.082922</v>
+        <v>0.082291</v>
       </c>
       <c r="H249" s="7">
-        <v>0.156702</v>
+        <v>0.156029</v>
       </c>
       <c r="I249" s="7">
-        <v>0.308283</v>
+        <v>0.307521</v>
       </c>
       <c r="J249" s="7">
-        <v>1.782953</v>
+        <v>1.781332</v>
       </c>
       <c r="K249" s="7">
-        <v>6.028521</v>
+        <v>6.024426999999999</v>
       </c>
     </row>
     <row r="250" spans="1:11" x14ac:dyDescent="0.25">
@@ -14761,19 +14761,19 @@
         <v>6</v>
       </c>
       <c r="E250" s="7">
-        <v>0</v>
+        <v>-0.21170100000000003</v>
       </c>
       <c r="F250" s="7">
-        <v>0</v>
+        <v>-0.15074099999999999</v>
       </c>
       <c r="G250" s="7">
-        <v>0</v>
+        <v>-0.069075</v>
       </c>
       <c r="H250" s="7">
-        <v>0</v>
+        <v>0.066244</v>
       </c>
       <c r="I250" s="7">
-        <v>0</v>
+        <v>0.076963</v>
       </c>
       <c r="J250" s="7"/>
       <c r="K250" s="7"/>
@@ -15411,19 +15411,19 @@
         <v>1</v>
       </c>
       <c r="E270" s="7">
-        <v>0</v>
+        <v>0.030302</v>
       </c>
       <c r="F270" s="7">
-        <v>0</v>
+        <v>0.099511</v>
       </c>
       <c r="G270" s="7">
-        <v>0</v>
+        <v>0.209843</v>
       </c>
       <c r="H270" s="7">
-        <v>0</v>
+        <v>0.321812</v>
       </c>
       <c r="I270" s="7">
-        <v>0</v>
+        <v>0.454509</v>
       </c>
       <c r="J270" s="7"/>
       <c r="K270" s="7"/>
@@ -16596,7 +16596,7 @@
         <v>6</v>
       </c>
       <c r="E305" s="7">
-        <v>0</v>
+        <v>-0.033083</v>
       </c>
       <c r="F305" s="7"/>
       <c r="G305" s="7"/>
@@ -16689,22 +16689,22 @@
         <v>7</v>
       </c>
       <c r="E308" s="7">
-        <v>0</v>
+        <v>-0.084987</v>
       </c>
       <c r="F308" s="7">
-        <v>0</v>
+        <v>0.057184</v>
       </c>
       <c r="G308" s="7">
-        <v>0</v>
+        <v>-0.12893000000000002</v>
       </c>
       <c r="H308" s="7">
-        <v>0</v>
+        <v>-0.106727</v>
       </c>
       <c r="I308" s="7">
-        <v>0</v>
+        <v>0.451805</v>
       </c>
       <c r="J308" s="7">
-        <v>0</v>
+        <v>3.122595</v>
       </c>
       <c r="K308" s="7"/>
     </row>
@@ -17009,22 +17009,22 @@
         <v>1</v>
       </c>
       <c r="E318" s="7">
-        <v>0</v>
+        <v>0.026261999999999997</v>
       </c>
       <c r="F318" s="7">
-        <v>0</v>
+        <v>0.099196</v>
       </c>
       <c r="G318" s="7">
-        <v>0</v>
+        <v>0.225666</v>
       </c>
       <c r="H318" s="7">
-        <v>0</v>
+        <v>0.357479</v>
       </c>
       <c r="I318" s="7">
-        <v>0</v>
+        <v>0.513075</v>
       </c>
       <c r="J318" s="7">
-        <v>0</v>
+        <v>2.762217</v>
       </c>
       <c r="K318" s="7"/>
     </row>
@@ -17042,19 +17042,19 @@
         <v>6</v>
       </c>
       <c r="E319" s="7">
-        <v>0</v>
+        <v>-0.125158</v>
       </c>
       <c r="F319" s="7">
-        <v>0</v>
+        <v>-0.061341</v>
       </c>
       <c r="G319" s="7">
-        <v>0</v>
+        <v>0.051285</v>
       </c>
       <c r="H319" s="7">
-        <v>0</v>
+        <v>0.277942</v>
       </c>
       <c r="I319" s="7">
-        <v>0</v>
+        <v>0.364902</v>
       </c>
       <c r="J319" s="7"/>
       <c r="K319" s="7"/>
@@ -17160,13 +17160,13 @@
         <v>1</v>
       </c>
       <c r="E323" s="7">
-        <v>0</v>
+        <v>0.040536</v>
       </c>
       <c r="F323" s="7">
-        <v>0</v>
+        <v>0.11426</v>
       </c>
       <c r="G323" s="7">
-        <v>0</v>
+        <v>0.23201899999999998</v>
       </c>
       <c r="H323" s="7"/>
       <c r="I323" s="7"/>
@@ -17222,25 +17222,25 @@
         <v>2</v>
       </c>
       <c r="E325" s="7">
-        <v>0</v>
+        <v>0.013117</v>
       </c>
       <c r="F325" s="7">
-        <v>0</v>
+        <v>0.075335</v>
       </c>
       <c r="G325" s="7">
-        <v>0</v>
+        <v>0.159166</v>
       </c>
       <c r="H325" s="7">
-        <v>0</v>
+        <v>0.258962</v>
       </c>
       <c r="I325" s="7">
-        <v>0</v>
+        <v>0.375638</v>
       </c>
       <c r="J325" s="7">
-        <v>0</v>
+        <v>2.074939</v>
       </c>
       <c r="K325" s="7">
-        <v>0</v>
+        <v>3.9028739999999997</v>
       </c>
     </row>
     <row r="326" spans="1:11" x14ac:dyDescent="0.25">
@@ -17255,25 +17255,25 @@
       </c>
       <c r="D326" s="6"/>
       <c r="E326" s="7">
-        <v>0</v>
+        <v>-0.008475</v>
       </c>
       <c r="F326" s="7">
-        <v>0</v>
+        <v>0.030077</v>
       </c>
       <c r="G326" s="7">
-        <v>0</v>
+        <v>0.12175000000000001</v>
       </c>
       <c r="H326" s="7">
-        <v>0</v>
+        <v>0.13170099999999998</v>
       </c>
       <c r="I326" s="7">
-        <v>0</v>
+        <v>0.201245</v>
       </c>
       <c r="J326" s="7">
-        <v>0</v>
+        <v>1.281886</v>
       </c>
       <c r="K326" s="7">
-        <v>0</v>
+        <v>5.9658619999999996</v>
       </c>
     </row>
     <row r="327" spans="1:11" x14ac:dyDescent="0.25">
@@ -17556,19 +17556,19 @@
         <v>5</v>
       </c>
       <c r="E335" s="7">
-        <v>-0.049682000000000004</v>
+        <v>-0.044866</v>
       </c>
       <c r="F335" s="7">
-        <v>-0.015205999999999999</v>
+        <v>-0.010216000000000001</v>
       </c>
       <c r="G335" s="7">
-        <v>0.02033</v>
+        <v>0.025501</v>
       </c>
       <c r="H335" s="7">
-        <v>0.155953</v>
+        <v>0.16181</v>
       </c>
       <c r="I335" s="7">
-        <v>0.270217</v>
+        <v>0.276654</v>
       </c>
       <c r="J335" s="7"/>
       <c r="K335" s="7"/>
@@ -18616,19 +18616,19 @@
         <v>6</v>
       </c>
       <c r="E367" s="7">
-        <v>0</v>
+        <v>-0.036351</v>
       </c>
       <c r="F367" s="7">
-        <v>0</v>
+        <v>0.09608</v>
       </c>
       <c r="G367" s="7">
-        <v>0</v>
+        <v>-0.0018160000000000001</v>
       </c>
       <c r="H367" s="7">
-        <v>0</v>
+        <v>0.090413</v>
       </c>
       <c r="I367" s="7">
-        <v>0</v>
+        <v>0.310348</v>
       </c>
       <c r="J367" s="7"/>
       <c r="K367" s="7"/>
@@ -18676,19 +18676,19 @@
         <v>2</v>
       </c>
       <c r="E369" s="7">
-        <v>0</v>
+        <v>-0.00208</v>
       </c>
       <c r="F369" s="7">
-        <v>0</v>
+        <v>0.012015</v>
       </c>
       <c r="G369" s="7">
-        <v>0</v>
+        <v>0.056666</v>
       </c>
       <c r="H369" s="7">
-        <v>0</v>
+        <v>0.118516</v>
       </c>
       <c r="I369" s="7">
-        <v>0</v>
+        <v>0.207101</v>
       </c>
       <c r="J369" s="7"/>
       <c r="K369" s="7"/>
@@ -18804,10 +18804,10 @@
         <v>5</v>
       </c>
       <c r="E373" s="7">
-        <v>0</v>
+        <v>-0.038983</v>
       </c>
       <c r="F373" s="7">
-        <v>0</v>
+        <v>0.103493</v>
       </c>
       <c r="G373" s="7"/>
       <c r="H373" s="7"/>
@@ -18829,19 +18829,19 @@
         <v>2</v>
       </c>
       <c r="E374" s="7">
-        <v>0</v>
+        <v>0.02077</v>
       </c>
       <c r="F374" s="7">
-        <v>0</v>
+        <v>0.068219</v>
       </c>
       <c r="G374" s="7">
-        <v>0</v>
+        <v>0.160002</v>
       </c>
       <c r="H374" s="7">
-        <v>0</v>
+        <v>0.24567699999999998</v>
       </c>
       <c r="I374" s="7">
-        <v>0</v>
+        <v>0.35253599999999996</v>
       </c>
       <c r="J374" s="7"/>
       <c r="K374" s="7"/>
@@ -18883,22 +18883,22 @@
         <v>2</v>
       </c>
       <c r="E376" s="7">
-        <v>0</v>
+        <v>0.015315</v>
       </c>
       <c r="F376" s="7">
-        <v>0</v>
+        <v>0.057159</v>
       </c>
       <c r="G376" s="7">
-        <v>0</v>
+        <v>0.108157</v>
       </c>
       <c r="H376" s="7">
-        <v>0</v>
+        <v>0.186589</v>
       </c>
       <c r="I376" s="7">
-        <v>0</v>
+        <v>0.261957</v>
       </c>
       <c r="J376" s="7">
-        <v>0</v>
+        <v>1.818835</v>
       </c>
       <c r="K376" s="7"/>
     </row>
@@ -18916,22 +18916,22 @@
         <v>3</v>
       </c>
       <c r="E377" s="7">
-        <v>0</v>
+        <v>0.019847999999999998</v>
       </c>
       <c r="F377" s="7">
-        <v>0</v>
+        <v>0.074249</v>
       </c>
       <c r="G377" s="7">
-        <v>0</v>
+        <v>0.18924</v>
       </c>
       <c r="H377" s="7">
-        <v>0</v>
+        <v>0.27459700000000004</v>
       </c>
       <c r="I377" s="7">
-        <v>0</v>
+        <v>0.38738999999999996</v>
       </c>
       <c r="J377" s="7">
-        <v>0</v>
+        <v>2.649748</v>
       </c>
       <c r="K377" s="7"/>
     </row>
@@ -18949,19 +18949,19 @@
         <v>6</v>
       </c>
       <c r="E378" s="7">
-        <v>0</v>
+        <v>-0.113954</v>
       </c>
       <c r="F378" s="7">
-        <v>0</v>
+        <v>-0.00772</v>
       </c>
       <c r="G378" s="7">
-        <v>0</v>
+        <v>0.077302</v>
       </c>
       <c r="H378" s="7">
-        <v>0</v>
+        <v>0.281658</v>
       </c>
       <c r="I378" s="7">
-        <v>0</v>
+        <v>0.255195</v>
       </c>
       <c r="J378" s="7"/>
       <c r="K378" s="7"/>
@@ -19032,22 +19032,22 @@
         <v>6</v>
       </c>
       <c r="E381" s="7">
-        <v>0</v>
+        <v>-0.112234</v>
       </c>
       <c r="F381" s="7">
-        <v>0</v>
+        <v>0.02476</v>
       </c>
       <c r="G381" s="7">
-        <v>0</v>
+        <v>0.046627</v>
       </c>
       <c r="H381" s="7">
-        <v>0</v>
+        <v>0.34663200000000005</v>
       </c>
       <c r="I381" s="7">
-        <v>0</v>
+        <v>0.328911</v>
       </c>
       <c r="J381" s="7">
-        <v>0</v>
+        <v>1.27477</v>
       </c>
       <c r="K381" s="7"/>
     </row>
@@ -19065,16 +19065,16 @@
         <v>5</v>
       </c>
       <c r="E382" s="7">
-        <v>0</v>
+        <v>0.042024</v>
       </c>
       <c r="F382" s="7">
-        <v>0</v>
+        <v>0.109385</v>
       </c>
       <c r="G382" s="7">
-        <v>0</v>
+        <v>0.141928</v>
       </c>
       <c r="H382" s="7">
-        <v>0</v>
+        <v>0.36611899999999997</v>
       </c>
       <c r="I382" s="7"/>
       <c r="J382" s="7"/>
@@ -19094,22 +19094,22 @@
         <v>7</v>
       </c>
       <c r="E383" s="7">
-        <v>0</v>
+        <v>-0.132331</v>
       </c>
       <c r="F383" s="7">
-        <v>0</v>
+        <v>-0.159619</v>
       </c>
       <c r="G383" s="7">
-        <v>0</v>
+        <v>-0.14788</v>
       </c>
       <c r="H383" s="7">
-        <v>0</v>
+        <v>-0.069497</v>
       </c>
       <c r="I383" s="7">
-        <v>0</v>
+        <v>-0.095369</v>
       </c>
       <c r="J383" s="7">
-        <v>0</v>
+        <v>1.070855</v>
       </c>
       <c r="K383" s="7"/>
     </row>
@@ -19127,19 +19127,19 @@
         <v>3</v>
       </c>
       <c r="E384" s="7">
-        <v>0</v>
+        <v>0.024054000000000002</v>
       </c>
       <c r="F384" s="7">
-        <v>0</v>
+        <v>0.08440099999999999</v>
       </c>
       <c r="G384" s="7">
-        <v>0</v>
+        <v>0.18777999999999997</v>
       </c>
       <c r="H384" s="7">
-        <v>0</v>
+        <v>0.303533</v>
       </c>
       <c r="I384" s="7">
-        <v>0</v>
+        <v>0.449511</v>
       </c>
       <c r="J384" s="7"/>
       <c r="K384" s="7"/>
@@ -19158,16 +19158,16 @@
         <v>6</v>
       </c>
       <c r="E385" s="7">
-        <v>0</v>
+        <v>-0.075964</v>
       </c>
       <c r="F385" s="7">
-        <v>0</v>
+        <v>-0.05391</v>
       </c>
       <c r="G385" s="7">
-        <v>0</v>
+        <v>-0.21259</v>
       </c>
       <c r="H385" s="7">
-        <v>0</v>
+        <v>-0.390194</v>
       </c>
       <c r="I385" s="7"/>
       <c r="J385" s="7"/>
@@ -19218,22 +19218,22 @@
         <v>2</v>
       </c>
       <c r="E387" s="7">
-        <v>0</v>
+        <v>0.023874</v>
       </c>
       <c r="F387" s="7">
-        <v>0</v>
+        <v>0.076648</v>
       </c>
       <c r="G387" s="7">
-        <v>0</v>
+        <v>0.17334700000000003</v>
       </c>
       <c r="H387" s="7">
-        <v>0</v>
+        <v>0.266719</v>
       </c>
       <c r="I387" s="7">
-        <v>0</v>
+        <v>0.374089</v>
       </c>
       <c r="J387" s="7">
-        <v>0</v>
+        <v>2.464659</v>
       </c>
       <c r="K387" s="7"/>
     </row>
@@ -19282,22 +19282,22 @@
         <v>6</v>
       </c>
       <c r="E389" s="7">
-        <v>0</v>
+        <v>-0.036091000000000005</v>
       </c>
       <c r="F389" s="7">
-        <v>0</v>
+        <v>0.101343</v>
       </c>
       <c r="G389" s="7">
-        <v>0</v>
+        <v>0.10756500000000001</v>
       </c>
       <c r="H389" s="7">
-        <v>0</v>
+        <v>0.32233199999999995</v>
       </c>
       <c r="I389" s="7">
-        <v>0</v>
+        <v>0.403439</v>
       </c>
       <c r="J389" s="7">
-        <v>0</v>
+        <v>1.627724</v>
       </c>
       <c r="K389" s="7"/>
     </row>
@@ -19346,22 +19346,22 @@
         <v>6</v>
       </c>
       <c r="E391" s="7">
-        <v>0</v>
+        <v>-0.09223699999999999</v>
       </c>
       <c r="F391" s="7">
-        <v>0</v>
+        <v>-0.047571</v>
       </c>
       <c r="G391" s="7">
-        <v>0</v>
+        <v>0.016659999999999998</v>
       </c>
       <c r="H391" s="7">
-        <v>0</v>
+        <v>0.010297</v>
       </c>
       <c r="I391" s="7">
-        <v>0</v>
+        <v>0.017925</v>
       </c>
       <c r="J391" s="7">
-        <v>0</v>
+        <v>0.6441880000000001</v>
       </c>
       <c r="K391" s="7"/>
     </row>
@@ -19379,16 +19379,16 @@
         <v>1</v>
       </c>
       <c r="E392" s="7">
-        <v>0</v>
+        <v>0.02328</v>
       </c>
       <c r="F392" s="7">
-        <v>0</v>
+        <v>0.102837</v>
       </c>
       <c r="G392" s="7">
-        <v>0</v>
+        <v>0.227288</v>
       </c>
       <c r="H392" s="7">
-        <v>0</v>
+        <v>0.365541</v>
       </c>
       <c r="I392" s="7"/>
       <c r="J392" s="7"/>
@@ -19408,22 +19408,22 @@
         <v>7</v>
       </c>
       <c r="E393" s="7">
-        <v>0</v>
+        <v>-0.35979799999999995</v>
       </c>
       <c r="F393" s="7">
-        <v>0</v>
+        <v>-0.39780299999999996</v>
       </c>
       <c r="G393" s="7">
-        <v>0</v>
+        <v>-0.335199</v>
       </c>
       <c r="H393" s="7">
-        <v>0</v>
+        <v>-0.38429800000000003</v>
       </c>
       <c r="I393" s="7">
-        <v>0</v>
+        <v>-0.46962499999999996</v>
       </c>
       <c r="J393" s="7">
-        <v>0</v>
+        <v>-0.057312</v>
       </c>
       <c r="K393" s="7"/>
     </row>
@@ -19472,22 +19472,22 @@
         <v>5</v>
       </c>
       <c r="E395" s="7">
-        <v>0</v>
+        <v>0.111594</v>
       </c>
       <c r="F395" s="7">
-        <v>0</v>
+        <v>0.20877700000000002</v>
       </c>
       <c r="G395" s="7">
-        <v>0</v>
+        <v>0.277523</v>
       </c>
       <c r="H395" s="7">
-        <v>0</v>
+        <v>0.264362</v>
       </c>
       <c r="I395" s="7">
-        <v>0</v>
+        <v>0.273904</v>
       </c>
       <c r="J395" s="7">
-        <v>0</v>
+        <v>0.972135</v>
       </c>
       <c r="K395" s="7"/>
     </row>
@@ -19536,19 +19536,19 @@
       </c>
       <c r="D397" s="6"/>
       <c r="E397" s="7">
-        <v>0</v>
+        <v>0.014006000000000001</v>
       </c>
       <c r="F397" s="7">
-        <v>0</v>
+        <v>0.056935</v>
       </c>
       <c r="G397" s="7">
-        <v>0</v>
+        <v>0.077432</v>
       </c>
       <c r="H397" s="7">
-        <v>0</v>
+        <v>0.12403700000000001</v>
       </c>
       <c r="I397" s="7">
-        <v>0</v>
+        <v>0.168617</v>
       </c>
       <c r="J397" s="7"/>
       <c r="K397" s="7"/>
@@ -19662,22 +19662,22 @@
       </c>
       <c r="D401" s="6"/>
       <c r="E401" s="7">
-        <v>0</v>
+        <v>0.019574</v>
       </c>
       <c r="F401" s="7">
-        <v>0</v>
+        <v>0.06520100000000001</v>
       </c>
       <c r="G401" s="7">
-        <v>0</v>
+        <v>0.131556</v>
       </c>
       <c r="H401" s="7">
-        <v>0</v>
+        <v>0.17690899999999998</v>
       </c>
       <c r="I401" s="7">
-        <v>0</v>
+        <v>0.216269</v>
       </c>
       <c r="J401" s="7">
-        <v>0</v>
+        <v>1.128516</v>
       </c>
       <c r="K401" s="7"/>
     </row>
@@ -19728,19 +19728,19 @@
         <v>1</v>
       </c>
       <c r="E403" s="7">
-        <v>0</v>
+        <v>0.022803</v>
       </c>
       <c r="F403" s="7">
-        <v>0</v>
+        <v>0.08286500000000001</v>
       </c>
       <c r="G403" s="7">
-        <v>0</v>
+        <v>0.19392199999999998</v>
       </c>
       <c r="H403" s="7">
-        <v>0</v>
+        <v>0.305775</v>
       </c>
       <c r="I403" s="7">
-        <v>0</v>
+        <v>0.43770600000000004</v>
       </c>
       <c r="J403" s="7"/>
       <c r="K403" s="7"/>
@@ -19984,19 +19984,19 @@
         <v>4</v>
       </c>
       <c r="E411" s="7">
-        <v>0</v>
+        <v>0.026423000000000002</v>
       </c>
       <c r="F411" s="7">
-        <v>0</v>
+        <v>0.118178</v>
       </c>
       <c r="G411" s="7">
-        <v>0</v>
+        <v>0.42623199999999994</v>
       </c>
       <c r="H411" s="7">
-        <v>0</v>
+        <v>0.34608199999999995</v>
       </c>
       <c r="I411" s="7">
-        <v>0</v>
+        <v>0.386468</v>
       </c>
       <c r="J411" s="7"/>
       <c r="K411" s="7"/>
@@ -20015,10 +20015,10 @@
         <v>6</v>
       </c>
       <c r="E412" s="7">
-        <v>-0.075158</v>
+        <v>-0.076486</v>
       </c>
       <c r="F412" s="7">
-        <v>-0.056268000000000006</v>
+        <v>-0.057622</v>
       </c>
       <c r="G412" s="7"/>
       <c r="H412" s="7"/>
@@ -20098,22 +20098,22 @@
         <v>2</v>
       </c>
       <c r="E415" s="7">
-        <v>0</v>
+        <v>0.031948</v>
       </c>
       <c r="F415" s="7">
-        <v>0</v>
+        <v>-0.074514</v>
       </c>
       <c r="G415" s="7">
-        <v>0</v>
+        <v>0.021602</v>
       </c>
       <c r="H415" s="7">
-        <v>0</v>
+        <v>0.12642799999999998</v>
       </c>
       <c r="I415" s="7">
-        <v>0</v>
+        <v>0.24521</v>
       </c>
       <c r="J415" s="7">
-        <v>0</v>
+        <v>2.1327789999999998</v>
       </c>
       <c r="K415" s="7"/>
     </row>
@@ -20327,25 +20327,25 @@
         <v>1</v>
       </c>
       <c r="E422" s="7">
-        <v>0</v>
+        <v>0.024438</v>
       </c>
       <c r="F422" s="7">
-        <v>0</v>
+        <v>0.093424</v>
       </c>
       <c r="G422" s="7">
-        <v>0</v>
+        <v>0.20529499999999998</v>
       </c>
       <c r="H422" s="7">
-        <v>0</v>
+        <v>0.316635</v>
       </c>
       <c r="I422" s="7">
-        <v>0</v>
+        <v>0.460544</v>
       </c>
       <c r="J422" s="7">
-        <v>0</v>
+        <v>2.64096</v>
       </c>
       <c r="K422" s="7">
-        <v>0</v>
+        <v>4.837326</v>
       </c>
     </row>
     <row r="423" spans="1:11" x14ac:dyDescent="0.25">
@@ -20494,22 +20494,22 @@
         <v>3</v>
       </c>
       <c r="E427" s="7">
-        <v>0.024116</v>
+        <v>0.024107</v>
       </c>
       <c r="F427" s="7">
-        <v>0.079455</v>
+        <v>0.079446</v>
       </c>
       <c r="G427" s="7">
-        <v>0.176021</v>
+        <v>0.17601199999999997</v>
       </c>
       <c r="H427" s="7">
-        <v>0.26609700000000003</v>
+        <v>0.266086</v>
       </c>
       <c r="I427" s="7">
-        <v>0.372139</v>
+        <v>0.372127</v>
       </c>
       <c r="J427" s="7">
-        <v>2.1225620000000003</v>
+        <v>2.122536</v>
       </c>
       <c r="K427" s="7"/>
     </row>
@@ -20593,25 +20593,25 @@
         <v>6</v>
       </c>
       <c r="E430" s="7">
-        <v>0</v>
+        <v>-0.037426</v>
       </c>
       <c r="F430" s="7">
-        <v>0</v>
+        <v>0.08497400000000001</v>
       </c>
       <c r="G430" s="7">
-        <v>0</v>
+        <v>-0.015346</v>
       </c>
       <c r="H430" s="7">
-        <v>0</v>
+        <v>0.048699000000000006</v>
       </c>
       <c r="I430" s="7">
-        <v>0</v>
+        <v>0.21100100000000002</v>
       </c>
       <c r="J430" s="7">
-        <v>0</v>
+        <v>2.7054</v>
       </c>
       <c r="K430" s="7">
-        <v>0</v>
+        <v>10.564579000000002</v>
       </c>
     </row>
     <row r="431" spans="1:11" x14ac:dyDescent="0.25">
@@ -20628,25 +20628,25 @@
         <v>4</v>
       </c>
       <c r="E431" s="7">
-        <v>0</v>
+        <v>-0.032536</v>
       </c>
       <c r="F431" s="7">
-        <v>0</v>
+        <v>0.00105</v>
       </c>
       <c r="G431" s="7">
-        <v>0</v>
+        <v>0.086384</v>
       </c>
       <c r="H431" s="7">
-        <v>0</v>
+        <v>0.183574</v>
       </c>
       <c r="I431" s="7">
-        <v>0</v>
+        <v>0.246449</v>
       </c>
       <c r="J431" s="7">
-        <v>0</v>
+        <v>1.518582</v>
       </c>
       <c r="K431" s="7">
-        <v>0</v>
+        <v>8.020407</v>
       </c>
     </row>
     <row r="432" spans="1:11" x14ac:dyDescent="0.25">
@@ -20663,25 +20663,25 @@
         <v>2</v>
       </c>
       <c r="E432" s="7">
-        <v>0</v>
+        <v>0.026059000000000002</v>
       </c>
       <c r="F432" s="7">
-        <v>0</v>
+        <v>0.089803</v>
       </c>
       <c r="G432" s="7">
-        <v>0</v>
+        <v>0.17921199999999998</v>
       </c>
       <c r="H432" s="7">
-        <v>0</v>
+        <v>0.249015</v>
       </c>
       <c r="I432" s="7">
-        <v>0</v>
+        <v>0.360573</v>
       </c>
       <c r="J432" s="7">
-        <v>0</v>
+        <v>2.065884</v>
       </c>
       <c r="K432" s="7">
-        <v>0</v>
+        <v>5.241354</v>
       </c>
     </row>
     <row r="433" spans="1:11" x14ac:dyDescent="0.25">
@@ -20733,25 +20733,25 @@
         <v>6</v>
       </c>
       <c r="E434" s="7">
-        <v>0</v>
+        <v>-0.070793</v>
       </c>
       <c r="F434" s="7">
-        <v>0</v>
+        <v>-0.056414</v>
       </c>
       <c r="G434" s="7">
-        <v>0</v>
+        <v>0.057435</v>
       </c>
       <c r="H434" s="7">
-        <v>0</v>
+        <v>0.158975</v>
       </c>
       <c r="I434" s="7">
-        <v>0</v>
+        <v>0.158135</v>
       </c>
       <c r="J434" s="7">
-        <v>0</v>
+        <v>0.77959</v>
       </c>
       <c r="K434" s="7">
-        <v>0</v>
+        <v>13.186811</v>
       </c>
     </row>
     <row r="435" spans="1:11" x14ac:dyDescent="0.25">
@@ -20837,25 +20837,25 @@
       </c>
       <c r="D438" s="6"/>
       <c r="E438" s="7">
-        <v>0</v>
+        <v>0.009531</v>
       </c>
       <c r="F438" s="7">
-        <v>0</v>
+        <v>0.045240999999999996</v>
       </c>
       <c r="G438" s="7">
-        <v>0</v>
+        <v>0.07843</v>
       </c>
       <c r="H438" s="7">
-        <v>0</v>
+        <v>0.126855</v>
       </c>
       <c r="I438" s="7">
-        <v>0</v>
+        <v>0.132403</v>
       </c>
       <c r="J438" s="7">
-        <v>0</v>
+        <v>0.727605</v>
       </c>
       <c r="K438" s="7">
-        <v>0</v>
+        <v>4.126455</v>
       </c>
     </row>
     <row r="439" spans="1:11" x14ac:dyDescent="0.25">
@@ -20872,25 +20872,25 @@
         <v>2</v>
       </c>
       <c r="E439" s="7">
-        <v>0</v>
+        <v>0.024157</v>
       </c>
       <c r="F439" s="7">
-        <v>0</v>
+        <v>0.06759699999999999</v>
       </c>
       <c r="G439" s="7">
-        <v>0</v>
+        <v>0.16090800000000002</v>
       </c>
       <c r="H439" s="7">
-        <v>0</v>
+        <v>0.22358699999999998</v>
       </c>
       <c r="I439" s="7">
-        <v>0</v>
+        <v>0.305045</v>
       </c>
       <c r="J439" s="7">
-        <v>0</v>
+        <v>2.084693</v>
       </c>
       <c r="K439" s="7">
-        <v>0</v>
+        <v>4.556831</v>
       </c>
     </row>
     <row r="440" spans="1:11" x14ac:dyDescent="0.25">
@@ -21140,25 +21140,25 @@
         <v>4</v>
       </c>
       <c r="E447" s="7">
-        <v>0</v>
+        <v>0.011022</v>
       </c>
       <c r="F447" s="7">
-        <v>0</v>
+        <v>0.04156</v>
       </c>
       <c r="G447" s="7">
-        <v>0</v>
+        <v>0.178361</v>
       </c>
       <c r="H447" s="7">
-        <v>0</v>
+        <v>0.315161</v>
       </c>
       <c r="I447" s="7">
-        <v>0</v>
+        <v>0.469943</v>
       </c>
       <c r="J447" s="7">
-        <v>0</v>
+        <v>2.367433</v>
       </c>
       <c r="K447" s="7">
-        <v>0</v>
+        <v>6.058825000000001</v>
       </c>
     </row>
     <row r="448" spans="1:11" x14ac:dyDescent="0.25">
@@ -21262,22 +21262,22 @@
         <v>6</v>
       </c>
       <c r="E451" s="7">
-        <v>0</v>
+        <v>-0.071508</v>
       </c>
       <c r="F451" s="7">
-        <v>0</v>
+        <v>-0.09398</v>
       </c>
       <c r="G451" s="7">
-        <v>0</v>
+        <v>-0.012087</v>
       </c>
       <c r="H451" s="7">
-        <v>0</v>
+        <v>0.080147</v>
       </c>
       <c r="I451" s="7">
-        <v>0</v>
+        <v>0.064163</v>
       </c>
       <c r="J451" s="7">
-        <v>0</v>
+        <v>0.6533880000000001</v>
       </c>
       <c r="K451" s="7"/>
     </row>
@@ -22217,25 +22217,25 @@
         <v>5</v>
       </c>
       <c r="E480" s="7">
-        <v>0</v>
+        <v>-0.016555</v>
       </c>
       <c r="F480" s="7">
-        <v>0</v>
+        <v>0.038751</v>
       </c>
       <c r="G480" s="7">
-        <v>0</v>
+        <v>0.092643</v>
       </c>
       <c r="H480" s="7">
-        <v>0</v>
+        <v>0.093056</v>
       </c>
       <c r="I480" s="7">
-        <v>0</v>
+        <v>0.225226</v>
       </c>
       <c r="J480" s="7">
-        <v>0</v>
+        <v>0.968487</v>
       </c>
       <c r="K480" s="7">
-        <v>0</v>
+        <v>3.127234</v>
       </c>
     </row>
     <row r="481" spans="1:11" x14ac:dyDescent="0.25">
@@ -22518,22 +22518,22 @@
         <v>3</v>
       </c>
       <c r="E489" s="7">
-        <v>0</v>
+        <v>0.015182</v>
       </c>
       <c r="F489" s="7">
-        <v>0</v>
+        <v>0.10206</v>
       </c>
       <c r="G489" s="7">
-        <v>0</v>
+        <v>0.253231</v>
       </c>
       <c r="H489" s="7">
-        <v>0</v>
+        <v>0.389706</v>
       </c>
       <c r="I489" s="7">
-        <v>0</v>
+        <v>0.580621</v>
       </c>
       <c r="J489" s="7">
-        <v>0</v>
+        <v>2.111663</v>
       </c>
       <c r="K489" s="7"/>
     </row>
@@ -23195,19 +23195,19 @@
         <v>6</v>
       </c>
       <c r="E510" s="7">
-        <v>0</v>
+        <v>-0.060136</v>
       </c>
       <c r="F510" s="7">
-        <v>0</v>
+        <v>-0.005704</v>
       </c>
       <c r="G510" s="7">
-        <v>0</v>
+        <v>0.040951</v>
       </c>
       <c r="H510" s="7">
-        <v>0</v>
+        <v>0.195202</v>
       </c>
       <c r="I510" s="7">
-        <v>0</v>
+        <v>0.284502</v>
       </c>
       <c r="J510" s="7"/>
       <c r="K510" s="7"/>
@@ -23400,19 +23400,19 @@
         <v>6</v>
       </c>
       <c r="E517" s="7">
-        <v>-0.071116</v>
+        <v>-0.071113</v>
       </c>
       <c r="F517" s="7">
-        <v>0.062599</v>
+        <v>0.062603</v>
       </c>
       <c r="G517" s="7">
-        <v>-0.090094</v>
+        <v>-0.090091</v>
       </c>
       <c r="H517" s="7">
-        <v>-0.057293000000000004</v>
+        <v>-0.05728900000000001</v>
       </c>
       <c r="I517" s="7">
-        <v>0.49579900000000005</v>
+        <v>0.49580399999999997</v>
       </c>
       <c r="J517" s="7"/>
       <c r="K517" s="7"/>
@@ -23493,19 +23493,19 @@
         <v>7</v>
       </c>
       <c r="E520" s="7">
-        <v>0</v>
+        <v>-0.225582</v>
       </c>
       <c r="F520" s="7">
-        <v>0</v>
+        <v>-0.19733699999999998</v>
       </c>
       <c r="G520" s="7">
-        <v>0</v>
+        <v>-0.101281</v>
       </c>
       <c r="H520" s="7">
-        <v>0</v>
+        <v>0.025041</v>
       </c>
       <c r="I520" s="7">
-        <v>0</v>
+        <v>0.016519</v>
       </c>
       <c r="J520" s="7"/>
       <c r="K520" s="7"/>
@@ -23685,22 +23685,22 @@
         <v>2</v>
       </c>
       <c r="E526" s="7">
-        <v>0.032225000000000004</v>
+        <v>0.032226</v>
       </c>
       <c r="F526" s="7">
-        <v>0.11066000000000001</v>
+        <v>0.11066100000000001</v>
       </c>
       <c r="G526" s="7">
         <v>0.230187</v>
       </c>
       <c r="H526" s="7">
-        <v>0.319432</v>
+        <v>0.319433</v>
       </c>
       <c r="I526" s="7">
-        <v>0.456885</v>
+        <v>0.456886</v>
       </c>
       <c r="J526" s="7">
-        <v>2.595055</v>
+        <v>2.595056</v>
       </c>
       <c r="K526" s="7"/>
     </row>
@@ -23718,19 +23718,19 @@
         <v>2</v>
       </c>
       <c r="E527" s="7">
-        <v>0</v>
+        <v>0.026173000000000002</v>
       </c>
       <c r="F527" s="7">
-        <v>0</v>
+        <v>0.087326</v>
       </c>
       <c r="G527" s="7">
-        <v>0</v>
+        <v>0.187183</v>
       </c>
       <c r="H527" s="7">
-        <v>0</v>
+        <v>0.27027999999999996</v>
       </c>
       <c r="I527" s="7">
-        <v>0</v>
+        <v>0.34027999999999997</v>
       </c>
       <c r="J527" s="7"/>
       <c r="K527" s="7"/>
@@ -23815,19 +23815,19 @@
         <v>4</v>
       </c>
       <c r="E530" s="7">
-        <v>0</v>
+        <v>-0.004852</v>
       </c>
       <c r="F530" s="7">
-        <v>0</v>
+        <v>0.050321</v>
       </c>
       <c r="G530" s="7">
-        <v>0</v>
+        <v>0.100609</v>
       </c>
       <c r="H530" s="7">
-        <v>0</v>
+        <v>0.120774</v>
       </c>
       <c r="I530" s="7">
-        <v>0</v>
+        <v>0.165382</v>
       </c>
       <c r="J530" s="7"/>
       <c r="K530" s="7"/>
@@ -24156,19 +24156,19 @@
         <v>5</v>
       </c>
       <c r="E541" s="7">
-        <v>-0.05437</v>
+        <v>-0.054558</v>
       </c>
       <c r="F541" s="7">
-        <v>0.088565</v>
+        <v>0.088349</v>
       </c>
       <c r="G541" s="7">
-        <v>0.10876</v>
+        <v>0.10854</v>
       </c>
       <c r="H541" s="7">
-        <v>0.43422499999999997</v>
+        <v>0.433941</v>
       </c>
       <c r="I541" s="7">
-        <v>0.5695239999999999</v>
+        <v>0.569213</v>
       </c>
       <c r="J541" s="7"/>
       <c r="K541" s="7"/>
@@ -24243,19 +24243,19 @@
         <v>6</v>
       </c>
       <c r="E544" s="7">
-        <v>0</v>
+        <v>-0.008637</v>
       </c>
       <c r="F544" s="7">
-        <v>0</v>
+        <v>0.039608</v>
       </c>
       <c r="G544" s="7">
-        <v>0</v>
+        <v>0.06827</v>
       </c>
       <c r="H544" s="7">
-        <v>0</v>
+        <v>0.076555</v>
       </c>
       <c r="I544" s="7">
-        <v>0</v>
+        <v>0.102551</v>
       </c>
       <c r="J544" s="7"/>
       <c r="K544" s="7"/>
@@ -24462,19 +24462,19 @@
         <v>1</v>
       </c>
       <c r="E551" s="7">
-        <v>0.02944</v>
+        <v>0.029405999999999998</v>
       </c>
       <c r="F551" s="7">
-        <v>0.100029</v>
+        <v>0.099993</v>
       </c>
       <c r="G551" s="7">
-        <v>0.21363600000000002</v>
+        <v>0.213597</v>
       </c>
       <c r="H551" s="7">
-        <v>0.331412</v>
+        <v>0.33136899999999997</v>
       </c>
       <c r="I551" s="7">
-        <v>0.471578</v>
+        <v>0.47153</v>
       </c>
       <c r="J551" s="7"/>
       <c r="K551" s="7"/>
@@ -24561,25 +24561,25 @@
         <v>5</v>
       </c>
       <c r="E554" s="7">
-        <v>0</v>
+        <v>-0.021928</v>
       </c>
       <c r="F554" s="7">
-        <v>0</v>
+        <v>0.046659</v>
       </c>
       <c r="G554" s="7">
-        <v>0</v>
+        <v>0.124307</v>
       </c>
       <c r="H554" s="7">
-        <v>0</v>
+        <v>0.23319099999999998</v>
       </c>
       <c r="I554" s="7">
-        <v>0</v>
+        <v>0.354897</v>
       </c>
       <c r="J554" s="7">
-        <v>0</v>
+        <v>2.088691</v>
       </c>
       <c r="K554" s="7">
-        <v>0</v>
+        <v>10.055814</v>
       </c>
     </row>
     <row r="555" spans="1:11" x14ac:dyDescent="0.25">
@@ -24623,25 +24623,25 @@
         <v>5</v>
       </c>
       <c r="E556" s="7">
-        <v>0</v>
+        <v>0.000373</v>
       </c>
       <c r="F556" s="7">
-        <v>0</v>
+        <v>0.056326999999999995</v>
       </c>
       <c r="G556" s="7">
-        <v>0</v>
+        <v>0.144392</v>
       </c>
       <c r="H556" s="7">
-        <v>0</v>
+        <v>0.153814</v>
       </c>
       <c r="I556" s="7">
-        <v>0</v>
+        <v>0.21282800000000002</v>
       </c>
       <c r="J556" s="7">
-        <v>0</v>
+        <v>1.3249119999999999</v>
       </c>
       <c r="K556" s="7">
-        <v>0</v>
+        <v>5.619389999999999</v>
       </c>
     </row>
     <row r="557" spans="1:11" x14ac:dyDescent="0.25">
@@ -24658,25 +24658,25 @@
         <v>3</v>
       </c>
       <c r="E557" s="7">
-        <v>0</v>
+        <v>0.006714</v>
       </c>
       <c r="F557" s="7">
-        <v>0</v>
+        <v>0.049572000000000005</v>
       </c>
       <c r="G557" s="7">
-        <v>0</v>
+        <v>0.123764</v>
       </c>
       <c r="H557" s="7">
-        <v>0</v>
+        <v>0.16220600000000002</v>
       </c>
       <c r="I557" s="7">
-        <v>0</v>
+        <v>0.219205</v>
       </c>
       <c r="J557" s="7">
-        <v>0</v>
+        <v>1.152105</v>
       </c>
       <c r="K557" s="7">
-        <v>0</v>
+        <v>6.090031</v>
       </c>
     </row>
     <row r="558" spans="1:11" x14ac:dyDescent="0.25">
@@ -24693,22 +24693,22 @@
         <v>2</v>
       </c>
       <c r="E558" s="7">
-        <v>0</v>
+        <v>0.026407</v>
       </c>
       <c r="F558" s="7">
-        <v>0</v>
+        <v>0.102027</v>
       </c>
       <c r="G558" s="7">
-        <v>0</v>
+        <v>0.22084099999999998</v>
       </c>
       <c r="H558" s="7">
-        <v>0</v>
+        <v>0.347325</v>
       </c>
       <c r="I558" s="7">
-        <v>0</v>
+        <v>0.49975499999999995</v>
       </c>
       <c r="J558" s="7">
-        <v>0</v>
+        <v>2.823048</v>
       </c>
       <c r="K558" s="7"/>
     </row>
@@ -24887,19 +24887,19 @@
         <v>6</v>
       </c>
       <c r="E564" s="7">
-        <v>0.054661</v>
+        <v>0.054397</v>
       </c>
       <c r="F564" s="7">
-        <v>0.057189</v>
+        <v>0.056924</v>
       </c>
       <c r="G564" s="7">
-        <v>0.569464</v>
+        <v>0.56907</v>
       </c>
       <c r="H564" s="7">
-        <v>0.6039249999999999</v>
+        <v>0.603523</v>
       </c>
       <c r="I564" s="7">
-        <v>0.663973</v>
+        <v>0.6635559999999999</v>
       </c>
       <c r="J564" s="7"/>
       <c r="K564" s="7"/>
@@ -25182,25 +25182,25 @@
         <v>6</v>
       </c>
       <c r="E573" s="7">
-        <v>0</v>
+        <v>0.0069689999999999995</v>
       </c>
       <c r="F573" s="7">
-        <v>0</v>
+        <v>0.06038299999999999</v>
       </c>
       <c r="G573" s="7">
-        <v>0</v>
+        <v>0.167955</v>
       </c>
       <c r="H573" s="7">
-        <v>0</v>
+        <v>0.135464</v>
       </c>
       <c r="I573" s="7">
-        <v>0</v>
+        <v>0.178633</v>
       </c>
       <c r="J573" s="7">
-        <v>0</v>
+        <v>1.512431</v>
       </c>
       <c r="K573" s="7">
-        <v>0</v>
+        <v>6.505163</v>
       </c>
     </row>
     <row r="574" spans="1:11" x14ac:dyDescent="0.25">
@@ -25248,22 +25248,22 @@
         <v>6</v>
       </c>
       <c r="E575" s="7">
-        <v>-0.049542</v>
+        <v>-0.049557000000000004</v>
       </c>
       <c r="F575" s="7">
-        <v>0.083222</v>
+        <v>0.083206</v>
       </c>
       <c r="G575" s="7">
-        <v>-0.036715</v>
+        <v>-0.036729</v>
       </c>
       <c r="H575" s="7">
-        <v>0.036208</v>
+        <v>0.036192</v>
       </c>
       <c r="I575" s="7">
-        <v>0.390923</v>
+        <v>0.390901</v>
       </c>
       <c r="J575" s="7">
-        <v>3.070084</v>
+        <v>3.0700209999999997</v>
       </c>
       <c r="K575" s="7"/>
     </row>
@@ -25281,16 +25281,16 @@
         <v>2</v>
       </c>
       <c r="E576" s="7">
-        <v>0</v>
+        <v>0.024186</v>
       </c>
       <c r="F576" s="7">
-        <v>0</v>
+        <v>0.077926</v>
       </c>
       <c r="G576" s="7">
-        <v>0</v>
+        <v>0.172673</v>
       </c>
       <c r="H576" s="7">
-        <v>0</v>
+        <v>0.264928</v>
       </c>
       <c r="I576" s="7"/>
       <c r="J576" s="7"/>
@@ -25403,25 +25403,25 @@
         <v>6</v>
       </c>
       <c r="E580" s="7">
-        <v>0</v>
+        <v>-0.09565099999999999</v>
       </c>
       <c r="F580" s="7">
-        <v>0</v>
+        <v>-0.088989</v>
       </c>
       <c r="G580" s="7">
-        <v>0</v>
+        <v>-0.068093</v>
       </c>
       <c r="H580" s="7">
-        <v>0</v>
+        <v>-0.00738</v>
       </c>
       <c r="I580" s="7">
-        <v>0</v>
+        <v>0.053492</v>
       </c>
       <c r="J580" s="7">
-        <v>0</v>
+        <v>0.695176</v>
       </c>
       <c r="K580" s="7">
-        <v>0</v>
+        <v>11.264576</v>
       </c>
     </row>
     <row r="581" spans="1:11" x14ac:dyDescent="0.25">
@@ -25438,19 +25438,19 @@
         <v>3</v>
       </c>
       <c r="E581" s="7">
-        <v>0</v>
+        <v>-0.0013</v>
       </c>
       <c r="F581" s="7">
-        <v>0</v>
+        <v>0.026082</v>
       </c>
       <c r="G581" s="7">
-        <v>0</v>
+        <v>0.141164</v>
       </c>
       <c r="H581" s="7">
-        <v>0</v>
+        <v>0.17305</v>
       </c>
       <c r="I581" s="7">
-        <v>0</v>
+        <v>0.24947299999999997</v>
       </c>
       <c r="J581" s="7"/>
       <c r="K581" s="7"/>
@@ -25942,19 +25942,19 @@
         <v>6</v>
       </c>
       <c r="E597" s="7">
-        <v>0.031702</v>
+        <v>0.03266</v>
       </c>
       <c r="F597" s="7">
-        <v>0.194775</v>
+        <v>0.195885</v>
       </c>
       <c r="G597" s="7">
-        <v>0.064427</v>
+        <v>0.065416</v>
       </c>
       <c r="H597" s="7">
-        <v>0.20739999999999997</v>
+        <v>0.208521</v>
       </c>
       <c r="I597" s="7">
-        <v>0.347965</v>
+        <v>0.349217</v>
       </c>
       <c r="J597" s="7"/>
       <c r="K597" s="7"/>
@@ -26037,19 +26037,19 @@
         <v>2</v>
       </c>
       <c r="E600" s="7">
-        <v>0</v>
+        <v>0.014959</v>
       </c>
       <c r="F600" s="7">
-        <v>0</v>
+        <v>0.10164</v>
       </c>
       <c r="G600" s="7">
-        <v>0</v>
+        <v>0.152076</v>
       </c>
       <c r="H600" s="7">
-        <v>0</v>
+        <v>0.199583</v>
       </c>
       <c r="I600" s="7">
-        <v>0</v>
+        <v>0.306898</v>
       </c>
       <c r="J600" s="7"/>
       <c r="K600" s="7"/>
@@ -26462,19 +26462,19 @@
         <v>1</v>
       </c>
       <c r="E613" s="7">
-        <v>0.027745000000000002</v>
+        <v>0.027746</v>
       </c>
       <c r="F613" s="7">
-        <v>0.09061</v>
+        <v>0.090611</v>
       </c>
       <c r="G613" s="7">
-        <v>0.199085</v>
+        <v>0.19908599999999999</v>
       </c>
       <c r="H613" s="7">
         <v>0.302623</v>
       </c>
       <c r="I613" s="7">
-        <v>0.42790100000000003</v>
+        <v>0.427902</v>
       </c>
       <c r="J613" s="7"/>
       <c r="K613" s="7"/>
@@ -26590,25 +26590,25 @@
         <v>7</v>
       </c>
       <c r="E617" s="7">
-        <v>0.024177</v>
+        <v>0.024190999999999997</v>
       </c>
       <c r="F617" s="7">
-        <v>-0.057103</v>
+        <v>-0.057091</v>
       </c>
       <c r="G617" s="7">
-        <v>0.125308</v>
+        <v>0.125323</v>
       </c>
       <c r="H617" s="7">
-        <v>0.127872</v>
+        <v>0.127887</v>
       </c>
       <c r="I617" s="7">
-        <v>0.139762</v>
+        <v>0.139777</v>
       </c>
       <c r="J617" s="7">
-        <v>1.14573</v>
+        <v>1.145758</v>
       </c>
       <c r="K617" s="7">
-        <v>5.4113999999999995</v>
+        <v>5.411486</v>
       </c>
     </row>
     <row r="618" spans="1:11" x14ac:dyDescent="0.25">
@@ -26658,19 +26658,19 @@
       </c>
       <c r="D619" s="6"/>
       <c r="E619" s="7">
-        <v>0</v>
+        <v>-0.030179</v>
       </c>
       <c r="F619" s="7">
-        <v>0</v>
+        <v>0.013844</v>
       </c>
       <c r="G619" s="7">
-        <v>0</v>
+        <v>0.038964</v>
       </c>
       <c r="H619" s="7">
-        <v>0</v>
+        <v>0.032355999999999996</v>
       </c>
       <c r="I619" s="7">
-        <v>0</v>
+        <v>0.020824</v>
       </c>
       <c r="J619" s="7"/>
       <c r="K619" s="7"/>
@@ -26844,13 +26844,13 @@
         <v>-0.109602</v>
       </c>
       <c r="G625" s="7">
-        <v>0.019129</v>
+        <v>0.01913</v>
       </c>
       <c r="H625" s="7">
         <v>0.118935</v>
       </c>
       <c r="I625" s="7">
-        <v>0.401004</v>
+        <v>0.40100499999999994</v>
       </c>
       <c r="J625" s="7"/>
       <c r="K625" s="7"/>
@@ -26966,22 +26966,22 @@
         <v>6</v>
       </c>
       <c r="E629" s="7">
-        <v>0</v>
+        <v>0.004545</v>
       </c>
       <c r="F629" s="7">
-        <v>0</v>
+        <v>-0.020804999999999997</v>
       </c>
       <c r="G629" s="7">
-        <v>0</v>
+        <v>0.297</v>
       </c>
       <c r="H629" s="7">
-        <v>0</v>
+        <v>0.16078499999999998</v>
       </c>
       <c r="I629" s="7">
-        <v>0</v>
+        <v>0.229139</v>
       </c>
       <c r="J629" s="7">
-        <v>0</v>
+        <v>2.048095</v>
       </c>
       <c r="K629" s="7"/>
     </row>
@@ -27538,16 +27538,16 @@
         <v>5</v>
       </c>
       <c r="E647" s="7">
-        <v>-0.097958</v>
+        <v>-0.097149</v>
       </c>
       <c r="F647" s="7">
-        <v>0.01988</v>
+        <v>0.020794</v>
       </c>
       <c r="G647" s="7">
-        <v>0.164849</v>
+        <v>0.165893</v>
       </c>
       <c r="H647" s="7">
-        <v>0.358622</v>
+        <v>0.35983899999999996</v>
       </c>
       <c r="I647" s="7"/>
       <c r="J647" s="7"/>
@@ -27567,19 +27567,19 @@
         <v>6</v>
       </c>
       <c r="E648" s="7">
-        <v>-0.088687</v>
+        <v>-0.087501</v>
       </c>
       <c r="F648" s="7">
-        <v>-0.045742000000000005</v>
+        <v>-0.044501</v>
       </c>
       <c r="G648" s="7">
-        <v>0.146424</v>
+        <v>0.14791600000000002</v>
       </c>
       <c r="H648" s="7">
-        <v>0.206194</v>
+        <v>0.20776399999999998</v>
       </c>
       <c r="I648" s="7">
-        <v>0.17406400000000002</v>
+        <v>0.175592</v>
       </c>
       <c r="J648" s="7"/>
       <c r="K648" s="7"/>
@@ -27658,16 +27658,16 @@
         <v>2</v>
       </c>
       <c r="E651" s="7">
-        <v>0</v>
+        <v>-0.034349</v>
       </c>
       <c r="F651" s="7">
-        <v>0</v>
+        <v>0.028260999999999998</v>
       </c>
       <c r="G651" s="7">
-        <v>0</v>
+        <v>0.133691</v>
       </c>
       <c r="H651" s="7">
-        <v>0</v>
+        <v>0.213521</v>
       </c>
       <c r="I651" s="7"/>
       <c r="J651" s="7"/>
@@ -27687,25 +27687,25 @@
         <v>6</v>
       </c>
       <c r="E652" s="7">
-        <v>0</v>
+        <v>-0.16270600000000002</v>
       </c>
       <c r="F652" s="7">
-        <v>0</v>
+        <v>-0.165079</v>
       </c>
       <c r="G652" s="7">
-        <v>0</v>
+        <v>-0.075123</v>
       </c>
       <c r="H652" s="7">
-        <v>0</v>
+        <v>-0.058935</v>
       </c>
       <c r="I652" s="7">
-        <v>0</v>
+        <v>-0.031425</v>
       </c>
       <c r="J652" s="7">
-        <v>0</v>
+        <v>0.533888</v>
       </c>
       <c r="K652" s="7">
-        <v>0</v>
+        <v>11.515404</v>
       </c>
     </row>
     <row r="653" spans="1:11" x14ac:dyDescent="0.25">
@@ -27753,19 +27753,19 @@
         <v>6</v>
       </c>
       <c r="E654" s="7">
-        <v>-0.09487</v>
+        <v>-0.094522</v>
       </c>
       <c r="F654" s="7">
-        <v>-0.105396</v>
+        <v>-0.105051</v>
       </c>
       <c r="G654" s="7">
-        <v>-0.105226</v>
+        <v>-0.104882</v>
       </c>
       <c r="H654" s="7">
-        <v>-0.061148</v>
+        <v>-0.06078700000000001</v>
       </c>
       <c r="I654" s="7">
-        <v>0.034979</v>
+        <v>0.035377</v>
       </c>
       <c r="J654" s="7"/>
       <c r="K654" s="7"/>
@@ -27912,19 +27912,19 @@
         <v>2</v>
       </c>
       <c r="E659" s="7">
-        <v>0</v>
+        <v>0.016428</v>
       </c>
       <c r="F659" s="7">
-        <v>0</v>
+        <v>0.08161199999999999</v>
       </c>
       <c r="G659" s="7">
-        <v>0</v>
+        <v>0.192595</v>
       </c>
       <c r="H659" s="7">
-        <v>0</v>
+        <v>0.30269999999999997</v>
       </c>
       <c r="I659" s="7">
-        <v>0</v>
+        <v>0.417449</v>
       </c>
       <c r="J659" s="7"/>
       <c r="K659" s="7"/>
@@ -28676,22 +28676,22 @@
       </c>
       <c r="D683" s="6"/>
       <c r="E683" s="7">
-        <v>0</v>
+        <v>-0.021109</v>
       </c>
       <c r="F683" s="7">
-        <v>0</v>
+        <v>0.044236000000000004</v>
       </c>
       <c r="G683" s="7">
-        <v>0</v>
+        <v>0.115746</v>
       </c>
       <c r="H683" s="7">
-        <v>0</v>
+        <v>0.189349</v>
       </c>
       <c r="I683" s="7">
-        <v>0</v>
+        <v>0.279704</v>
       </c>
       <c r="J683" s="7">
-        <v>0</v>
+        <v>1.364782</v>
       </c>
       <c r="K683" s="7"/>
     </row>
@@ -28709,25 +28709,25 @@
         <v>4</v>
       </c>
       <c r="E684" s="7">
-        <v>0</v>
+        <v>-0.016736</v>
       </c>
       <c r="F684" s="7">
-        <v>0</v>
+        <v>0.057778</v>
       </c>
       <c r="G684" s="7">
-        <v>0</v>
+        <v>0.10508200000000001</v>
       </c>
       <c r="H684" s="7">
-        <v>0</v>
+        <v>0.180308</v>
       </c>
       <c r="I684" s="7">
-        <v>0</v>
+        <v>0.295179</v>
       </c>
       <c r="J684" s="7">
-        <v>0</v>
+        <v>1.638947</v>
       </c>
       <c r="K684" s="7">
-        <v>0</v>
+        <v>6.207504</v>
       </c>
     </row>
     <row r="685" spans="1:11" x14ac:dyDescent="0.25">
@@ -28981,25 +28981,25 @@
         <v>6</v>
       </c>
       <c r="E692" s="7">
-        <v>0.018649</v>
+        <v>0.018112</v>
       </c>
       <c r="F692" s="7">
-        <v>0.042781</v>
+        <v>0.042231</v>
       </c>
       <c r="G692" s="7">
-        <v>0.46313200000000004</v>
+        <v>0.46236</v>
       </c>
       <c r="H692" s="7">
-        <v>0.43817999999999996</v>
+        <v>0.437421</v>
       </c>
       <c r="I692" s="7">
-        <v>0.499881</v>
+        <v>0.499089</v>
       </c>
       <c r="J692" s="7">
-        <v>2.678419</v>
+        <v>2.6764780000000004</v>
       </c>
       <c r="K692" s="7">
-        <v>10.698592000000001</v>
+        <v>10.69242</v>
       </c>
     </row>
     <row r="693" spans="1:11" x14ac:dyDescent="0.25">
@@ -29707,22 +29707,22 @@
         <v>6</v>
       </c>
       <c r="E714" s="7">
-        <v>0</v>
+        <v>-0.050961</v>
       </c>
       <c r="F714" s="7">
-        <v>0</v>
+        <v>0.075726</v>
       </c>
       <c r="G714" s="7">
-        <v>0</v>
+        <v>-0.047271</v>
       </c>
       <c r="H714" s="7">
-        <v>0</v>
+        <v>-0.0039829999999999996</v>
       </c>
       <c r="I714" s="7">
-        <v>0</v>
+        <v>0.355975</v>
       </c>
       <c r="J714" s="7">
-        <v>0</v>
+        <v>2.596316</v>
       </c>
       <c r="K714" s="7"/>
     </row>
@@ -29901,10 +29901,10 @@
         <v>6</v>
       </c>
       <c r="E720" s="7">
-        <v>0</v>
+        <v>-0.042495000000000005</v>
       </c>
       <c r="F720" s="7">
-        <v>0</v>
+        <v>0.052612</v>
       </c>
       <c r="G720" s="7"/>
       <c r="H720" s="7"/>
@@ -30684,16 +30684,16 @@
         <v>1</v>
       </c>
       <c r="E745" s="7">
-        <v>0</v>
+        <v>0.034876</v>
       </c>
       <c r="F745" s="7">
-        <v>0</v>
+        <v>0.11233599999999999</v>
       </c>
       <c r="G745" s="7">
-        <v>0</v>
+        <v>0.241397</v>
       </c>
       <c r="H745" s="7">
-        <v>0</v>
+        <v>0.38216700000000003</v>
       </c>
       <c r="I745" s="7"/>
       <c r="J745" s="7"/>
@@ -30800,19 +30800,19 @@
         <v>6</v>
       </c>
       <c r="E749" s="7">
-        <v>0</v>
+        <v>-0.125251</v>
       </c>
       <c r="F749" s="7">
-        <v>0</v>
+        <v>-0.047774000000000004</v>
       </c>
       <c r="G749" s="7">
-        <v>0</v>
+        <v>-0.008708</v>
       </c>
       <c r="H749" s="7">
-        <v>0</v>
+        <v>0.012624</v>
       </c>
       <c r="I749" s="7">
-        <v>0</v>
+        <v>0.059177999999999994</v>
       </c>
       <c r="J749" s="7"/>
       <c r="K749" s="7"/>
@@ -30864,10 +30864,10 @@
         <v>1</v>
       </c>
       <c r="E751" s="7">
-        <v>0</v>
+        <v>0.026099999999999998</v>
       </c>
       <c r="F751" s="7">
-        <v>0</v>
+        <v>0.096984</v>
       </c>
       <c r="G751" s="7"/>
       <c r="H751" s="7"/>
@@ -30978,19 +30978,19 @@
         <v>1</v>
       </c>
       <c r="E755" s="7">
-        <v>0</v>
+        <v>0.03515</v>
       </c>
       <c r="F755" s="7">
-        <v>0</v>
+        <v>0.114693</v>
       </c>
       <c r="G755" s="7">
-        <v>0</v>
+        <v>0.24581499999999998</v>
       </c>
       <c r="H755" s="7">
-        <v>0</v>
+        <v>0.38922199999999996</v>
       </c>
       <c r="I755" s="7">
-        <v>0</v>
+        <v>0.555662</v>
       </c>
       <c r="J755" s="7"/>
       <c r="K755" s="7"/>
@@ -31071,13 +31071,13 @@
         <v>2</v>
       </c>
       <c r="E758" s="7">
-        <v>0</v>
+        <v>0.024321000000000002</v>
       </c>
       <c r="F758" s="7">
-        <v>0</v>
+        <v>0.111929</v>
       </c>
       <c r="G758" s="7">
-        <v>0</v>
+        <v>0.251154</v>
       </c>
       <c r="H758" s="7"/>
       <c r="I758" s="7"/>
@@ -31817,19 +31817,19 @@
         <v>2</v>
       </c>
       <c r="E782" s="7">
-        <v>0</v>
+        <v>0.020282</v>
       </c>
       <c r="F782" s="7">
-        <v>0</v>
+        <v>0.105788</v>
       </c>
       <c r="G782" s="7">
-        <v>0</v>
+        <v>0.24417100000000003</v>
       </c>
       <c r="H782" s="7">
-        <v>0</v>
+        <v>0.391791</v>
       </c>
       <c r="I782" s="7">
-        <v>0</v>
+        <v>0.570538</v>
       </c>
       <c r="J782" s="7"/>
       <c r="K782" s="7"/>
@@ -32185,10 +32185,10 @@
         <v>5</v>
       </c>
       <c r="E794" s="7">
-        <v>0</v>
+        <v>-0.028529</v>
       </c>
       <c r="F794" s="7">
-        <v>0</v>
+        <v>0.131089</v>
       </c>
       <c r="G794" s="7"/>
       <c r="H794" s="7"/>
@@ -33513,22 +33513,22 @@
         <v>2</v>
       </c>
       <c r="E836" s="7">
-        <v>0</v>
+        <v>0.029809000000000002</v>
       </c>
       <c r="F836" s="7">
-        <v>0</v>
+        <v>0.100138</v>
       </c>
       <c r="G836" s="7">
-        <v>0</v>
+        <v>0.214234</v>
       </c>
       <c r="H836" s="7">
-        <v>0</v>
+        <v>0.329428</v>
       </c>
       <c r="I836" s="7">
-        <v>0</v>
+        <v>0.46712899999999996</v>
       </c>
       <c r="J836" s="7">
-        <v>0</v>
+        <v>2.6377620000000004</v>
       </c>
       <c r="K836" s="7"/>
     </row>
@@ -33577,22 +33577,22 @@
         <v>1</v>
       </c>
       <c r="E838" s="7">
-        <v>0</v>
+        <v>0.027295</v>
       </c>
       <c r="F838" s="7">
-        <v>0</v>
+        <v>0.093593</v>
       </c>
       <c r="G838" s="7">
-        <v>0</v>
+        <v>0.204522</v>
       </c>
       <c r="H838" s="7">
-        <v>0</v>
+        <v>0.317523</v>
       </c>
       <c r="I838" s="7">
-        <v>0</v>
+        <v>0.45339100000000004</v>
       </c>
       <c r="J838" s="7">
-        <v>0</v>
+        <v>2.622923</v>
       </c>
       <c r="K838" s="7"/>
     </row>
@@ -33608,22 +33608,22 @@
       </c>
       <c r="D839" s="6"/>
       <c r="E839" s="7">
-        <v>0</v>
+        <v>0.015773</v>
       </c>
       <c r="F839" s="7">
-        <v>0</v>
+        <v>0.056481</v>
       </c>
       <c r="G839" s="7">
-        <v>0</v>
+        <v>0.11481</v>
       </c>
       <c r="H839" s="7">
-        <v>0</v>
+        <v>0.167274</v>
       </c>
       <c r="I839" s="7">
-        <v>0</v>
+        <v>0.21769</v>
       </c>
       <c r="J839" s="7">
-        <v>0</v>
+        <v>1.043159</v>
       </c>
       <c r="K839" s="7"/>
     </row>
@@ -33703,19 +33703,19 @@
         <v>2</v>
       </c>
       <c r="E842" s="7">
-        <v>0</v>
+        <v>0.03169</v>
       </c>
       <c r="F842" s="7">
-        <v>0</v>
+        <v>0.10280900000000001</v>
       </c>
       <c r="G842" s="7">
-        <v>0</v>
+        <v>0.21868200000000002</v>
       </c>
       <c r="H842" s="7">
-        <v>0</v>
+        <v>0.338832</v>
       </c>
       <c r="I842" s="7">
-        <v>0</v>
+        <v>0.48305</v>
       </c>
       <c r="J842" s="7"/>
       <c r="K842" s="7"/>
@@ -33990,19 +33990,19 @@
         <v>7</v>
       </c>
       <c r="E851" s="7">
-        <v>0</v>
+        <v>-0.09955</v>
       </c>
       <c r="F851" s="7">
-        <v>0</v>
+        <v>-0.199439</v>
       </c>
       <c r="G851" s="7">
-        <v>0</v>
+        <v>-0.08379400000000001</v>
       </c>
       <c r="H851" s="7">
-        <v>0</v>
+        <v>0.037602000000000003</v>
       </c>
       <c r="I851" s="7">
-        <v>0</v>
+        <v>0.19581099999999999</v>
       </c>
       <c r="J851" s="7"/>
       <c r="K851" s="7"/>
@@ -34021,7 +34021,7 @@
         <v>5</v>
       </c>
       <c r="E852" s="7">
-        <v>0</v>
+        <v>-0.061752</v>
       </c>
       <c r="F852" s="7"/>
       <c r="G852" s="7"/>
@@ -34075,7 +34075,7 @@
         <v>5</v>
       </c>
       <c r="E854" s="7">
-        <v>-0.052168</v>
+        <v>-0.052177</v>
       </c>
       <c r="F854" s="7"/>
       <c r="G854" s="7"/>
@@ -34152,22 +34152,22 @@
         <v>7</v>
       </c>
       <c r="E857" s="7">
-        <v>0</v>
+        <v>-0.069659</v>
       </c>
       <c r="F857" s="7">
-        <v>0</v>
+        <v>-0.078052</v>
       </c>
       <c r="G857" s="7">
-        <v>0</v>
+        <v>-0.03073</v>
       </c>
       <c r="H857" s="7">
-        <v>0</v>
+        <v>0.058106</v>
       </c>
       <c r="I857" s="7">
-        <v>0</v>
+        <v>0.075903</v>
       </c>
       <c r="J857" s="7">
-        <v>0</v>
+        <v>1.071631</v>
       </c>
       <c r="K857" s="7"/>
     </row>
@@ -34185,16 +34185,16 @@
         <v>7</v>
       </c>
       <c r="E858" s="7">
-        <v>0</v>
+        <v>-0.293221</v>
       </c>
       <c r="F858" s="7">
-        <v>0</v>
+        <v>-0.28181100000000003</v>
       </c>
       <c r="G858" s="7">
-        <v>0</v>
+        <v>-0.18519200000000002</v>
       </c>
       <c r="H858" s="7">
-        <v>0</v>
+        <v>0.041985999999999996</v>
       </c>
       <c r="I858" s="7"/>
       <c r="J858" s="7"/>
@@ -34334,19 +34334,19 @@
         <v>3</v>
       </c>
       <c r="E863" s="7">
-        <v>0</v>
+        <v>-0.08353300000000001</v>
       </c>
       <c r="F863" s="7">
-        <v>0</v>
+        <v>0.088768</v>
       </c>
       <c r="G863" s="7">
-        <v>0</v>
+        <v>0.183811</v>
       </c>
       <c r="H863" s="7">
-        <v>0</v>
+        <v>0.253886</v>
       </c>
       <c r="I863" s="7">
-        <v>0</v>
+        <v>0.33646099999999995</v>
       </c>
       <c r="J863" s="7"/>
       <c r="K863" s="7"/>
@@ -34652,19 +34652,19 @@
         <v>6</v>
       </c>
       <c r="E873" s="7">
-        <v>0.101543</v>
+        <v>0.100884</v>
       </c>
       <c r="F873" s="7">
-        <v>0.130946</v>
+        <v>0.130269</v>
       </c>
       <c r="G873" s="7">
-        <v>0.199522</v>
+        <v>0.198804</v>
       </c>
       <c r="H873" s="7">
-        <v>0.397077</v>
+        <v>0.396241</v>
       </c>
       <c r="I873" s="7">
-        <v>0.21546900000000002</v>
+        <v>0.214741</v>
       </c>
       <c r="J873" s="7"/>
       <c r="K873" s="7"/>
@@ -34718,25 +34718,25 @@
         <v>6</v>
       </c>
       <c r="E875" s="7">
-        <v>-0.065707</v>
+        <v>-0.06575199999999999</v>
       </c>
       <c r="F875" s="7">
-        <v>-0.058853</v>
+        <v>-0.058899</v>
       </c>
       <c r="G875" s="7">
-        <v>-0.010216000000000001</v>
+        <v>-0.010264</v>
       </c>
       <c r="H875" s="7">
-        <v>0.080381</v>
+        <v>0.080328</v>
       </c>
       <c r="I875" s="7">
-        <v>0.179273</v>
+        <v>0.17921600000000001</v>
       </c>
       <c r="J875" s="7">
-        <v>0.889478</v>
+        <v>0.8893859999999999</v>
       </c>
       <c r="K875" s="7">
-        <v>7.219285</v>
+        <v>7.218885</v>
       </c>
     </row>
     <row r="876" spans="1:11" x14ac:dyDescent="0.25">
@@ -34753,25 +34753,25 @@
         <v>6</v>
       </c>
       <c r="E876" s="7">
-        <v>0.027404</v>
+        <v>0.027634</v>
       </c>
       <c r="F876" s="7">
-        <v>0.099178</v>
+        <v>0.099424</v>
       </c>
       <c r="G876" s="7">
-        <v>0.28427800000000003</v>
+        <v>0.28456600000000004</v>
       </c>
       <c r="H876" s="7">
-        <v>0.298567</v>
+        <v>0.298859</v>
       </c>
       <c r="I876" s="7">
-        <v>0.422378</v>
+        <v>0.422697</v>
       </c>
       <c r="J876" s="7">
-        <v>2.168047</v>
+        <v>2.168758</v>
       </c>
       <c r="K876" s="7">
-        <v>7.465218</v>
+        <v>7.467116999999999</v>
       </c>
     </row>
     <row r="877" spans="1:11" x14ac:dyDescent="0.25">
@@ -34949,25 +34949,25 @@
         <v>3</v>
       </c>
       <c r="E882" s="7">
-        <v>0</v>
+        <v>-0.005845</v>
       </c>
       <c r="F882" s="7">
-        <v>0</v>
+        <v>0.02754</v>
       </c>
       <c r="G882" s="7">
-        <v>0</v>
+        <v>0.12085000000000001</v>
       </c>
       <c r="H882" s="7">
-        <v>0</v>
+        <v>0.057234999999999994</v>
       </c>
       <c r="I882" s="7">
-        <v>0</v>
+        <v>0.187041</v>
       </c>
       <c r="J882" s="7">
-        <v>0</v>
+        <v>0.7566670000000001</v>
       </c>
       <c r="K882" s="7">
-        <v>0</v>
+        <v>1.330127</v>
       </c>
     </row>
     <row r="883" spans="1:11" x14ac:dyDescent="0.25">
@@ -35051,7 +35051,7 @@
         <v>17</v>
       </c>
       <c r="D885" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E885" s="7">
         <v>0.030018</v>
@@ -35225,25 +35225,25 @@
         <v>4</v>
       </c>
       <c r="E890" s="7">
-        <v>0</v>
+        <v>-0.037554</v>
       </c>
       <c r="F890" s="7">
-        <v>0</v>
+        <v>0.020034999999999997</v>
       </c>
       <c r="G890" s="7">
-        <v>0</v>
+        <v>0.121192</v>
       </c>
       <c r="H890" s="7">
-        <v>0</v>
+        <v>0.272774</v>
       </c>
       <c r="I890" s="7">
-        <v>0</v>
+        <v>0.410619</v>
       </c>
       <c r="J890" s="7">
-        <v>0</v>
+        <v>2.164808</v>
       </c>
       <c r="K890" s="7">
-        <v>0</v>
+        <v>5.197306</v>
       </c>
     </row>
     <row r="891" spans="1:11" x14ac:dyDescent="0.25">
@@ -35260,25 +35260,25 @@
         <v>3</v>
       </c>
       <c r="E891" s="7">
-        <v>0</v>
+        <v>0.024340999999999998</v>
       </c>
       <c r="F891" s="7">
-        <v>0</v>
+        <v>0.095423</v>
       </c>
       <c r="G891" s="7">
-        <v>0</v>
+        <v>0.199486</v>
       </c>
       <c r="H891" s="7">
-        <v>0</v>
+        <v>0.32201500000000005</v>
       </c>
       <c r="I891" s="7">
-        <v>0</v>
+        <v>0.467488</v>
       </c>
       <c r="J891" s="7">
-        <v>0</v>
+        <v>1.9629269999999999</v>
       </c>
       <c r="K891" s="7">
-        <v>0</v>
+        <v>5.208319</v>
       </c>
     </row>
     <row r="892" spans="1:11" x14ac:dyDescent="0.25">
@@ -35326,25 +35326,25 @@
         <v>6</v>
       </c>
       <c r="E893" s="7">
-        <v>0</v>
+        <v>0.061109</v>
       </c>
       <c r="F893" s="7">
-        <v>0</v>
+        <v>0.093528</v>
       </c>
       <c r="G893" s="7">
-        <v>0</v>
+        <v>0.585261</v>
       </c>
       <c r="H893" s="7">
-        <v>0</v>
+        <v>0.461279</v>
       </c>
       <c r="I893" s="7">
-        <v>0</v>
+        <v>0.519243</v>
       </c>
       <c r="J893" s="7">
-        <v>0</v>
+        <v>2.48591</v>
       </c>
       <c r="K893" s="7">
-        <v>0</v>
+        <v>8.2727</v>
       </c>
     </row>
     <row r="894" spans="1:11" x14ac:dyDescent="0.25">
@@ -35932,22 +35932,22 @@
       </c>
       <c r="D911" s="6"/>
       <c r="E911" s="7">
-        <v>0</v>
+        <v>-0.016605</v>
       </c>
       <c r="F911" s="7">
-        <v>0</v>
+        <v>0.036529</v>
       </c>
       <c r="G911" s="7">
-        <v>0</v>
+        <v>0.113293</v>
       </c>
       <c r="H911" s="7">
-        <v>0</v>
+        <v>0.113262</v>
       </c>
       <c r="I911" s="7">
-        <v>0</v>
+        <v>0.17537299999999997</v>
       </c>
       <c r="J911" s="7">
-        <v>0</v>
+        <v>1.266147</v>
       </c>
       <c r="K911" s="7"/>
     </row>
@@ -36101,16 +36101,16 @@
         <v>1</v>
       </c>
       <c r="E916" s="7">
-        <v>0</v>
+        <v>0.010998</v>
       </c>
       <c r="F916" s="7">
-        <v>0</v>
+        <v>0.08164099999999999</v>
       </c>
       <c r="G916" s="7">
-        <v>0</v>
+        <v>0.204081</v>
       </c>
       <c r="H916" s="7">
-        <v>0</v>
+        <v>0.32874400000000004</v>
       </c>
       <c r="I916" s="7"/>
       <c r="J916" s="7"/>
@@ -36394,25 +36394,25 @@
         <v>1</v>
       </c>
       <c r="E925" s="7">
-        <v>0</v>
+        <v>0.028912</v>
       </c>
       <c r="F925" s="7">
-        <v>0</v>
+        <v>0.09687</v>
       </c>
       <c r="G925" s="7">
-        <v>0</v>
+        <v>0.20349</v>
       </c>
       <c r="H925" s="7">
-        <v>0</v>
+        <v>0.318363</v>
       </c>
       <c r="I925" s="7">
-        <v>0</v>
+        <v>0.451339</v>
       </c>
       <c r="J925" s="7">
-        <v>0</v>
+        <v>2.324734</v>
       </c>
       <c r="K925" s="7">
-        <v>0</v>
+        <v>3.813538</v>
       </c>
     </row>
     <row r="926" spans="1:11" x14ac:dyDescent="0.25">
@@ -36460,25 +36460,25 @@
         <v>6</v>
       </c>
       <c r="E927" s="7">
-        <v>0</v>
+        <v>-0.070656</v>
       </c>
       <c r="F927" s="7">
-        <v>0</v>
+        <v>0.055452</v>
       </c>
       <c r="G927" s="7">
-        <v>0</v>
+        <v>-0.035689</v>
       </c>
       <c r="H927" s="7">
-        <v>0</v>
+        <v>-0.000236</v>
       </c>
       <c r="I927" s="7">
-        <v>0</v>
+        <v>0.214221</v>
       </c>
       <c r="J927" s="7">
-        <v>0</v>
+        <v>1.6159000000000001</v>
       </c>
       <c r="K927" s="7">
-        <v>0</v>
+        <v>5.724417</v>
       </c>
     </row>
     <row r="928" spans="1:11" x14ac:dyDescent="0.25">
@@ -36528,25 +36528,25 @@
       </c>
       <c r="D929" s="6"/>
       <c r="E929" s="7">
-        <v>0</v>
+        <v>0.013059000000000001</v>
       </c>
       <c r="F929" s="7">
-        <v>0</v>
+        <v>0.057431</v>
       </c>
       <c r="G929" s="7">
-        <v>0</v>
+        <v>0.142882</v>
       </c>
       <c r="H929" s="7">
-        <v>0</v>
+        <v>0.163107</v>
       </c>
       <c r="I929" s="7">
-        <v>0</v>
+        <v>0.23414100000000002</v>
       </c>
       <c r="J929" s="7">
-        <v>0</v>
+        <v>1.251387</v>
       </c>
       <c r="K929" s="7">
-        <v>0</v>
+        <v>6.35782</v>
       </c>
     </row>
     <row r="930" spans="1:11" x14ac:dyDescent="0.25">
@@ -36563,25 +36563,25 @@
         <v>6</v>
       </c>
       <c r="E930" s="7">
-        <v>0</v>
+        <v>-0.005816</v>
       </c>
       <c r="F930" s="7">
-        <v>0</v>
+        <v>0.028553000000000002</v>
       </c>
       <c r="G930" s="7">
-        <v>0</v>
+        <v>0.118185</v>
       </c>
       <c r="H930" s="7">
-        <v>0</v>
+        <v>0.122904</v>
       </c>
       <c r="I930" s="7">
-        <v>0</v>
+        <v>0.18546600000000002</v>
       </c>
       <c r="J930" s="7">
-        <v>0</v>
+        <v>1.106162</v>
       </c>
       <c r="K930" s="7">
-        <v>0</v>
+        <v>5.593589</v>
       </c>
     </row>
     <row r="931" spans="1:11" x14ac:dyDescent="0.25">
@@ -36596,25 +36596,25 @@
       </c>
       <c r="D931" s="6"/>
       <c r="E931" s="7">
-        <v>0</v>
+        <v>-0.016878</v>
       </c>
       <c r="F931" s="7">
-        <v>0</v>
+        <v>0.026142</v>
       </c>
       <c r="G931" s="7">
-        <v>0</v>
+        <v>0.174089</v>
       </c>
       <c r="H931" s="7">
-        <v>0</v>
+        <v>0.275057</v>
       </c>
       <c r="I931" s="7">
-        <v>0</v>
+        <v>0.549812</v>
       </c>
       <c r="J931" s="7">
-        <v>0</v>
+        <v>2.397673</v>
       </c>
       <c r="K931" s="7">
-        <v>0</v>
+        <v>20.310301</v>
       </c>
     </row>
     <row r="932" spans="1:11" x14ac:dyDescent="0.25">
@@ -36666,25 +36666,25 @@
         <v>6</v>
       </c>
       <c r="E933" s="7">
-        <v>0</v>
+        <v>0.011739</v>
       </c>
       <c r="F933" s="7">
-        <v>0</v>
+        <v>0.054845</v>
       </c>
       <c r="G933" s="7">
-        <v>0</v>
+        <v>0.12998900000000002</v>
       </c>
       <c r="H933" s="7">
-        <v>0</v>
+        <v>0.173419</v>
       </c>
       <c r="I933" s="7">
-        <v>0</v>
+        <v>0.237931</v>
       </c>
       <c r="J933" s="7">
-        <v>0</v>
+        <v>1.277633</v>
       </c>
       <c r="K933" s="7">
-        <v>0</v>
+        <v>6.604895</v>
       </c>
     </row>
     <row r="934" spans="1:11" x14ac:dyDescent="0.25">
@@ -36930,25 +36930,25 @@
         <v>6</v>
       </c>
       <c r="E941" s="7">
-        <v>0</v>
+        <v>-0.04346</v>
       </c>
       <c r="F941" s="7">
-        <v>0</v>
+        <v>0.08718400000000001</v>
       </c>
       <c r="G941" s="7">
-        <v>0</v>
+        <v>-0.011322</v>
       </c>
       <c r="H941" s="7">
-        <v>0</v>
+        <v>0.058651</v>
       </c>
       <c r="I941" s="7">
-        <v>0</v>
+        <v>0.22943100000000002</v>
       </c>
       <c r="J941" s="7">
-        <v>0</v>
+        <v>2.879103</v>
       </c>
       <c r="K941" s="7">
-        <v>0</v>
+        <v>11.355349</v>
       </c>
     </row>
     <row r="942" spans="1:11" x14ac:dyDescent="0.25">
@@ -36965,16 +36965,16 @@
         <v>6</v>
       </c>
       <c r="E942" s="7">
-        <v>-0.105898</v>
+        <v>-0.10586499999999999</v>
       </c>
       <c r="F942" s="7">
-        <v>-0.09491300000000001</v>
+        <v>-0.09487999999999999</v>
       </c>
       <c r="G942" s="7">
-        <v>-0.066929</v>
+        <v>-0.066895</v>
       </c>
       <c r="H942" s="7">
-        <v>0.033613</v>
+        <v>0.033651</v>
       </c>
       <c r="I942" s="7"/>
       <c r="J942" s="7"/>
@@ -37027,25 +37027,25 @@
         <v>6</v>
       </c>
       <c r="E944" s="7">
-        <v>0</v>
+        <v>-0.08041999999999999</v>
       </c>
       <c r="F944" s="7">
-        <v>0</v>
+        <v>-0.057076</v>
       </c>
       <c r="G944" s="7">
-        <v>0</v>
+        <v>-0.01262</v>
       </c>
       <c r="H944" s="7">
-        <v>0</v>
+        <v>0.078344</v>
       </c>
       <c r="I944" s="7">
-        <v>0</v>
+        <v>0.113567</v>
       </c>
       <c r="J944" s="7">
-        <v>0</v>
+        <v>0.7750879999999999</v>
       </c>
       <c r="K944" s="7">
-        <v>0</v>
+        <v>11.845944999999999</v>
       </c>
     </row>
     <row r="945" spans="1:11" x14ac:dyDescent="0.25">
@@ -37132,22 +37132,22 @@
         <v>7</v>
       </c>
       <c r="E947" s="7">
-        <v>0.042762</v>
+        <v>0.043023</v>
       </c>
       <c r="F947" s="7">
-        <v>0.07447</v>
+        <v>0.074739</v>
       </c>
       <c r="G947" s="7">
-        <v>0.21053899999999998</v>
+        <v>0.210842</v>
       </c>
       <c r="H947" s="7">
-        <v>0.213863</v>
+        <v>0.214167</v>
       </c>
       <c r="I947" s="7">
-        <v>0.284431</v>
+        <v>0.28475300000000003</v>
       </c>
       <c r="J947" s="7">
-        <v>2.271901</v>
+        <v>2.27272</v>
       </c>
       <c r="K947" s="7"/>
     </row>
@@ -37532,10 +37532,10 @@
         <v>6</v>
       </c>
       <c r="E959" s="7">
-        <v>0</v>
+        <v>-0.036185</v>
       </c>
       <c r="F959" s="7">
-        <v>0</v>
+        <v>0.061003</v>
       </c>
       <c r="G959" s="7"/>
       <c r="H959" s="7"/>
@@ -37678,19 +37678,19 @@
         <v>2</v>
       </c>
       <c r="E965" s="7">
-        <v>0</v>
+        <v>0.030387</v>
       </c>
       <c r="F965" s="7">
-        <v>0</v>
+        <v>0.101419</v>
       </c>
       <c r="G965" s="7">
-        <v>0</v>
+        <v>0.210979</v>
       </c>
       <c r="H965" s="7">
-        <v>0</v>
+        <v>0.331851</v>
       </c>
       <c r="I965" s="7">
-        <v>0</v>
+        <v>0.47217</v>
       </c>
       <c r="J965" s="7"/>
       <c r="K965" s="7"/>
@@ -37709,19 +37709,19 @@
         <v>3</v>
       </c>
       <c r="E966" s="7">
-        <v>0</v>
+        <v>0.017103</v>
       </c>
       <c r="F966" s="7">
-        <v>0</v>
+        <v>0.076189</v>
       </c>
       <c r="G966" s="7">
-        <v>0</v>
+        <v>0.109754</v>
       </c>
       <c r="H966" s="7">
-        <v>0</v>
+        <v>0.20406400000000002</v>
       </c>
       <c r="I966" s="7">
-        <v>0</v>
+        <v>0.359401</v>
       </c>
       <c r="J966" s="7"/>
       <c r="K966" s="7"/>
@@ -37828,13 +37828,13 @@
         <v>2</v>
       </c>
       <c r="E971" s="7">
-        <v>0</v>
+        <v>0.033529</v>
       </c>
       <c r="F971" s="7">
-        <v>0</v>
+        <v>0.10627</v>
       </c>
       <c r="G971" s="7">
-        <v>0</v>
+        <v>0.18901800000000002</v>
       </c>
       <c r="H971" s="7"/>
       <c r="I971" s="7"/>
@@ -37855,13 +37855,13 @@
         <v>6</v>
       </c>
       <c r="E972" s="7">
-        <v>0</v>
+        <v>-0.161563</v>
       </c>
       <c r="F972" s="7">
-        <v>0</v>
+        <v>-0.401407</v>
       </c>
       <c r="G972" s="7">
-        <v>0</v>
+        <v>-0.446853</v>
       </c>
       <c r="H972" s="7"/>
       <c r="I972" s="7"/>
@@ -37911,25 +37911,25 @@
         <v>5</v>
       </c>
       <c r="E974" s="7">
-        <v>0</v>
+        <v>-0.0033139999999999997</v>
       </c>
       <c r="F974" s="7">
-        <v>0</v>
+        <v>0.048858</v>
       </c>
       <c r="G974" s="7">
-        <v>0</v>
+        <v>0.12617599999999998</v>
       </c>
       <c r="H974" s="7">
-        <v>0</v>
+        <v>0.185237</v>
       </c>
       <c r="I974" s="7">
-        <v>0</v>
+        <v>0.274547</v>
       </c>
       <c r="J974" s="7">
-        <v>0</v>
+        <v>1.347537</v>
       </c>
       <c r="K974" s="7">
-        <v>0</v>
+        <v>5.829751</v>
       </c>
     </row>
     <row r="975" spans="1:11" x14ac:dyDescent="0.25">
@@ -38008,25 +38008,25 @@
         <v>4</v>
       </c>
       <c r="E977" s="7">
-        <v>0</v>
+        <v>0.025865999999999997</v>
       </c>
       <c r="F977" s="7">
-        <v>0</v>
+        <v>0.083843</v>
       </c>
       <c r="G977" s="7">
-        <v>0</v>
+        <v>0.176389</v>
       </c>
       <c r="H977" s="7">
-        <v>0</v>
+        <v>0.263112</v>
       </c>
       <c r="I977" s="7">
-        <v>0</v>
+        <v>0.363011</v>
       </c>
       <c r="J977" s="7">
-        <v>0</v>
+        <v>1.249987</v>
       </c>
       <c r="K977" s="7">
-        <v>0</v>
+        <v>4.913374</v>
       </c>
     </row>
     <row r="978" spans="1:11" x14ac:dyDescent="0.25">
@@ -38309,25 +38309,25 @@
         <v>2</v>
       </c>
       <c r="E986" s="7">
-        <v>0</v>
+        <v>0.008553</v>
       </c>
       <c r="F986" s="7">
-        <v>0</v>
+        <v>0.072714</v>
       </c>
       <c r="G986" s="7">
-        <v>0</v>
+        <v>0.16865300000000003</v>
       </c>
       <c r="H986" s="7">
-        <v>0</v>
+        <v>0.282592</v>
       </c>
       <c r="I986" s="7">
-        <v>0</v>
+        <v>0.39643300000000004</v>
       </c>
       <c r="J986" s="7">
-        <v>0</v>
+        <v>1.781819</v>
       </c>
       <c r="K986" s="7">
-        <v>0</v>
+        <v>3.166532</v>
       </c>
     </row>
     <row r="987" spans="1:11" x14ac:dyDescent="0.25">
@@ -38779,19 +38779,19 @@
         <v>6</v>
       </c>
       <c r="E1000" s="7">
-        <v>0</v>
+        <v>0.039573</v>
       </c>
       <c r="F1000" s="7">
-        <v>0</v>
+        <v>-0.087152</v>
       </c>
       <c r="G1000" s="7">
-        <v>0</v>
+        <v>0.526098</v>
       </c>
       <c r="H1000" s="7">
-        <v>0</v>
+        <v>0.691001</v>
       </c>
       <c r="I1000" s="7">
-        <v>0</v>
+        <v>0.883728</v>
       </c>
       <c r="J1000" s="7"/>
       <c r="K1000" s="7"/>
@@ -38845,25 +38845,25 @@
         <v>5</v>
       </c>
       <c r="E1002" s="7">
-        <v>0</v>
+        <v>0.008365000000000001</v>
       </c>
       <c r="F1002" s="7">
-        <v>0</v>
+        <v>-0.019211</v>
       </c>
       <c r="G1002" s="7">
-        <v>0</v>
+        <v>0.43482</v>
       </c>
       <c r="H1002" s="7">
-        <v>0</v>
+        <v>0.480403</v>
       </c>
       <c r="I1002" s="7">
-        <v>0</v>
+        <v>0.5972529999999999</v>
       </c>
       <c r="J1002" s="7">
-        <v>0</v>
+        <v>2.376909</v>
       </c>
       <c r="K1002" s="7">
-        <v>0</v>
+        <v>4.843186</v>
       </c>
     </row>
     <row r="1003" spans="1:11" x14ac:dyDescent="0.25">
@@ -39470,25 +39470,25 @@
         <v>5</v>
       </c>
       <c r="E1021" s="7">
-        <v>0</v>
+        <v>-0.015208</v>
       </c>
       <c r="F1021" s="7">
-        <v>0</v>
+        <v>0.032489</v>
       </c>
       <c r="G1021" s="7">
-        <v>0</v>
+        <v>0.112953</v>
       </c>
       <c r="H1021" s="7">
-        <v>0</v>
+        <v>0.17197199999999999</v>
       </c>
       <c r="I1021" s="7">
-        <v>0</v>
+        <v>0.198135</v>
       </c>
       <c r="J1021" s="7">
-        <v>0</v>
+        <v>1.021868</v>
       </c>
       <c r="K1021" s="7">
-        <v>0</v>
+        <v>4.48996</v>
       </c>
     </row>
     <row r="1022" spans="1:11" x14ac:dyDescent="0.25">
@@ -39652,25 +39652,25 @@
         <v>6</v>
       </c>
       <c r="E1027" s="7">
-        <v>0</v>
+        <v>0.058029000000000004</v>
       </c>
       <c r="F1027" s="7">
-        <v>0</v>
+        <v>0.063541</v>
       </c>
       <c r="G1027" s="7">
-        <v>0</v>
+        <v>0.435437</v>
       </c>
       <c r="H1027" s="7">
-        <v>0</v>
+        <v>0.291601</v>
       </c>
       <c r="I1027" s="7">
-        <v>0</v>
+        <v>0.415164</v>
       </c>
       <c r="J1027" s="7">
-        <v>0</v>
+        <v>2.3132919999999997</v>
       </c>
       <c r="K1027" s="7">
-        <v>0</v>
+        <v>8.746088</v>
       </c>
     </row>
     <row r="1028" spans="1:11" x14ac:dyDescent="0.25">
@@ -39939,25 +39939,25 @@
         <v>7</v>
       </c>
       <c r="E1036" s="7">
-        <v>0</v>
+        <v>-0.079357</v>
       </c>
       <c r="F1036" s="7">
-        <v>0</v>
+        <v>0.06368</v>
       </c>
       <c r="G1036" s="7">
-        <v>0</v>
+        <v>-0.101451</v>
       </c>
       <c r="H1036" s="7">
-        <v>0</v>
+        <v>-0.073283</v>
       </c>
       <c r="I1036" s="7">
-        <v>0</v>
+        <v>0.47139200000000003</v>
       </c>
       <c r="J1036" s="7">
-        <v>0</v>
+        <v>3.343014</v>
       </c>
       <c r="K1036" s="7">
-        <v>0</v>
+        <v>11.497940000000002</v>
       </c>
     </row>
     <row r="1037" spans="1:11" x14ac:dyDescent="0.25">
@@ -39974,25 +39974,25 @@
         <v>7</v>
       </c>
       <c r="E1037" s="7">
-        <v>0</v>
+        <v>-0.057769</v>
       </c>
       <c r="F1037" s="7">
-        <v>0</v>
+        <v>-0.14904799999999999</v>
       </c>
       <c r="G1037" s="7">
-        <v>0</v>
+        <v>-0.00043400000000000003</v>
       </c>
       <c r="H1037" s="7">
-        <v>0</v>
+        <v>-0.047736</v>
       </c>
       <c r="I1037" s="7">
-        <v>0</v>
+        <v>0.015264</v>
       </c>
       <c r="J1037" s="7">
-        <v>0</v>
+        <v>0.870715</v>
       </c>
       <c r="K1037" s="7">
-        <v>0</v>
+        <v>11.914126000000001</v>
       </c>
     </row>
     <row r="1038" spans="1:11" x14ac:dyDescent="0.25">
@@ -40457,25 +40457,25 @@
         <v>7</v>
       </c>
       <c r="E1052" s="7">
-        <v>-0.08135400000000001</v>
+        <v>-0.081368</v>
       </c>
       <c r="F1052" s="7">
-        <v>-0.024104</v>
+        <v>-0.024119</v>
       </c>
       <c r="G1052" s="7">
-        <v>-0.20785900000000002</v>
+        <v>-0.207871</v>
       </c>
       <c r="H1052" s="7">
-        <v>-0.24996300000000002</v>
+        <v>-0.249974</v>
       </c>
       <c r="I1052" s="7">
-        <v>-0.262342</v>
+        <v>-0.262353</v>
       </c>
       <c r="J1052" s="7">
-        <v>1.7702959999999999</v>
+        <v>1.770255</v>
       </c>
       <c r="K1052" s="7">
-        <v>8.455818</v>
+        <v>8.455675</v>
       </c>
     </row>
     <row r="1053" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>